<commit_message>
changed fo.py and 30 min csh since i now only keep nifty and bn as FO shares
</commit_message>
<xml_diff>
--- a/algo high low.xlsx
+++ b/algo high low.xlsx
@@ -655,22 +655,22 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>514.8</v>
+        <v>3307.55</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>504.5</v>
+        <v>3205.25</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>512</v>
+        <v>449.5</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>510.9</v>
+        <v>448.35</v>
       </c>
       <c r="F2" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>507.75</v>
+        <v>3284</v>
       </c>
     </row>
     <row r="3">
@@ -680,22 +680,22 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>7455.5</v>
+        <v>11199.55</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>7318.05</v>
+        <v>10972.05</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>7439.85</v>
+        <v>7413</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>7429.45</v>
+        <v>7394.85</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>7448.5</v>
+        <v>11135.4</v>
       </c>
     </row>
     <row r="4">
@@ -705,22 +705,22 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>212</v>
+        <v>456.55</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>201</v>
+        <v>449.25</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>202.93</v>
+        <v>194.59</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>203.23</v>
+        <v>193.81</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>234</v>
+        <v>23</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>211.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5">
@@ -730,22 +730,22 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>309.9</v>
+        <v>456.55</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>303</v>
+        <v>449.25</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>308.3</v>
+        <v>316</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>308.15</v>
+        <v>315.7</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>304.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6">
@@ -755,22 +755,22 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>2976.5</v>
+        <v>456.55</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>2933.85</v>
+        <v>449.25</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>2948.95</v>
+        <v>2437</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2947.25</v>
+        <v>2437.1</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>11</v>
+        <v>144</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2937.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7">
@@ -780,22 +780,22 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1401</v>
+        <v>456.55</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>1372.1</v>
+        <v>449.25</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>1376</v>
+        <v>1169.55</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1375.95</v>
+        <v>1167.6</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>18</v>
+        <v>156</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>1389.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="8">
@@ -805,22 +805,22 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>5854.5</v>
+        <v>456.55</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>5763.4</v>
+        <v>449.25</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>5781.3</v>
+        <v>5480</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>5779.25</v>
+        <v>5457.15</v>
       </c>
       <c r="F8" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>5801.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="9">
@@ -830,22 +830,22 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>586.8</v>
+        <v>456.55</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>576.35</v>
+        <v>449.25</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>581</v>
+        <v>513</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>580.55</v>
+        <v>513</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>577.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="10">
@@ -855,22 +855,22 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>7050</v>
+        <v>456.55</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>6956.05</v>
+        <v>449.25</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>7007.45</v>
+        <v>6867.9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>7022.7</v>
+        <v>6841.1</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>7000.1</v>
+        <v>450</v>
       </c>
     </row>
     <row r="11">
@@ -880,22 +880,22 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>508</v>
+        <v>456.55</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>497.25</v>
+        <v>449.25</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>504.95</v>
+        <v>510.4</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>498.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="12">
@@ -905,22 +905,22 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>209.9</v>
+        <v>456.55</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>206.81</v>
+        <v>449.25</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>208.65</v>
+        <v>231.79</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>208.18</v>
+        <v>231.58</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>208.94</v>
+        <v>450</v>
       </c>
     </row>
     <row r="13">
@@ -930,22 +930,22 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>1775</v>
+        <v>456.55</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>1740</v>
+        <v>449.25</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>1768.5</v>
+        <v>1806</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1770.35</v>
+        <v>1808.45</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1753.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="14">
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>7877.95</v>
+        <v>456.55</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>7670.05</v>
+        <v>449.25</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>7877.95</v>
+        <v>7252.4</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>7841.9</v>
+        <v>7224.45</v>
       </c>
       <c r="F14" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>7694</v>
+        <v>450</v>
       </c>
     </row>
     <row r="15">
@@ -980,22 +980,22 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>616</v>
+        <v>456.55</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>606.15</v>
+        <v>449.25</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>614.5</v>
+        <v>587.3</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>612.45</v>
+        <v>585.8</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>610.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="16">
@@ -1005,22 +1005,22 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>1406.7</v>
+        <v>456.55</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>1388.95</v>
+        <v>449.25</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1395</v>
+        <v>1244</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1396.5</v>
+        <v>1238.4</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1403.25</v>
+        <v>450</v>
       </c>
     </row>
     <row r="17">
@@ -1030,22 +1030,22 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>10012.25</v>
+        <v>456.55</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>9805</v>
+        <v>449.25</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>9827</v>
+        <v>9020</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>9836.299999999999</v>
+        <v>9013.5</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>10001.05</v>
+        <v>450</v>
       </c>
     </row>
     <row r="18">
@@ -1055,22 +1055,22 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>1755</v>
+        <v>456.55</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>1725.05</v>
+        <v>449.25</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1748</v>
+        <v>1582.3</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>1750.75</v>
+        <v>1575.05</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1742.85</v>
+        <v>450</v>
       </c>
     </row>
     <row r="19">
@@ -1080,22 +1080,22 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>6970.8</v>
+        <v>456.55</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>6879.75</v>
+        <v>449.25</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>6897.35</v>
+        <v>6539</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>6889.75</v>
+        <v>6509.4</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>6918</v>
+        <v>450</v>
       </c>
     </row>
     <row r="20">
@@ -1105,22 +1105,22 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>2863</v>
+        <v>456.55</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>2821.65</v>
+        <v>449.25</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>2859</v>
+        <v>2722.05</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>2837.45</v>
+        <v>2717.95</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>2862.95</v>
+        <v>450</v>
       </c>
     </row>
     <row r="21">
@@ -1130,22 +1130,22 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>657.3</v>
+        <v>456.55</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>611.6</v>
+        <v>449.25</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>620</v>
+        <v>560.2</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>627.8</v>
+        <v>561.1</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>654.6</v>
+        <v>450</v>
       </c>
     </row>
     <row r="22">
@@ -1155,22 +1155,22 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>183.25</v>
+        <v>456.55</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>176.77</v>
+        <v>449.25</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>182.5</v>
+        <v>171.49</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>182.21</v>
+        <v>170.96</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>169</v>
+        <v>80</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>177.4</v>
+        <v>450</v>
       </c>
     </row>
     <row r="23">
@@ -1180,22 +1180,22 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>254.18</v>
+        <v>456.55</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>248.2</v>
+        <v>449.25</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>252.25</v>
+        <v>250.15</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>250.96</v>
+        <v>249</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>251.85</v>
+        <v>450</v>
       </c>
     </row>
     <row r="24">
@@ -1205,22 +1205,22 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>1370</v>
+        <v>456.55</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>1346.55</v>
+        <v>449.25</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>1357</v>
+        <v>1358.05</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1355.65</v>
+        <v>1362.25</v>
       </c>
       <c r="F24" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1358.25</v>
+        <v>450</v>
       </c>
     </row>
     <row r="25">
@@ -1230,22 +1230,22 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>288.45</v>
+        <v>456.55</v>
       </c>
       <c r="C25" s="10" t="n">
-        <v>283.75</v>
+        <v>449.25</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>285.15</v>
+        <v>305.8</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>284.9</v>
+        <v>305.75</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>187</v>
+        <v>277</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>285.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="26">
@@ -1255,22 +1255,22 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>1440.85</v>
+        <v>456.55</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>1395.25</v>
+        <v>449.25</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>1411.05</v>
+        <v>1332</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>1410.15</v>
+        <v>1329.2</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>1427.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="27">
@@ -1280,22 +1280,22 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>240.8</v>
+        <v>456.55</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>233.5</v>
+        <v>449.25</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>239</v>
+        <v>253.15</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>239</v>
+        <v>252.49</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>143</v>
+        <v>177</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>234.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="28">
@@ -1305,22 +1305,22 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>323.1</v>
+        <v>456.55</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>311.2</v>
+        <v>449.25</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>315.85</v>
+        <v>364.95</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>316.1</v>
+        <v>363.95</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>136</v>
+        <v>39</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>314.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="29">
@@ -1330,22 +1330,22 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>5757.4</v>
+        <v>456.55</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>5708</v>
+        <v>449.25</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>5730</v>
+        <v>4930</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>5726.9</v>
+        <v>4923.65</v>
       </c>
       <c r="F29" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>5743.7</v>
+        <v>450</v>
       </c>
     </row>
     <row r="30">
@@ -1355,22 +1355,22 @@
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>565.45</v>
+        <v>456.55</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>547.45</v>
+        <v>449.25</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>548.95</v>
+        <v>592.3</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>550.1</v>
+        <v>591.2</v>
       </c>
       <c r="F30" s="16" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>564.65</v>
+        <v>450</v>
       </c>
     </row>
     <row r="31">
@@ -1380,22 +1380,22 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>104.15</v>
+        <v>456.55</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>102.15</v>
+        <v>449.25</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>103.02</v>
+        <v>103.34</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>102.65</v>
+        <v>102.9</v>
       </c>
       <c r="F31" s="16" t="n">
-        <v>154</v>
+        <v>215</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>103.15</v>
+        <v>450</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -1405,22 +1405,22 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>882.95</v>
+        <v>456.55</v>
       </c>
       <c r="C32" s="10" t="n">
-        <v>861.7</v>
+        <v>449.25</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>869</v>
+        <v>823</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>867.95</v>
+        <v>821.85</v>
       </c>
       <c r="F32" s="16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>878.6</v>
+        <v>450</v>
       </c>
     </row>
     <row r="33">
@@ -1430,22 +1430,22 @@
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>487.7</v>
+        <v>456.55</v>
       </c>
       <c r="C33" s="10" t="n">
-        <v>472.5</v>
+        <v>449.25</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>484</v>
+        <v>498</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>483.6</v>
+        <v>498</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>473.35</v>
+        <v>450</v>
       </c>
     </row>
     <row r="34">
@@ -1455,22 +1455,22 @@
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>1281.4</v>
+        <v>456.55</v>
       </c>
       <c r="C34" s="10" t="n">
-        <v>1251.5</v>
+        <v>449.25</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>1270</v>
+        <v>1268.05</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>1272.75</v>
+        <v>1268.35</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>1260.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="35">
@@ -1480,22 +1480,22 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>1565.95</v>
+        <v>456.55</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>1518.05</v>
+        <v>449.25</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>1553</v>
+        <v>1498.15</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>1551.75</v>
+        <v>1492.75</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>174</v>
+        <v>43</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>1528.95</v>
+        <v>450</v>
       </c>
     </row>
     <row r="36">
@@ -1505,22 +1505,22 @@
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>7649.8</v>
+        <v>456.55</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>7420</v>
+        <v>449.25</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>7601</v>
+        <v>8630.700000000001</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>7624.1</v>
+        <v>8661.049999999999</v>
       </c>
       <c r="F36" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>7617.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="37">
@@ -1530,22 +1530,22 @@
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>853</v>
+        <v>456.55</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>836.8</v>
+        <v>449.25</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>844</v>
+        <v>824.65</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>847.1</v>
+        <v>821.2</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>845.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="38">
@@ -1555,22 +1555,22 @@
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>1677.2</v>
+        <v>456.55</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>1636.05</v>
+        <v>449.25</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>1667.1</v>
+        <v>1765</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>1668.65</v>
+        <v>1755.75</v>
       </c>
       <c r="F38" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1647.6</v>
+        <v>450</v>
       </c>
     </row>
     <row r="39">
@@ -1580,22 +1580,22 @@
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>396.5</v>
+        <v>456.55</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>389.1</v>
+        <v>449.25</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>392.9</v>
+        <v>406.05</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>391</v>
+        <v>406.65</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>390</v>
+        <v>450</v>
       </c>
     </row>
     <row r="40">
@@ -1605,22 +1605,22 @@
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>3562.95</v>
+        <v>456.55</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>3461.55</v>
+        <v>449.25</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>3495.7</v>
+        <v>3481</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>3500.6</v>
+        <v>3481.25</v>
       </c>
       <c r="F40" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>3547.25</v>
+        <v>450</v>
       </c>
     </row>
     <row r="41">
@@ -1630,22 +1630,22 @@
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>547.2</v>
+        <v>456.55</v>
       </c>
       <c r="C41" s="10" t="n">
-        <v>538.4</v>
+        <v>449.25</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>541.25</v>
+        <v>525.7</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>540</v>
+        <v>526</v>
       </c>
       <c r="F41" s="16" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>547</v>
+        <v>450</v>
       </c>
     </row>
     <row r="42">
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>1863.9</v>
+        <v>456.55</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>1818.15</v>
+        <v>449.25</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>1838</v>
+        <v>1822</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>1833.2</v>
+        <v>1819.3</v>
       </c>
       <c r="F42" s="16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>1832.55</v>
+        <v>450</v>
       </c>
     </row>
     <row r="43">
@@ -1680,22 +1680,22 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>1263</v>
+        <v>456.55</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>1189</v>
+        <v>449.25</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>1246</v>
+        <v>1346.2</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>1251.45</v>
+        <v>1352.65</v>
       </c>
       <c r="F43" s="16" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>1196.45</v>
+        <v>450</v>
       </c>
     </row>
     <row r="44">
@@ -1705,22 +1705,22 @@
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>2695.3</v>
+        <v>456.55</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>2611.1</v>
+        <v>449.25</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>2644</v>
+        <v>2718</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>2636.3</v>
+        <v>2706</v>
       </c>
       <c r="F44" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>2687</v>
+        <v>450</v>
       </c>
     </row>
     <row r="45">
@@ -1730,22 +1730,22 @@
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>116.89</v>
+        <v>456.55</v>
       </c>
       <c r="C45" s="10" t="n">
-        <v>115.95</v>
+        <v>449.25</v>
       </c>
       <c r="D45" s="13" t="n">
-        <v>116.55</v>
+        <v>116</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>116.19</v>
+        <v>115.84</v>
       </c>
       <c r="F45" s="16" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>116.46</v>
+        <v>450</v>
       </c>
     </row>
     <row r="46">
@@ -1755,22 +1755,22 @@
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>5912.15</v>
+        <v>456.55</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>5858.65</v>
+        <v>449.25</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>5875</v>
+        <v>5967.05</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>5889.65</v>
+        <v>5951.8</v>
       </c>
       <c r="F46" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>5878</v>
+        <v>450</v>
       </c>
     </row>
     <row r="47">
@@ -1780,22 +1780,22 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>14210.95</v>
+        <v>456.55</v>
       </c>
       <c r="C47" s="10" t="n">
-        <v>13920.2</v>
+        <v>449.25</v>
       </c>
       <c r="D47" s="13" t="n">
-        <v>14100</v>
+        <v>15635</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>14061.6</v>
+        <v>15608.2</v>
       </c>
       <c r="F47" s="16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>14157.95</v>
+        <v>450</v>
       </c>
     </row>
     <row r="48">
@@ -1805,22 +1805,22 @@
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>828.7</v>
+        <v>456.55</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>814.3</v>
+        <v>449.25</v>
       </c>
       <c r="D48" s="13" t="n">
-        <v>819.7</v>
+        <v>815.4</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>819.85</v>
+        <v>813.85</v>
       </c>
       <c r="F48" s="16" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>824.6</v>
+        <v>450</v>
       </c>
     </row>
     <row r="49">
@@ -1830,22 +1830,22 @@
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>1283.65</v>
+        <v>456.55</v>
       </c>
       <c r="C49" s="10" t="n">
-        <v>1248</v>
+        <v>449.25</v>
       </c>
       <c r="D49" s="13" t="n">
-        <v>1274</v>
+        <v>1197.85</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>1274.2</v>
+        <v>1191.95</v>
       </c>
       <c r="F49" s="16" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>1263.35</v>
+        <v>450</v>
       </c>
     </row>
     <row r="50">
@@ -1855,22 +1855,22 @@
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>3777</v>
+        <v>456.55</v>
       </c>
       <c r="C50" s="10" t="n">
-        <v>3630.05</v>
+        <v>449.25</v>
       </c>
       <c r="D50" s="13" t="n">
-        <v>3772</v>
+        <v>3515</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>3745.1</v>
+        <v>3513.35</v>
       </c>
       <c r="F50" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>3665.95</v>
+        <v>450</v>
       </c>
     </row>
     <row r="51">
@@ -1880,22 +1880,22 @@
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>462.35</v>
+        <v>456.55</v>
       </c>
       <c r="C51" s="10" t="n">
-        <v>451.5</v>
+        <v>449.25</v>
       </c>
       <c r="D51" s="13" t="n">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>455.45</v>
+        <v>457.05</v>
       </c>
       <c r="F51" s="16" t="n">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>454.1</v>
+        <v>450</v>
       </c>
     </row>
     <row r="52">
@@ -1905,22 +1905,22 @@
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>1699</v>
+        <v>456.55</v>
       </c>
       <c r="C52" s="10" t="n">
-        <v>1668.7</v>
+        <v>449.25</v>
       </c>
       <c r="D52" s="13" t="n">
-        <v>1698.8</v>
+        <v>1505</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>1694.55</v>
+        <v>1495.15</v>
       </c>
       <c r="F52" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>1680.7</v>
+        <v>450</v>
       </c>
     </row>
     <row r="53">
@@ -1930,22 +1930,22 @@
         </is>
       </c>
       <c r="B53" s="8" t="n">
-        <v>1065.3</v>
+        <v>456.55</v>
       </c>
       <c r="C53" s="10" t="n">
-        <v>1018.2</v>
+        <v>449.25</v>
       </c>
       <c r="D53" s="13" t="n">
-        <v>1050</v>
+        <v>1071</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>1057.2</v>
+        <v>1080.6</v>
       </c>
       <c r="F53" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>1033.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="54">
@@ -1955,22 +1955,22 @@
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>631.35</v>
+        <v>456.55</v>
       </c>
       <c r="C54" s="10" t="n">
-        <v>622.7</v>
+        <v>449.25</v>
       </c>
       <c r="D54" s="13" t="n">
-        <v>626.8</v>
+        <v>614</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>625.15</v>
+        <v>614.25</v>
       </c>
       <c r="F54" s="16" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G54" s="5" t="n">
-        <v>624</v>
+        <v>450</v>
       </c>
     </row>
     <row r="55">
@@ -1980,22 +1980,22 @@
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>1291.65</v>
+        <v>456.55</v>
       </c>
       <c r="C55" s="10" t="n">
-        <v>1277.2</v>
+        <v>449.25</v>
       </c>
       <c r="D55" s="13" t="n">
-        <v>1284.15</v>
+        <v>1247.2</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1283.15</v>
+        <v>1251.25</v>
       </c>
       <c r="F55" s="16" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="G55" s="5" t="n">
-        <v>1291</v>
+        <v>450</v>
       </c>
     </row>
     <row r="56">
@@ -2005,22 +2005,22 @@
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>2895</v>
+        <v>456.55</v>
       </c>
       <c r="C56" s="10" t="n">
-        <v>2835.1</v>
+        <v>449.25</v>
       </c>
       <c r="D56" s="13" t="n">
-        <v>2883.5</v>
+        <v>2819</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>2875.7</v>
+        <v>2815.75</v>
       </c>
       <c r="F56" s="16" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G56" s="5" t="n">
-        <v>2848.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="57">
@@ -2030,22 +2030,22 @@
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>572</v>
+        <v>456.55</v>
       </c>
       <c r="C57" s="10" t="n">
-        <v>554.45</v>
+        <v>449.25</v>
       </c>
       <c r="D57" s="13" t="n">
-        <v>572</v>
+        <v>583.45</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>569.6</v>
+        <v>583.65</v>
       </c>
       <c r="F57" s="16" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>556.15</v>
+        <v>450</v>
       </c>
     </row>
     <row r="58">
@@ -2055,22 +2055,22 @@
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>2704</v>
+        <v>456.55</v>
       </c>
       <c r="C58" s="10" t="n">
-        <v>2644.45</v>
+        <v>449.25</v>
       </c>
       <c r="D58" s="13" t="n">
-        <v>2703.5</v>
+        <v>2586</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>2695.85</v>
+        <v>2570.45</v>
       </c>
       <c r="F58" s="16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>2661.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="59">
@@ -2080,22 +2080,22 @@
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>526.5</v>
+        <v>456.55</v>
       </c>
       <c r="C59" s="10" t="n">
-        <v>517</v>
+        <v>449.25</v>
       </c>
       <c r="D59" s="13" t="n">
-        <v>521</v>
+        <v>474</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>519.15</v>
+        <v>472</v>
       </c>
       <c r="F59" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G59" s="5" t="n">
-        <v>524.55</v>
+        <v>450</v>
       </c>
     </row>
     <row r="60">
@@ -2105,22 +2105,22 @@
         </is>
       </c>
       <c r="B60" s="8" t="n">
-        <v>4270.2</v>
+        <v>456.55</v>
       </c>
       <c r="C60" s="10" t="n">
-        <v>4201</v>
+        <v>449.25</v>
       </c>
       <c r="D60" s="13" t="n">
-        <v>4254</v>
+        <v>4459</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>4246.7</v>
+        <v>4466.85</v>
       </c>
       <c r="F60" s="16" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G60" s="5" t="n">
-        <v>4215.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="61">
@@ -2130,22 +2130,22 @@
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>1658.65</v>
+        <v>456.55</v>
       </c>
       <c r="C61" s="10" t="n">
-        <v>1632.6</v>
+        <v>449.25</v>
       </c>
       <c r="D61" s="13" t="n">
-        <v>1641</v>
+        <v>1711.4</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>1638.4</v>
+        <v>1717.6</v>
       </c>
       <c r="F61" s="16" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="G61" s="5" t="n">
-        <v>1654.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="62">
@@ -2155,22 +2155,22 @@
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>1819.9</v>
+        <v>456.55</v>
       </c>
       <c r="C62" s="10" t="n">
-        <v>1756.55</v>
+        <v>449.25</v>
       </c>
       <c r="D62" s="13" t="n">
-        <v>1772.5</v>
+        <v>1844</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>1766.05</v>
+        <v>1840.9</v>
       </c>
       <c r="F62" s="16" t="n">
         <v>36</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>1817.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="63">
@@ -2180,22 +2180,22 @@
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>4375.45</v>
+        <v>456.55</v>
       </c>
       <c r="C63" s="10" t="n">
-        <v>4258.5</v>
+        <v>449.25</v>
       </c>
       <c r="D63" s="13" t="n">
-        <v>4299.85</v>
+        <v>4270</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>4299.45</v>
+        <v>4209.75</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>4354.35</v>
+        <v>450</v>
       </c>
     </row>
     <row r="64">
@@ -2205,22 +2205,22 @@
         </is>
       </c>
       <c r="B64" s="8" t="n">
-        <v>723.5</v>
+        <v>456.55</v>
       </c>
       <c r="C64" s="10" t="n">
-        <v>713.15</v>
+        <v>449.25</v>
       </c>
       <c r="D64" s="13" t="n">
-        <v>720</v>
+        <v>655.1</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>720.15</v>
+        <v>657.7</v>
       </c>
       <c r="F64" s="16" t="n">
-        <v>20</v>
+        <v>136</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>717.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="65">
@@ -2230,22 +2230,22 @@
         </is>
       </c>
       <c r="B65" s="8" t="n">
-        <v>689.55</v>
+        <v>456.55</v>
       </c>
       <c r="C65" s="10" t="n">
-        <v>679.25</v>
+        <v>449.25</v>
       </c>
       <c r="D65" s="13" t="n">
-        <v>684.1</v>
+        <v>651.95</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>686.05</v>
+        <v>650.25</v>
       </c>
       <c r="F65" s="16" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>685.4</v>
+        <v>450</v>
       </c>
     </row>
     <row r="66">
@@ -2255,22 +2255,22 @@
         </is>
       </c>
       <c r="B66" s="8" t="n">
-        <v>295</v>
+        <v>456.55</v>
       </c>
       <c r="C66" s="10" t="n">
-        <v>288.35</v>
+        <v>449.25</v>
       </c>
       <c r="D66" s="13" t="n">
-        <v>293.85</v>
+        <v>274.9</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>294.2</v>
+        <v>274.85</v>
       </c>
       <c r="F66" s="16" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>289.35</v>
+        <v>450</v>
       </c>
     </row>
     <row r="67">
@@ -2280,22 +2280,22 @@
         </is>
       </c>
       <c r="B67" s="8" t="n">
-        <v>1928.6</v>
+        <v>456.55</v>
       </c>
       <c r="C67" s="10" t="n">
-        <v>1892.9</v>
+        <v>449.25</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>1918.8</v>
+        <v>1879.8</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1917.35</v>
+        <v>1871.1</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>1910.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="68">
@@ -2305,22 +2305,22 @@
         </is>
       </c>
       <c r="B68" s="8" t="n">
-        <v>756</v>
+        <v>456.55</v>
       </c>
       <c r="C68" s="10" t="n">
-        <v>736.4</v>
+        <v>449.25</v>
       </c>
       <c r="D68" s="13" t="n">
-        <v>742</v>
+        <v>693</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>741</v>
+        <v>691.85</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>739.1</v>
+        <v>450</v>
       </c>
     </row>
     <row r="69">
@@ -2330,22 +2330,22 @@
         </is>
       </c>
       <c r="B69" s="8" t="n">
-        <v>179.5</v>
+        <v>456.55</v>
       </c>
       <c r="C69" s="10" t="n">
-        <v>174.82</v>
+        <v>449.25</v>
       </c>
       <c r="D69" s="13" t="n">
-        <v>177.6</v>
+        <v>175.09</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>177.76</v>
+        <v>174.9</v>
       </c>
       <c r="F69" s="16" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G69" s="5" t="n">
-        <v>176.05</v>
+        <v>450</v>
       </c>
     </row>
     <row r="70">
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="B70" s="8" t="n">
-        <v>421.85</v>
+        <v>456.55</v>
       </c>
       <c r="C70" s="10" t="n">
-        <v>415.65</v>
+        <v>449.25</v>
       </c>
       <c r="D70" s="13" t="n">
-        <v>420.1</v>
+        <v>319.1</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>420.15</v>
+        <v>319.45</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="G70" s="5" t="n">
-        <v>420.15</v>
+        <v>450</v>
       </c>
     </row>
     <row r="71">
@@ -2380,22 +2380,22 @@
         </is>
       </c>
       <c r="B71" s="8" t="n">
-        <v>680.5</v>
+        <v>456.55</v>
       </c>
       <c r="C71" s="10" t="n">
-        <v>669.1</v>
+        <v>449.25</v>
       </c>
       <c r="D71" s="13" t="n">
-        <v>676.3</v>
+        <v>781.9</v>
       </c>
       <c r="E71" s="5" t="n">
-        <v>676.7</v>
+        <v>778.55</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="G71" s="5" t="n">
-        <v>673</v>
+        <v>450</v>
       </c>
     </row>
     <row r="72">
@@ -2405,22 +2405,22 @@
         </is>
       </c>
       <c r="B72" s="8" t="n">
-        <v>364.5</v>
+        <v>456.55</v>
       </c>
       <c r="C72" s="10" t="n">
-        <v>358.15</v>
+        <v>449.25</v>
       </c>
       <c r="D72" s="13" t="n">
-        <v>363.95</v>
+        <v>363.85</v>
       </c>
       <c r="E72" s="5" t="n">
-        <v>363.9</v>
+        <v>363.1</v>
       </c>
       <c r="F72" s="16" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>358.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="73">
@@ -2430,22 +2430,22 @@
         </is>
       </c>
       <c r="B73" s="8" t="n">
-        <v>2555.75</v>
+        <v>456.55</v>
       </c>
       <c r="C73" s="10" t="n">
-        <v>2488.5</v>
+        <v>449.25</v>
       </c>
       <c r="D73" s="13" t="n">
-        <v>2499.75</v>
+        <v>2351</v>
       </c>
       <c r="E73" s="5" t="n">
-        <v>2500</v>
+        <v>2341.4</v>
       </c>
       <c r="F73" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>2539</v>
+        <v>450</v>
       </c>
     </row>
     <row r="74">
@@ -2455,22 +2455,22 @@
         </is>
       </c>
       <c r="B74" s="8" t="n">
-        <v>4072.7</v>
+        <v>456.55</v>
       </c>
       <c r="C74" s="10" t="n">
-        <v>4010.05</v>
+        <v>449.25</v>
       </c>
       <c r="D74" s="13" t="n">
-        <v>4049.55</v>
+        <v>4355</v>
       </c>
       <c r="E74" s="5" t="n">
-        <v>4052.5</v>
+        <v>4352.65</v>
       </c>
       <c r="F74" s="16" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G74" s="5" t="n">
-        <v>4052</v>
+        <v>450</v>
       </c>
     </row>
     <row r="75">
@@ -2480,22 +2480,22 @@
         </is>
       </c>
       <c r="B75" s="8" t="n">
-        <v>1066.9</v>
+        <v>456.55</v>
       </c>
       <c r="C75" s="10" t="n">
-        <v>1044</v>
+        <v>449.25</v>
       </c>
       <c r="D75" s="13" t="n">
-        <v>1055</v>
+        <v>993.75</v>
       </c>
       <c r="E75" s="5" t="n">
-        <v>1055.6</v>
+        <v>993.6</v>
       </c>
       <c r="F75" s="16" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G75" s="5" t="n">
-        <v>1050.4</v>
+        <v>450</v>
       </c>
     </row>
     <row r="76">
@@ -2505,22 +2505,22 @@
         </is>
       </c>
       <c r="B76" s="8" t="n">
-        <v>345.25</v>
+        <v>456.55</v>
       </c>
       <c r="C76" s="10" t="n">
-        <v>338.65</v>
+        <v>449.25</v>
       </c>
       <c r="D76" s="13" t="n">
-        <v>340.6</v>
+        <v>349.9</v>
       </c>
       <c r="E76" s="5" t="n">
-        <v>340.55</v>
+        <v>348.25</v>
       </c>
       <c r="F76" s="16" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="G76" s="5" t="n">
-        <v>343.25</v>
+        <v>450</v>
       </c>
     </row>
     <row r="77">
@@ -2530,22 +2530,22 @@
         </is>
       </c>
       <c r="B77" s="8" t="n">
-        <v>755.8</v>
+        <v>456.55</v>
       </c>
       <c r="C77" s="10" t="n">
-        <v>730</v>
+        <v>449.25</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>733.05</v>
+        <v>716.8</v>
       </c>
       <c r="E77" s="5" t="n">
-        <v>736.15</v>
+        <v>717</v>
       </c>
       <c r="F77" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G77" s="5" t="n">
-        <v>750.4</v>
+        <v>450</v>
       </c>
     </row>
     <row r="78">
@@ -2555,22 +2555,22 @@
         </is>
       </c>
       <c r="B78" s="8" t="n">
-        <v>1596</v>
+        <v>456.55</v>
       </c>
       <c r="C78" s="10" t="n">
-        <v>1562.65</v>
+        <v>449.25</v>
       </c>
       <c r="D78" s="13" t="n">
-        <v>1593.75</v>
+        <v>1515</v>
       </c>
       <c r="E78" s="5" t="n">
-        <v>1588.8</v>
+        <v>1513</v>
       </c>
       <c r="F78" s="16" t="n">
         <v>5</v>
       </c>
       <c r="G78" s="5" t="n">
-        <v>1569.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="79">
@@ -2580,22 +2580,22 @@
         </is>
       </c>
       <c r="B79" s="8" t="n">
-        <v>931.7</v>
+        <v>456.55</v>
       </c>
       <c r="C79" s="10" t="n">
-        <v>911.55</v>
+        <v>449.25</v>
       </c>
       <c r="D79" s="13" t="n">
-        <v>919</v>
+        <v>899</v>
       </c>
       <c r="E79" s="5" t="n">
-        <v>920.5</v>
+        <v>897</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G79" s="5" t="n">
-        <v>922.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="80">
@@ -2605,22 +2605,22 @@
         </is>
       </c>
       <c r="B80" s="8" t="n">
-        <v>4352.3</v>
+        <v>456.55</v>
       </c>
       <c r="C80" s="10" t="n">
-        <v>4276.3</v>
+        <v>449.25</v>
       </c>
       <c r="D80" s="13" t="n">
-        <v>4301.35</v>
+        <v>4200</v>
       </c>
       <c r="E80" s="5" t="n">
-        <v>4322.3</v>
+        <v>4144</v>
       </c>
       <c r="F80" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>4314.7</v>
+        <v>450</v>
       </c>
     </row>
     <row r="81">
@@ -2630,22 +2630,22 @@
         </is>
       </c>
       <c r="B81" s="8" t="n">
-        <v>967.85</v>
+        <v>456.55</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>955.1</v>
+        <v>449.25</v>
       </c>
       <c r="D81" s="13" t="n">
-        <v>963.65</v>
+        <v>958.5</v>
       </c>
       <c r="E81" s="5" t="n">
-        <v>963.65</v>
+        <v>954.15</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G81" s="5" t="n">
-        <v>958.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="82">
@@ -2655,22 +2655,22 @@
         </is>
       </c>
       <c r="B82" s="8" t="n">
-        <v>579.7</v>
+        <v>456.55</v>
       </c>
       <c r="C82" s="10" t="n">
-        <v>570.1</v>
+        <v>449.25</v>
       </c>
       <c r="D82" s="13" t="n">
-        <v>574</v>
+        <v>642.6</v>
       </c>
       <c r="E82" s="5" t="n">
-        <v>576</v>
+        <v>642.3</v>
       </c>
       <c r="F82" s="16" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>576.55</v>
+        <v>450</v>
       </c>
     </row>
     <row r="83">
@@ -2680,22 +2680,22 @@
         </is>
       </c>
       <c r="B83" s="8" t="n">
-        <v>1746.6</v>
+        <v>456.55</v>
       </c>
       <c r="C83" s="10" t="n">
-        <v>1723.95</v>
+        <v>449.25</v>
       </c>
       <c r="D83" s="13" t="n">
-        <v>1736</v>
+        <v>1763.8</v>
       </c>
       <c r="E83" s="5" t="n">
-        <v>1731.1</v>
+        <v>1759.2</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G83" s="5" t="n">
-        <v>1728.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="84">
@@ -2705,22 +2705,22 @@
         </is>
       </c>
       <c r="B84" s="8" t="n">
-        <v>3130</v>
+        <v>456.55</v>
       </c>
       <c r="C84" s="10" t="n">
-        <v>3012.05</v>
+        <v>449.25</v>
       </c>
       <c r="D84" s="13" t="n">
-        <v>3130</v>
+        <v>2979.95</v>
       </c>
       <c r="E84" s="5" t="n">
-        <v>3113</v>
+        <v>2980.6</v>
       </c>
       <c r="F84" s="16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G84" s="5" t="n">
-        <v>3058.65</v>
+        <v>450</v>
       </c>
     </row>
     <row r="85">
@@ -2730,22 +2730,22 @@
         </is>
       </c>
       <c r="B85" s="8" t="n">
-        <v>493</v>
+        <v>456.55</v>
       </c>
       <c r="C85" s="10" t="n">
-        <v>479.35</v>
+        <v>449.25</v>
       </c>
       <c r="D85" s="13" t="n">
-        <v>491</v>
+        <v>555</v>
       </c>
       <c r="E85" s="5" t="n">
-        <v>491.25</v>
+        <v>551.7</v>
       </c>
       <c r="F85" s="16" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G85" s="5" t="n">
-        <v>486.15</v>
+        <v>450</v>
       </c>
     </row>
     <row r="86">
@@ -2755,22 +2755,22 @@
         </is>
       </c>
       <c r="B86" s="8" t="n">
-        <v>635.45</v>
+        <v>456.55</v>
       </c>
       <c r="C86" s="10" t="n">
-        <v>621.45</v>
+        <v>449.25</v>
       </c>
       <c r="D86" s="13" t="n">
-        <v>632</v>
+        <v>636.2</v>
       </c>
       <c r="E86" s="5" t="n">
-        <v>631.05</v>
+        <v>634.7</v>
       </c>
       <c r="F86" s="16" t="n">
         <v>15</v>
       </c>
       <c r="G86" s="5" t="n">
-        <v>630.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="87">
@@ -2780,22 +2780,22 @@
         </is>
       </c>
       <c r="B87" s="8" t="n">
-        <v>5741.1</v>
+        <v>456.55</v>
       </c>
       <c r="C87" s="10" t="n">
-        <v>5621.2</v>
+        <v>449.25</v>
       </c>
       <c r="D87" s="13" t="n">
-        <v>5694.15</v>
+        <v>6169.95</v>
       </c>
       <c r="E87" s="5" t="n">
-        <v>5710.85</v>
+        <v>6159.75</v>
       </c>
       <c r="F87" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G87" s="5" t="n">
-        <v>5738.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="88">
@@ -2805,22 +2805,22 @@
         </is>
       </c>
       <c r="B88" s="8" t="n">
-        <v>5087.7</v>
+        <v>456.55</v>
       </c>
       <c r="C88" s="10" t="n">
-        <v>4909.3</v>
+        <v>449.25</v>
       </c>
       <c r="D88" s="13" t="n">
-        <v>4944.8</v>
+        <v>5242</v>
       </c>
       <c r="E88" s="5" t="n">
-        <v>4945.85</v>
+        <v>5249.65</v>
       </c>
       <c r="F88" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G88" s="5" t="n">
-        <v>5078.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="89">
@@ -2830,22 +2830,22 @@
         </is>
       </c>
       <c r="B89" s="8" t="n">
-        <v>2200</v>
+        <v>456.55</v>
       </c>
       <c r="C89" s="10" t="n">
-        <v>2148.35</v>
+        <v>449.25</v>
       </c>
       <c r="D89" s="13" t="n">
-        <v>2194.95</v>
+        <v>2000</v>
       </c>
       <c r="E89" s="5" t="n">
-        <v>2186.95</v>
+        <v>1998.4</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G89" s="5" t="n">
-        <v>2168.05</v>
+        <v>450</v>
       </c>
     </row>
     <row r="90">
@@ -2855,22 +2855,22 @@
         </is>
       </c>
       <c r="B90" s="8" t="n">
-        <v>274.55</v>
+        <v>456.55</v>
       </c>
       <c r="C90" s="10" t="n">
-        <v>266.7</v>
+        <v>449.25</v>
       </c>
       <c r="D90" s="13" t="n">
-        <v>269.8</v>
+        <v>272.85</v>
       </c>
       <c r="E90" s="5" t="n">
-        <v>270.6</v>
+        <v>272</v>
       </c>
       <c r="F90" s="16" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="G90" s="5" t="n">
-        <v>274.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="91">
@@ -2880,22 +2880,22 @@
         </is>
       </c>
       <c r="B91" s="8" t="n">
-        <v>157.95</v>
+        <v>456.55</v>
       </c>
       <c r="C91" s="10" t="n">
-        <v>154.29</v>
+        <v>449.25</v>
       </c>
       <c r="D91" s="13" t="n">
-        <v>157</v>
+        <v>157.2</v>
       </c>
       <c r="E91" s="5" t="n">
-        <v>157.05</v>
+        <v>156.71</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>176</v>
+        <v>69</v>
       </c>
       <c r="G91" s="5" t="n">
-        <v>156.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="92">
@@ -2905,22 +2905,22 @@
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>648.35</v>
+        <v>456.55</v>
       </c>
       <c r="C92" s="10" t="n">
-        <v>632.85</v>
+        <v>449.25</v>
       </c>
       <c r="D92" s="13" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E92" s="5" t="n">
-        <v>640</v>
+        <v>644.85</v>
       </c>
       <c r="F92" s="16" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="G92" s="5" t="n">
-        <v>647.95</v>
+        <v>450</v>
       </c>
     </row>
     <row r="93">
@@ -2930,22 +2930,22 @@
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>1454</v>
+        <v>456.55</v>
       </c>
       <c r="C93" s="10" t="n">
-        <v>1426.6</v>
+        <v>449.25</v>
       </c>
       <c r="D93" s="13" t="n">
-        <v>1450.2</v>
+        <v>1506.85</v>
       </c>
       <c r="E93" s="5" t="n">
-        <v>1449.1</v>
+        <v>1502.75</v>
       </c>
       <c r="F93" s="16" t="n">
         <v>5</v>
       </c>
       <c r="G93" s="5" t="n">
-        <v>1446.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="94">
@@ -2955,22 +2955,22 @@
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>6541.6</v>
+        <v>456.55</v>
       </c>
       <c r="C94" s="10" t="n">
-        <v>6390</v>
+        <v>449.25</v>
       </c>
       <c r="D94" s="13" t="n">
-        <v>6509</v>
+        <v>6087.15</v>
       </c>
       <c r="E94" s="5" t="n">
-        <v>6515.9</v>
+        <v>6103.65</v>
       </c>
       <c r="F94" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G94" s="5" t="n">
-        <v>6453.65</v>
+        <v>450</v>
       </c>
     </row>
     <row r="95">
@@ -2980,22 +2980,22 @@
         </is>
       </c>
       <c r="B95" s="8" t="n">
-        <v>2172.85</v>
+        <v>456.55</v>
       </c>
       <c r="C95" s="10" t="n">
-        <v>2123.8</v>
+        <v>449.25</v>
       </c>
       <c r="D95" s="13" t="n">
-        <v>2139.95</v>
+        <v>2130.95</v>
       </c>
       <c r="E95" s="5" t="n">
-        <v>2146.2</v>
+        <v>2139.85</v>
       </c>
       <c r="F95" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G95" s="5" t="n">
-        <v>2161.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="96">
@@ -3005,22 +3005,22 @@
         </is>
       </c>
       <c r="B96" s="8" t="n">
-        <v>1287</v>
+        <v>456.55</v>
       </c>
       <c r="C96" s="10" t="n">
-        <v>1250.35</v>
+        <v>449.25</v>
       </c>
       <c r="D96" s="13" t="n">
-        <v>1284</v>
+        <v>1149</v>
       </c>
       <c r="E96" s="5" t="n">
-        <v>1283</v>
+        <v>1140.3</v>
       </c>
       <c r="F96" s="16" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="G96" s="5" t="n">
-        <v>1255.85</v>
+        <v>450</v>
       </c>
     </row>
     <row r="97">
@@ -3030,22 +3030,22 @@
         </is>
       </c>
       <c r="B97" s="8" t="n">
-        <v>1448.75</v>
+        <v>456.55</v>
       </c>
       <c r="C97" s="10" t="n">
-        <v>1417.3</v>
+        <v>449.25</v>
       </c>
       <c r="D97" s="13" t="n">
-        <v>1441.4</v>
+        <v>1184</v>
       </c>
       <c r="E97" s="5" t="n">
-        <v>1441.6</v>
+        <v>1179.95</v>
       </c>
       <c r="F97" s="16" t="n">
         <v>5</v>
       </c>
       <c r="G97" s="5" t="n">
-        <v>1433.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="98">
@@ -3055,22 +3055,22 @@
         </is>
       </c>
       <c r="B98" s="8" t="n">
-        <v>2936.95</v>
+        <v>456.55</v>
       </c>
       <c r="C98" s="10" t="n">
-        <v>2852.3</v>
+        <v>449.25</v>
       </c>
       <c r="D98" s="13" t="n">
-        <v>2883.5</v>
+        <v>2963</v>
       </c>
       <c r="E98" s="5" t="n">
-        <v>2879.55</v>
+        <v>2957.6</v>
       </c>
       <c r="F98" s="16" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G98" s="5" t="n">
-        <v>2925.45</v>
+        <v>450</v>
       </c>
     </row>
     <row r="99">
@@ -3080,22 +3080,22 @@
         </is>
       </c>
       <c r="B99" s="8" t="n">
-        <v>1960</v>
+        <v>456.55</v>
       </c>
       <c r="C99" s="10" t="n">
-        <v>1909.35</v>
+        <v>449.25</v>
       </c>
       <c r="D99" s="13" t="n">
-        <v>1917</v>
+        <v>1909.95</v>
       </c>
       <c r="E99" s="5" t="n">
-        <v>1930.45</v>
+        <v>1911.95</v>
       </c>
       <c r="F99" s="16" t="n">
         <v>4</v>
       </c>
       <c r="G99" s="5" t="n">
-        <v>1951.15</v>
+        <v>450</v>
       </c>
     </row>
     <row r="100">
@@ -3105,22 +3105,22 @@
         </is>
       </c>
       <c r="B100" s="8" t="n">
-        <v>710</v>
+        <v>456.55</v>
       </c>
       <c r="C100" s="10" t="n">
-        <v>687.2</v>
+        <v>449.25</v>
       </c>
       <c r="D100" s="13" t="n">
-        <v>708</v>
+        <v>689.05</v>
       </c>
       <c r="E100" s="5" t="n">
-        <v>708.2</v>
+        <v>691.05</v>
       </c>
       <c r="F100" s="16" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="G100" s="5" t="n">
-        <v>701.7</v>
+        <v>450</v>
       </c>
     </row>
     <row r="101">
@@ -3130,22 +3130,22 @@
         </is>
       </c>
       <c r="B101" s="8" t="n">
-        <v>7641.55</v>
+        <v>456.55</v>
       </c>
       <c r="C101" s="10" t="n">
-        <v>7406.55</v>
+        <v>449.25</v>
       </c>
       <c r="D101" s="13" t="n">
-        <v>7430</v>
+        <v>8208</v>
       </c>
       <c r="E101" s="5" t="n">
-        <v>7440.95</v>
+        <v>8201.950000000001</v>
       </c>
       <c r="F101" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G101" s="5" t="n">
-        <v>7637.95</v>
+        <v>450</v>
       </c>
     </row>
     <row r="102">
@@ -3155,22 +3155,22 @@
         </is>
       </c>
       <c r="B102" s="8" t="n">
-        <v>3348.45</v>
+        <v>456.55</v>
       </c>
       <c r="C102" s="10" t="n">
-        <v>3280.05</v>
+        <v>449.25</v>
       </c>
       <c r="D102" s="13" t="n">
-        <v>3330.3</v>
+        <v>3475</v>
       </c>
       <c r="E102" s="5" t="n">
-        <v>3329.85</v>
+        <v>3468.55</v>
       </c>
       <c r="F102" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G102" s="5" t="n">
-        <v>3305.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="103">
@@ -3180,22 +3180,22 @@
         </is>
       </c>
       <c r="B103" s="8" t="n">
-        <v>225.09</v>
+        <v>456.55</v>
       </c>
       <c r="C103" s="10" t="n">
-        <v>218.65</v>
+        <v>449.25</v>
       </c>
       <c r="D103" s="13" t="n">
-        <v>221.7</v>
+        <v>228.15</v>
       </c>
       <c r="E103" s="5" t="n">
-        <v>221.87</v>
+        <v>227.73</v>
       </c>
       <c r="F103" s="16" t="n">
-        <v>107</v>
+        <v>60</v>
       </c>
       <c r="G103" s="5" t="n">
-        <v>223.65</v>
+        <v>450</v>
       </c>
     </row>
     <row r="104">
@@ -3205,22 +3205,22 @@
         </is>
       </c>
       <c r="B104" s="8" t="n">
-        <v>410.65</v>
+        <v>456.55</v>
       </c>
       <c r="C104" s="10" t="n">
-        <v>403.5</v>
+        <v>449.25</v>
       </c>
       <c r="D104" s="13" t="n">
-        <v>408.3</v>
+        <v>365.25</v>
       </c>
       <c r="E104" s="5" t="n">
-        <v>408.15</v>
+        <v>362.05</v>
       </c>
       <c r="F104" s="16" t="n">
-        <v>122</v>
+        <v>168</v>
       </c>
       <c r="G104" s="5" t="n">
-        <v>404.4</v>
+        <v>450</v>
       </c>
     </row>
     <row r="105">
@@ -3230,22 +3230,22 @@
         </is>
       </c>
       <c r="B105" s="8" t="n">
-        <v>1987.6</v>
+        <v>456.55</v>
       </c>
       <c r="C105" s="10" t="n">
-        <v>1911.05</v>
+        <v>449.25</v>
       </c>
       <c r="D105" s="13" t="n">
-        <v>1980</v>
+        <v>2009.3</v>
       </c>
       <c r="E105" s="5" t="n">
-        <v>1966.8</v>
+        <v>2019.3</v>
       </c>
       <c r="F105" s="16" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G105" s="5" t="n">
-        <v>1919.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="106">
@@ -3255,22 +3255,22 @@
         </is>
       </c>
       <c r="B106" s="8" t="n">
-        <v>268.3</v>
+        <v>456.55</v>
       </c>
       <c r="C106" s="10" t="n">
-        <v>261.8</v>
+        <v>449.25</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="E106" s="5" t="n">
-        <v>266.15</v>
+        <v>252.2</v>
       </c>
       <c r="F106" s="16" t="n">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="G106" s="5" t="n">
-        <v>263</v>
+        <v>450</v>
       </c>
     </row>
     <row r="107">
@@ -3280,22 +3280,22 @@
         </is>
       </c>
       <c r="B107" s="8" t="n">
-        <v>1092.9</v>
+        <v>456.55</v>
       </c>
       <c r="C107" s="10" t="n">
-        <v>1050</v>
+        <v>449.25</v>
       </c>
       <c r="D107" s="13" t="n">
-        <v>1060.1</v>
+        <v>1181.45</v>
       </c>
       <c r="E107" s="5" t="n">
-        <v>1061.2</v>
+        <v>1180</v>
       </c>
       <c r="F107" s="16" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G107" s="5" t="n">
-        <v>1080.85</v>
+        <v>450</v>
       </c>
     </row>
     <row r="108">
@@ -3305,22 +3305,22 @@
         </is>
       </c>
       <c r="B108" s="8" t="n">
-        <v>5488.55</v>
+        <v>456.55</v>
       </c>
       <c r="C108" s="10" t="n">
-        <v>5300.05</v>
+        <v>449.25</v>
       </c>
       <c r="D108" s="13" t="n">
-        <v>5372</v>
+        <v>5832</v>
       </c>
       <c r="E108" s="5" t="n">
-        <v>5372.5</v>
+        <v>5820.65</v>
       </c>
       <c r="F108" s="16" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G108" s="5" t="n">
-        <v>5480.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="109">
@@ -3330,22 +3330,22 @@
         </is>
       </c>
       <c r="B109" s="8" t="n">
-        <v>334.7</v>
+        <v>456.55</v>
       </c>
       <c r="C109" s="10" t="n">
-        <v>327.45</v>
+        <v>449.25</v>
       </c>
       <c r="D109" s="13" t="n">
-        <v>334.1</v>
+        <v>328.45</v>
       </c>
       <c r="E109" s="5" t="n">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="F109" s="16" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="G109" s="5" t="n">
-        <v>327.85</v>
+        <v>450</v>
       </c>
     </row>
     <row r="110">
@@ -3355,22 +3355,22 @@
         </is>
       </c>
       <c r="B110" s="8" t="n">
-        <v>3165.35</v>
+        <v>456.55</v>
       </c>
       <c r="C110" s="10" t="n">
-        <v>3122.35</v>
+        <v>449.25</v>
       </c>
       <c r="D110" s="13" t="n">
-        <v>3148.05</v>
+        <v>3041.45</v>
       </c>
       <c r="E110" s="5" t="n">
-        <v>3145.85</v>
+        <v>3043.9</v>
       </c>
       <c r="F110" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G110" s="5" t="n">
-        <v>3135.45</v>
+        <v>450</v>
       </c>
     </row>
     <row r="111">
@@ -3380,22 +3380,22 @@
         </is>
       </c>
       <c r="B111" s="8" t="n">
-        <v>6500.75</v>
+        <v>456.55</v>
       </c>
       <c r="C111" s="10" t="n">
-        <v>6342</v>
+        <v>449.25</v>
       </c>
       <c r="D111" s="13" t="n">
-        <v>6479</v>
+        <v>7146.7</v>
       </c>
       <c r="E111" s="5" t="n">
-        <v>6480.4</v>
+        <v>7149.2</v>
       </c>
       <c r="F111" s="16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G111" s="5" t="n">
-        <v>6355.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="112">
@@ -3405,22 +3405,22 @@
         </is>
       </c>
       <c r="B112" s="8" t="n">
-        <v>322.7</v>
+        <v>456.55</v>
       </c>
       <c r="C112" s="10" t="n">
-        <v>318.1</v>
+        <v>449.25</v>
       </c>
       <c r="D112" s="13" t="n">
-        <v>320.8</v>
+        <v>334.3</v>
       </c>
       <c r="E112" s="5" t="n">
-        <v>320.8</v>
+        <v>333.65</v>
       </c>
       <c r="F112" s="16" t="n">
-        <v>99</v>
+        <v>169</v>
       </c>
       <c r="G112" s="5" t="n">
-        <v>318.65</v>
+        <v>450</v>
       </c>
     </row>
     <row r="113">
@@ -3430,22 +3430,22 @@
         </is>
       </c>
       <c r="B113" s="8" t="n">
-        <v>163.95</v>
+        <v>456.55</v>
       </c>
       <c r="C113" s="10" t="n">
-        <v>161</v>
+        <v>449.25</v>
       </c>
       <c r="D113" s="13" t="n">
-        <v>161.5</v>
+        <v>152.1</v>
       </c>
       <c r="E113" s="5" t="n">
-        <v>161.57</v>
+        <v>152</v>
       </c>
       <c r="F113" s="16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G113" s="5" t="n">
-        <v>162.48</v>
+        <v>450</v>
       </c>
     </row>
     <row r="114">
@@ -3455,22 +3455,22 @@
         </is>
       </c>
       <c r="B114" s="8" t="n">
-        <v>891.9</v>
+        <v>456.55</v>
       </c>
       <c r="C114" s="10" t="n">
-        <v>872.5</v>
+        <v>449.25</v>
       </c>
       <c r="D114" s="13" t="n">
-        <v>888</v>
+        <v>974</v>
       </c>
       <c r="E114" s="5" t="n">
-        <v>886.55</v>
+        <v>974.9</v>
       </c>
       <c r="F114" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G114" s="5" t="n">
-        <v>878</v>
+        <v>450</v>
       </c>
     </row>
     <row r="115">
@@ -3480,22 +3480,22 @@
         </is>
       </c>
       <c r="B115" s="8" t="n">
-        <v>179.09</v>
+        <v>456.55</v>
       </c>
       <c r="C115" s="10" t="n">
-        <v>168.2</v>
+        <v>449.25</v>
       </c>
       <c r="D115" s="13" t="n">
-        <v>168.69</v>
+        <v>158.08</v>
       </c>
       <c r="E115" s="5" t="n">
-        <v>169.75</v>
+        <v>157.49</v>
       </c>
       <c r="F115" s="16" t="n">
-        <v>201</v>
+        <v>58</v>
       </c>
       <c r="G115" s="5" t="n">
-        <v>177.32</v>
+        <v>450</v>
       </c>
     </row>
     <row r="116">
@@ -3505,22 +3505,22 @@
         </is>
       </c>
       <c r="B116" s="8" t="n">
-        <v>532</v>
+        <v>456.55</v>
       </c>
       <c r="C116" s="10" t="n">
-        <v>517</v>
+        <v>449.25</v>
       </c>
       <c r="D116" s="13" t="n">
-        <v>522.65</v>
+        <v>529.5</v>
       </c>
       <c r="E116" s="5" t="n">
-        <v>522.6</v>
+        <v>528.25</v>
       </c>
       <c r="F116" s="16" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="G116" s="5" t="n">
-        <v>527</v>
+        <v>450</v>
       </c>
     </row>
     <row r="117">
@@ -3530,22 +3530,22 @@
         </is>
       </c>
       <c r="B117" s="8" t="n">
-        <v>699.5</v>
+        <v>456.55</v>
       </c>
       <c r="C117" s="10" t="n">
-        <v>671.15</v>
+        <v>449.25</v>
       </c>
       <c r="D117" s="13" t="n">
-        <v>688.4</v>
+        <v>710.9</v>
       </c>
       <c r="E117" s="5" t="n">
-        <v>688.4</v>
+        <v>711.9</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G117" s="5" t="n">
-        <v>675.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="118">
@@ -3555,22 +3555,22 @@
         </is>
       </c>
       <c r="B118" s="8" t="n">
-        <v>1631</v>
+        <v>456.55</v>
       </c>
       <c r="C118" s="10" t="n">
-        <v>1613.05</v>
+        <v>449.25</v>
       </c>
       <c r="D118" s="13" t="n">
-        <v>1618.05</v>
+        <v>1424</v>
       </c>
       <c r="E118" s="5" t="n">
-        <v>1622.15</v>
+        <v>1428.6</v>
       </c>
       <c r="F118" s="16" t="n">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="G118" s="5" t="n">
-        <v>1622.45</v>
+        <v>450</v>
       </c>
     </row>
     <row r="119">
@@ -3580,22 +3580,22 @@
         </is>
       </c>
       <c r="B119" s="8" t="n">
-        <v>7008.15</v>
+        <v>456.55</v>
       </c>
       <c r="C119" s="10" t="n">
-        <v>6918.9</v>
+        <v>449.25</v>
       </c>
       <c r="D119" s="13" t="n">
-        <v>6995</v>
+        <v>7430</v>
       </c>
       <c r="E119" s="5" t="n">
-        <v>6976.3</v>
+        <v>7420</v>
       </c>
       <c r="F119" s="16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G119" s="5" t="n">
-        <v>6961.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="120">
@@ -3605,22 +3605,22 @@
         </is>
       </c>
       <c r="B120" s="8" t="n">
-        <v>2255.05</v>
+        <v>456.55</v>
       </c>
       <c r="C120" s="10" t="n">
-        <v>2225.05</v>
+        <v>449.25</v>
       </c>
       <c r="D120" s="13" t="n">
-        <v>2240.4</v>
+        <v>2264.9</v>
       </c>
       <c r="E120" s="5" t="n">
-        <v>2243.15</v>
+        <v>2262.4</v>
       </c>
       <c r="F120" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G120" s="5" t="n">
-        <v>2247.25</v>
+        <v>450</v>
       </c>
     </row>
     <row r="121">
@@ -3630,22 +3630,22 @@
         </is>
       </c>
       <c r="B121" s="8" t="n">
-        <v>1563.55</v>
+        <v>456.55</v>
       </c>
       <c r="C121" s="10" t="n">
-        <v>1515.1</v>
+        <v>449.25</v>
       </c>
       <c r="D121" s="13" t="n">
-        <v>1560</v>
+        <v>1590.1</v>
       </c>
       <c r="E121" s="5" t="n">
-        <v>1555.5</v>
+        <v>1595.35</v>
       </c>
       <c r="F121" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G121" s="5" t="n">
-        <v>1527.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="122">
@@ -3655,22 +3655,22 @@
         </is>
       </c>
       <c r="B122" s="8" t="n">
-        <v>1872.5</v>
+        <v>456.55</v>
       </c>
       <c r="C122" s="10" t="n">
-        <v>1842.1</v>
+        <v>449.25</v>
       </c>
       <c r="D122" s="13" t="n">
-        <v>1858.1</v>
+        <v>1741.9</v>
       </c>
       <c r="E122" s="5" t="n">
-        <v>1848.9</v>
+        <v>1734.25</v>
       </c>
       <c r="F122" s="16" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G122" s="5" t="n">
-        <v>1865.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="123">
@@ -3680,22 +3680,22 @@
         </is>
       </c>
       <c r="B123" s="8" t="n">
-        <v>863.6</v>
+        <v>456.55</v>
       </c>
       <c r="C123" s="10" t="n">
-        <v>846.45</v>
+        <v>449.25</v>
       </c>
       <c r="D123" s="13" t="n">
-        <v>863.35</v>
+        <v>915</v>
       </c>
       <c r="E123" s="5" t="n">
-        <v>860.25</v>
+        <v>916.9</v>
       </c>
       <c r="F123" s="16" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G123" s="5" t="n">
-        <v>860.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="124">
@@ -3705,22 +3705,22 @@
         </is>
       </c>
       <c r="B124" s="8" t="n">
-        <v>1783.45</v>
+        <v>456.55</v>
       </c>
       <c r="C124" s="10" t="n">
-        <v>1747.15</v>
+        <v>449.25</v>
       </c>
       <c r="D124" s="13" t="n">
-        <v>1773.95</v>
+        <v>1745</v>
       </c>
       <c r="E124" s="5" t="n">
-        <v>1774.65</v>
+        <v>1745.1</v>
       </c>
       <c r="F124" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G124" s="5" t="n">
-        <v>1777.05</v>
+        <v>450</v>
       </c>
     </row>
     <row r="125">
@@ -3730,22 +3730,22 @@
         </is>
       </c>
       <c r="B125" s="8" t="n">
-        <v>839.9</v>
+        <v>456.55</v>
       </c>
       <c r="C125" s="10" t="n">
-        <v>831.85</v>
+        <v>449.25</v>
       </c>
       <c r="D125" s="13" t="n">
-        <v>835.25</v>
+        <v>781.5</v>
       </c>
       <c r="E125" s="5" t="n">
-        <v>834.05</v>
+        <v>779.45</v>
       </c>
       <c r="F125" s="16" t="n">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="G125" s="5" t="n">
-        <v>835.4</v>
+        <v>450</v>
       </c>
     </row>
     <row r="126">
@@ -3755,22 +3755,22 @@
         </is>
       </c>
       <c r="B126" s="8" t="n">
-        <v>4019.95</v>
+        <v>456.55</v>
       </c>
       <c r="C126" s="10" t="n">
-        <v>3960</v>
+        <v>449.25</v>
       </c>
       <c r="D126" s="13" t="n">
-        <v>3975</v>
+        <v>4250.8</v>
       </c>
       <c r="E126" s="5" t="n">
-        <v>3968.45</v>
+        <v>4244.9</v>
       </c>
       <c r="F126" s="16" t="n">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G126" s="5" t="n">
-        <v>4017.7</v>
+        <v>450</v>
       </c>
     </row>
     <row r="127">
@@ -3780,22 +3780,22 @@
         </is>
       </c>
       <c r="B127" s="8" t="n">
-        <v>1645.6</v>
+        <v>456.55</v>
       </c>
       <c r="C127" s="10" t="n">
-        <v>1595.55</v>
+        <v>449.25</v>
       </c>
       <c r="D127" s="13" t="n">
-        <v>1610.15</v>
+        <v>1715</v>
       </c>
       <c r="E127" s="5" t="n">
-        <v>1608.65</v>
+        <v>1713.35</v>
       </c>
       <c r="F127" s="16" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="G127" s="5" t="n">
-        <v>1643.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="128">
@@ -3805,22 +3805,22 @@
         </is>
       </c>
       <c r="B128" s="8" t="n">
-        <v>3286.4</v>
+        <v>456.55</v>
       </c>
       <c r="C128" s="10" t="n">
-        <v>3253.6</v>
+        <v>449.25</v>
       </c>
       <c r="D128" s="13" t="n">
-        <v>3277</v>
+        <v>3224.8</v>
       </c>
       <c r="E128" s="5" t="n">
-        <v>3267.05</v>
+        <v>3212.35</v>
       </c>
       <c r="F128" s="16" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G128" s="5" t="n">
-        <v>3270.8</v>
+        <v>450</v>
       </c>
     </row>
     <row r="129">
@@ -3830,22 +3830,22 @@
         </is>
       </c>
       <c r="B129" s="8" t="n">
-        <v>3229</v>
+        <v>456.55</v>
       </c>
       <c r="C129" s="10" t="n">
-        <v>3158.2</v>
+        <v>449.25</v>
       </c>
       <c r="D129" s="13" t="n">
-        <v>3195</v>
+        <v>3205</v>
       </c>
       <c r="E129" s="5" t="n">
-        <v>3202.65</v>
+        <v>3202.95</v>
       </c>
       <c r="F129" s="16" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G129" s="5" t="n">
-        <v>3191.1</v>
+        <v>450</v>
       </c>
     </row>
     <row r="130">
@@ -3855,22 +3855,22 @@
         </is>
       </c>
       <c r="B130" s="8" t="n">
-        <v>1844</v>
+        <v>456.55</v>
       </c>
       <c r="C130" s="10" t="n">
-        <v>1802</v>
+        <v>449.25</v>
       </c>
       <c r="D130" s="13" t="n">
-        <v>1823.45</v>
+        <v>1515</v>
       </c>
       <c r="E130" s="5" t="n">
-        <v>1821.75</v>
+        <v>1508.1</v>
       </c>
       <c r="F130" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G130" s="5" t="n">
-        <v>1812.15</v>
+        <v>450</v>
       </c>
     </row>
     <row r="131">
@@ -3880,22 +3880,22 @@
         </is>
       </c>
       <c r="B131" s="8" t="n">
-        <v>7199.95</v>
+        <v>456.55</v>
       </c>
       <c r="C131" s="10" t="n">
-        <v>7071</v>
+        <v>449.25</v>
       </c>
       <c r="D131" s="13" t="n">
-        <v>7140</v>
+        <v>6775</v>
       </c>
       <c r="E131" s="5" t="n">
-        <v>7128.35</v>
+        <v>6743.2</v>
       </c>
       <c r="F131" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G131" s="5" t="n">
-        <v>7188.35</v>
+        <v>450</v>
       </c>
     </row>
     <row r="132">
@@ -3905,22 +3905,22 @@
         </is>
       </c>
       <c r="B132" s="8" t="n">
-        <v>2500.7</v>
+        <v>456.55</v>
       </c>
       <c r="C132" s="10" t="n">
-        <v>2448.35</v>
+        <v>449.25</v>
       </c>
       <c r="D132" s="13" t="n">
-        <v>2490</v>
+        <v>2415</v>
       </c>
       <c r="E132" s="5" t="n">
-        <v>2493.7</v>
+        <v>2415.45</v>
       </c>
       <c r="F132" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G132" s="5" t="n">
-        <v>2460.05</v>
+        <v>450</v>
       </c>
     </row>
     <row r="133">
@@ -3930,22 +3930,22 @@
         </is>
       </c>
       <c r="B133" s="8" t="n">
-        <v>1925.65</v>
+        <v>456.55</v>
       </c>
       <c r="C133" s="10" t="n">
-        <v>1901.9</v>
+        <v>449.25</v>
       </c>
       <c r="D133" s="13" t="n">
-        <v>1920.05</v>
+        <v>1930.15</v>
       </c>
       <c r="E133" s="5" t="n">
-        <v>1921.55</v>
+        <v>1933.35</v>
       </c>
       <c r="F133" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G133" s="5" t="n">
-        <v>1918.85</v>
+        <v>450</v>
       </c>
     </row>
     <row r="134">
@@ -3955,22 +3955,22 @@
         </is>
       </c>
       <c r="B134" s="8" t="n">
-        <v>11250.9</v>
+        <v>456.55</v>
       </c>
       <c r="C134" s="10" t="n">
-        <v>11042.55</v>
+        <v>449.25</v>
       </c>
       <c r="D134" s="13" t="n">
-        <v>11076.9</v>
+        <v>11066</v>
       </c>
       <c r="E134" s="5" t="n">
-        <v>11065.65</v>
+        <v>10997.8</v>
       </c>
       <c r="F134" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G134" s="5" t="n">
-        <v>11115.2</v>
+        <v>450</v>
       </c>
     </row>
     <row r="135">
@@ -3980,22 +3980,22 @@
         </is>
       </c>
       <c r="B135" s="8" t="n">
-        <v>555.95</v>
+        <v>456.55</v>
       </c>
       <c r="C135" s="10" t="n">
-        <v>542</v>
+        <v>449.25</v>
       </c>
       <c r="D135" s="13" t="n">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="E135" s="5" t="n">
-        <v>553.65</v>
+        <v>546.9</v>
       </c>
       <c r="F135" s="16" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G135" s="5" t="n">
-        <v>543.9</v>
+        <v>450</v>
       </c>
     </row>
     <row r="136">
@@ -4005,22 +4005,22 @@
         </is>
       </c>
       <c r="B136" s="8" t="n">
-        <v>466.65</v>
+        <v>456.55</v>
       </c>
       <c r="C136" s="10" t="n">
-        <v>460</v>
+        <v>449.25</v>
       </c>
       <c r="D136" s="13" t="n">
-        <v>463.8</v>
+        <v>452.4</v>
       </c>
       <c r="E136" s="5" t="n">
-        <v>464.05</v>
+        <v>451.85</v>
       </c>
       <c r="F136" s="16" t="n">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="G136" s="5" t="n">
-        <v>463.55</v>
+        <v>450</v>
       </c>
     </row>
     <row r="137">
@@ -4030,22 +4030,22 @@
         </is>
       </c>
       <c r="B137" s="8" t="n">
-        <v>1684.85</v>
+        <v>456.55</v>
       </c>
       <c r="C137" s="10" t="n">
-        <v>1617.7</v>
+        <v>449.25</v>
       </c>
       <c r="D137" s="13" t="n">
-        <v>1651.9</v>
+        <v>1645.8</v>
       </c>
       <c r="E137" s="5" t="n">
-        <v>1649.5</v>
+        <v>1647.25</v>
       </c>
       <c r="F137" s="16" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="G137" s="5" t="n">
-        <v>1678</v>
+        <v>450</v>
       </c>
     </row>
     <row r="138">
@@ -4055,22 +4055,22 @@
         </is>
       </c>
       <c r="B138" s="8" t="n">
-        <v>123</v>
+        <v>456.55</v>
       </c>
       <c r="C138" s="10" t="n">
-        <v>120.85</v>
+        <v>449.25</v>
       </c>
       <c r="D138" s="13" t="n">
-        <v>122.26</v>
+        <v>123.22</v>
       </c>
       <c r="E138" s="5" t="n">
-        <v>122.15</v>
+        <v>123.11</v>
       </c>
       <c r="F138" s="16" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="G138" s="5" t="n">
-        <v>122.41</v>
+        <v>450</v>
       </c>
     </row>
     <row r="139" ht="15.75" customHeight="1" thickBot="1">
@@ -4080,22 +4080,22 @@
         </is>
       </c>
       <c r="B139" s="18" t="n">
-        <v>1004.45</v>
+        <v>456.55</v>
       </c>
       <c r="C139" s="11" t="n">
-        <v>989</v>
+        <v>449.25</v>
       </c>
       <c r="D139" s="14" t="n">
-        <v>1003.9</v>
+        <v>951.85</v>
       </c>
       <c r="E139" s="6" t="n">
-        <v>1001.25</v>
+        <v>948.7</v>
       </c>
       <c r="F139" s="17" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G139" s="6" t="n">
-        <v>993.35</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added chambal, modifed how md file outputs
</commit_message>
<xml_diff>
--- a/algo high low.xlsx
+++ b/algo high low.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="144525" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -655,22 +655,22 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>451.95</v>
+        <v>3124.95</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>445.2</v>
+        <v>3054.05</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>447.05</v>
+        <v>448.8</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>448.3</v>
+        <v>448.4</v>
       </c>
       <c r="F2" s="15" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>449.55</v>
+        <v>3093.45</v>
       </c>
     </row>
     <row r="3">
@@ -680,22 +680,22 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>7471.95</v>
+        <v>2000.15</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>7375</v>
+        <v>1954.1</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>7403</v>
+        <v>7587.95</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>7421.25</v>
+        <v>7569.75</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>7415.05</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="4">
@@ -705,22 +705,22 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>196.3</v>
+        <v>743</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>192.68</v>
+        <v>708.35</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>194.4</v>
+        <v>196.82</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>194.33</v>
+        <v>196.83</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>194.38</v>
+        <v>708.35</v>
       </c>
     </row>
     <row r="5">
@@ -730,22 +730,22 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>316</v>
+        <v>8531.9</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>311.25</v>
+        <v>8401</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>313.4</v>
+        <v>308.45</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>313.75</v>
+        <v>308.3</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>314.35</v>
+        <v>8499.700000000001</v>
       </c>
     </row>
     <row r="6">
@@ -755,22 +755,22 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>2520</v>
+        <v>3579.95</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>2400</v>
+        <v>3524.75</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>2457</v>
+        <v>2494.8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2463.15</v>
+        <v>2495.85</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>81</v>
+        <v>9</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2470.9</v>
+        <v>3547.25</v>
       </c>
     </row>
     <row r="7">
@@ -780,22 +780,22 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1215.6</v>
+        <v>242.34</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>1168.9</v>
+        <v>235.72</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>1187.5</v>
+        <v>1266.35</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1190.05</v>
+        <v>1266.85</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1184</v>
+        <v>238.99</v>
       </c>
     </row>
     <row r="8">
@@ -805,22 +805,22 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>5650</v>
+        <v>372.15</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>5519.8</v>
+        <v>367.75</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>5635.75</v>
+        <v>5495</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>5642.45</v>
+        <v>5484.6</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>5529.95</v>
+        <v>370.9</v>
       </c>
     </row>
     <row r="9">
@@ -830,22 +830,22 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>535.7</v>
+        <v>2177.35</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>518.25</v>
+        <v>2132.6</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>534</v>
+        <v>570</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>531.5</v>
+        <v>571.3</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>520.1</v>
+        <v>2153.95</v>
       </c>
     </row>
     <row r="10">
@@ -855,22 +855,22 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>6869.7</v>
+        <v>260</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>6812</v>
+        <v>257.7</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>6849</v>
+        <v>7203</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>6828.9</v>
+        <v>7193.85</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>6854.05</v>
+        <v>259.65</v>
       </c>
     </row>
     <row r="11">
@@ -880,22 +880,22 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>511.85</v>
+        <v>1250</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>504.4</v>
+        <v>1233.75</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>509.25</v>
+        <v>547.35</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>509.65</v>
+        <v>549.1</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>506.75</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="12">
@@ -905,22 +905,22 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>232.48</v>
+        <v>6272.45</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>229.21</v>
+        <v>6184.95</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>231.7</v>
+        <v>228.9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>232.08</v>
+        <v>228.66</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>229.58</v>
+        <v>6249.95</v>
       </c>
     </row>
     <row r="13">
@@ -930,22 +930,22 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>1807.9</v>
+        <v>338.45</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>1782.2</v>
+        <v>333.8</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>1789.65</v>
+        <v>1849</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1790.5</v>
+        <v>1850.55</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>1798.4</v>
+        <v>335.3</v>
       </c>
     </row>
     <row r="14">
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>7318.05</v>
+        <v>3168.65</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>7242.05</v>
+        <v>3120</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>7315.05</v>
+        <v>7296.35</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>7295.8</v>
+        <v>7285.1</v>
       </c>
       <c r="F14" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>7280.1</v>
+        <v>3143</v>
       </c>
     </row>
     <row r="15">
@@ -980,22 +980,22 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>591.65</v>
+        <v>7451</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>578.4</v>
+        <v>7361.05</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>584.5</v>
+        <v>581</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>583.35</v>
+        <v>581.2</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>590.85</v>
+        <v>7373.4</v>
       </c>
     </row>
     <row r="16">
@@ -1005,22 +1005,22 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>1269.15</v>
+        <v>330.65</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>1245.05</v>
+        <v>327.7</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1258.2</v>
+        <v>1240.1</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1262.6</v>
+        <v>1239.5</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>1256</v>
+        <v>329.8</v>
       </c>
     </row>
     <row r="17">
@@ -1030,22 +1030,22 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>9090.9</v>
+        <v>188.3</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>9005.299999999999</v>
+        <v>180.05</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>9029.799999999999</v>
+        <v>9072.950000000001</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>9033.65</v>
+        <v>9077.450000000001</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9033.450000000001</v>
+        <v>183.6</v>
       </c>
     </row>
     <row r="18">
@@ -1055,22 +1055,22 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>1587.95</v>
+        <v>1016.75</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>1574.95</v>
+        <v>1005.25</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1580</v>
+        <v>1637.1</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>1579.95</v>
+        <v>1637.05</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>1579</v>
+        <v>1009.1</v>
       </c>
     </row>
     <row r="19">
@@ -1080,22 +1080,22 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>6609</v>
+        <v>180</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>6510.35</v>
+        <v>170.6</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>6565</v>
+        <v>6878.95</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>6575.9</v>
+        <v>6868.35</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>6524.1</v>
+        <v>176.8</v>
       </c>
     </row>
     <row r="20">
@@ -1105,22 +1105,22 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>2794.95</v>
+        <v>568</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>2716.95</v>
+        <v>561</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>2780</v>
+        <v>2860</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>2780.15</v>
+        <v>2857.8</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>2717.95</v>
+        <v>564.1</v>
       </c>
     </row>
     <row r="21">
@@ -1130,22 +1130,22 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>588</v>
+        <v>724.9</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>560.75</v>
+        <v>718.55</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>586</v>
+        <v>575</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>585.1</v>
+        <v>575.85</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>562.25</v>
+        <v>720.65</v>
       </c>
     </row>
     <row r="22">
@@ -1155,22 +1155,22 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>171.58</v>
+        <v>1484.4</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>167.12</v>
+        <v>1459.15</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>168.94</v>
+        <v>174.6</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>169.08</v>
+        <v>174.55</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>171.1</v>
+        <v>1462.85</v>
       </c>
     </row>
     <row r="23">
@@ -1180,22 +1180,22 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>250.45</v>
+        <v>7937.35</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>244.25</v>
+        <v>7766.75</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>246.3</v>
+        <v>262.9</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>246.4</v>
+        <v>262.93</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>249.85</v>
+        <v>7795</v>
       </c>
     </row>
     <row r="24">
@@ -1205,22 +1205,22 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>1418.15</v>
+        <v>2318.15</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>1369.6</v>
+        <v>2257.8</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>1409.8</v>
+        <v>1445.1</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1410.85</v>
+        <v>1448.25</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>1371.5</v>
+        <v>2278.5</v>
       </c>
     </row>
     <row r="25">
@@ -1230,22 +1230,22 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>310.6</v>
+        <v>200.2</v>
       </c>
       <c r="C25" s="10" t="n">
-        <v>306.2</v>
+        <v>197.26</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>307.65</v>
+        <v>314.45</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>308</v>
+        <v>314.6</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>232</v>
+        <v>118</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>308.85</v>
+        <v>199.71</v>
       </c>
     </row>
     <row r="26">
@@ -1255,22 +1255,22 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>1345.85</v>
+        <v>1815</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>1325.95</v>
+        <v>1796.7</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>1330</v>
+        <v>1362.5</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>1332.25</v>
+        <v>1363.45</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>1335.65</v>
+        <v>1810.95</v>
       </c>
     </row>
     <row r="27">
@@ -1280,22 +1280,22 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>253.79</v>
+        <v>896</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>247.41</v>
+        <v>864.65</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>251</v>
+        <v>249.3</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>251.09</v>
+        <v>249.55</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>253.15</v>
+        <v>888.15</v>
       </c>
     </row>
     <row r="28">
@@ -1305,22 +1305,22 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>368.3</v>
+        <v>1803.5</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>362</v>
+        <v>1780</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>364.75</v>
+        <v>369</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>365.15</v>
+        <v>369.6</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>367.05</v>
+        <v>1794.55</v>
       </c>
     </row>
     <row r="29">
@@ -1330,22 +1330,22 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>4955.95</v>
+        <v>819.2</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>4905.7</v>
+        <v>797</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>4939</v>
+        <v>4798</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>4941.15</v>
+        <v>4793</v>
       </c>
       <c r="F29" s="16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>4905.7</v>
+        <v>818.75</v>
       </c>
     </row>
     <row r="30">
@@ -1355,22 +1355,22 @@
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>595.35</v>
+        <v>4469.4</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>587.7</v>
+        <v>4415.55</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>591.7</v>
+        <v>608.9</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>590.65</v>
+        <v>608.65</v>
       </c>
       <c r="F30" s="16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>588.65</v>
+        <v>4461.2</v>
       </c>
     </row>
     <row r="31">
@@ -1380,22 +1380,22 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>103.68</v>
+        <v>1800.75</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>100.75</v>
+        <v>1771.2</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>101.99</v>
+        <v>109</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>102.01</v>
+        <v>108.99</v>
       </c>
       <c r="F31" s="16" t="n">
-        <v>212</v>
+        <v>171</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>103.31</v>
+        <v>1798.9</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -1405,22 +1405,22 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>826.1</v>
+        <v>3488.25</v>
       </c>
       <c r="C32" s="10" t="n">
-        <v>817.6</v>
+        <v>3448.5</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>823.2</v>
+        <v>805.3</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>823.95</v>
+        <v>804.5</v>
       </c>
       <c r="F32" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>824.8</v>
+        <v>3476.8</v>
       </c>
     </row>
     <row r="33">
@@ -1430,22 +1430,22 @@
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>516.55</v>
+        <v>3369.5</v>
       </c>
       <c r="C33" s="10" t="n">
-        <v>497.75</v>
+        <v>3319.45</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>515.9</v>
+        <v>527</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>515.3</v>
+        <v>528.15</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>497.9</v>
+        <v>3342.35</v>
       </c>
     </row>
     <row r="34">
@@ -1455,22 +1455,22 @@
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>1259.1</v>
+        <v>1667.05</v>
       </c>
       <c r="C34" s="10" t="n">
-        <v>1229.05</v>
+        <v>1628.85</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>1235</v>
+        <v>1280.05</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>1233.95</v>
+        <v>1282.25</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>1255.1</v>
+        <v>1661.2</v>
       </c>
     </row>
     <row r="35">
@@ -1480,22 +1480,22 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>1547.7</v>
+        <v>7025</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>1513.05</v>
+        <v>6867.3</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>1532</v>
+        <v>1471.95</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>1533.9</v>
+        <v>1469</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>1517.55</v>
+        <v>7013.2</v>
       </c>
     </row>
     <row r="36">
@@ -1505,22 +1505,22 @@
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>8707.9</v>
+        <v>2532</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>8541</v>
+        <v>2481.05</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>8680.049999999999</v>
+        <v>8916.950000000001</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>8685.85</v>
+        <v>8918.6</v>
       </c>
       <c r="F36" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>8554.15</v>
+        <v>2531.9</v>
       </c>
     </row>
     <row r="37">
@@ -1530,22 +1530,22 @@
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>830.95</v>
+        <v>1968.8</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>821.25</v>
+        <v>1948.05</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>825.25</v>
+        <v>860.55</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>828.35</v>
+        <v>858.1</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>823.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1555,22 +1555,22 @@
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>1800.2</v>
+        <v>11861</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>1758.05</v>
+        <v>11718</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>1783.75</v>
+        <v>1762.05</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>1789</v>
+        <v>1769.8</v>
       </c>
       <c r="F38" s="16" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>1762.55</v>
+        <v>11770.75</v>
       </c>
     </row>
     <row r="39">
@@ -1580,22 +1580,22 @@
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>410.8</v>
+        <v>561.75</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>402.05</v>
+        <v>552.05</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>410.8</v>
+        <v>414.25</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>409.7</v>
+        <v>414.1</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>406.45</v>
+        <v>558.7</v>
       </c>
     </row>
     <row r="40">
@@ -1605,22 +1605,22 @@
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>3514</v>
+        <v>499.6</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>3460</v>
+        <v>488.8</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>3477.9</v>
+        <v>3501</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>3483.7</v>
+        <v>3509.15</v>
       </c>
       <c r="F40" s="16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>3483.1</v>
+        <v>497.25</v>
       </c>
     </row>
     <row r="41">
@@ -1630,22 +1630,22 @@
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>529.65</v>
+        <v>1767</v>
       </c>
       <c r="C41" s="10" t="n">
-        <v>522.5</v>
+        <v>1743.65</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>526.6</v>
+        <v>507</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>527.15</v>
+        <v>506.85</v>
       </c>
       <c r="F41" s="16" t="n">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>523</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="42">
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>1836.45</v>
+        <v>143.06</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>1812.5</v>
+        <v>140.6</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>1817.2</v>
+        <v>1897.45</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>1820.35</v>
+        <v>1897.75</v>
       </c>
       <c r="F42" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>1831.95</v>
+        <v>142.36</v>
       </c>
     </row>
     <row r="43">
@@ -1680,22 +1680,22 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>1387</v>
+        <v>998.8</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>1326.25</v>
+        <v>981</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>1370</v>
+        <v>1383</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>1374.95</v>
+        <v>1381.55</v>
       </c>
       <c r="F43" s="16" t="n">
         <v>9</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>1344.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="44">
@@ -1705,22 +1705,22 @@
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>2739</v>
+        <v>998.8</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>2710</v>
+        <v>981</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>2725.4</v>
+        <v>2682.5</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>2727.25</v>
+        <v>2674.3</v>
       </c>
       <c r="F44" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>2719.3</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="45">
@@ -1730,22 +1730,22 @@
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>119.25</v>
+        <v>998.8</v>
       </c>
       <c r="C45" s="10" t="n">
-        <v>116.83</v>
+        <v>981</v>
       </c>
       <c r="D45" s="13" t="n">
-        <v>117.6</v>
+        <v>123.9</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>117.56</v>
+        <v>124.2</v>
       </c>
       <c r="F45" s="16" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>117.86</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="46">
@@ -1755,22 +1755,22 @@
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>6208.3</v>
+        <v>998.8</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>6011.15</v>
+        <v>981</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>6183.25</v>
+        <v>5951.85</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>6172.7</v>
+        <v>5959.65</v>
       </c>
       <c r="F46" s="16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>6031.15</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="47">
@@ -1780,22 +1780,22 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>15987.95</v>
+        <v>998.8</v>
       </c>
       <c r="C47" s="10" t="n">
-        <v>15718.55</v>
+        <v>981</v>
       </c>
       <c r="D47" s="13" t="n">
-        <v>15813.1</v>
+        <v>17369</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>15807.4</v>
+        <v>17345.9</v>
       </c>
       <c r="F47" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>15813.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="48">
@@ -1805,22 +1805,22 @@
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>828.65</v>
+        <v>998.8</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>813.05</v>
+        <v>981</v>
       </c>
       <c r="D48" s="13" t="n">
-        <v>822</v>
+        <v>863</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>822.95</v>
+        <v>862.7</v>
       </c>
       <c r="F48" s="16" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>814.35</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="49">
@@ -1830,22 +1830,22 @@
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>1214.35</v>
+        <v>998.8</v>
       </c>
       <c r="C49" s="10" t="n">
-        <v>1199.25</v>
+        <v>981</v>
       </c>
       <c r="D49" s="13" t="n">
-        <v>1202.45</v>
+        <v>1255.5</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>1202.3</v>
+        <v>1255.15</v>
       </c>
       <c r="F49" s="16" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>1205.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="50">
@@ -1855,22 +1855,22 @@
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>3568.55</v>
+        <v>998.8</v>
       </c>
       <c r="C50" s="10" t="n">
-        <v>3515</v>
+        <v>981</v>
       </c>
       <c r="D50" s="13" t="n">
-        <v>3555</v>
+        <v>3538</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>3553.9</v>
+        <v>3546.4</v>
       </c>
       <c r="F50" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>3521</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="51">
@@ -1880,22 +1880,22 @@
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>459.55</v>
+        <v>998.8</v>
       </c>
       <c r="C51" s="10" t="n">
-        <v>446.5</v>
+        <v>981</v>
       </c>
       <c r="D51" s="13" t="n">
-        <v>451.1</v>
+        <v>467</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>452.6</v>
+        <v>467</v>
       </c>
       <c r="F51" s="16" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>450.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="52">
@@ -1905,22 +1905,22 @@
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>1531.5</v>
+        <v>998.8</v>
       </c>
       <c r="C52" s="10" t="n">
-        <v>1499.1</v>
+        <v>981</v>
       </c>
       <c r="D52" s="13" t="n">
-        <v>1528.1</v>
+        <v>1520.05</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>1528.65</v>
+        <v>1514.15</v>
       </c>
       <c r="F52" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>1509.95</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="53">
@@ -1930,22 +1930,22 @@
         </is>
       </c>
       <c r="B53" s="8" t="n">
-        <v>1093.85</v>
+        <v>998.8</v>
       </c>
       <c r="C53" s="10" t="n">
-        <v>1068.2</v>
+        <v>981</v>
       </c>
       <c r="D53" s="13" t="n">
-        <v>1083.7</v>
+        <v>1030.05</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>1084.1</v>
+        <v>1029.75</v>
       </c>
       <c r="F53" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>1080</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="54">
@@ -1955,22 +1955,22 @@
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>640.85</v>
+        <v>998.8</v>
       </c>
       <c r="C54" s="10" t="n">
-        <v>614.5</v>
+        <v>981</v>
       </c>
       <c r="D54" s="13" t="n">
-        <v>636.1</v>
+        <v>623.45</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>638.8</v>
+        <v>622.4</v>
       </c>
       <c r="F54" s="16" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>620.2</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="55">
@@ -1980,22 +1980,22 @@
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>1250.95</v>
+        <v>998.8</v>
       </c>
       <c r="C55" s="10" t="n">
-        <v>1236</v>
+        <v>981</v>
       </c>
       <c r="D55" s="13" t="n">
-        <v>1245</v>
+        <v>1126.5</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1244.65</v>
+        <v>1127.85</v>
       </c>
       <c r="F55" s="16" t="n">
-        <v>6</v>
+        <v>112</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>1244.2</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="56">
@@ -2005,22 +2005,22 @@
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>2813</v>
+        <v>998.8</v>
       </c>
       <c r="C56" s="10" t="n">
-        <v>2767.6</v>
+        <v>981</v>
       </c>
       <c r="D56" s="13" t="n">
-        <v>2778.95</v>
+        <v>2833.45</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>2776.15</v>
+        <v>2842.95</v>
       </c>
       <c r="F56" s="16" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>2777.4</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="57">
@@ -2030,22 +2030,22 @@
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>588.8</v>
+        <v>998.8</v>
       </c>
       <c r="C57" s="10" t="n">
-        <v>578.9</v>
+        <v>981</v>
       </c>
       <c r="D57" s="13" t="n">
-        <v>583</v>
+        <v>579.1</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>584.3</v>
+        <v>580.1</v>
       </c>
       <c r="F57" s="16" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>586.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="58">
@@ -2055,22 +2055,22 @@
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>2630.45</v>
+        <v>998.8</v>
       </c>
       <c r="C58" s="10" t="n">
-        <v>2576.55</v>
+        <v>981</v>
       </c>
       <c r="D58" s="13" t="n">
-        <v>2603.05</v>
+        <v>2680.55</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>2606.25</v>
+        <v>2681.4</v>
       </c>
       <c r="F58" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>2584.2</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="59">
@@ -2080,22 +2080,22 @@
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>481</v>
+        <v>998.8</v>
       </c>
       <c r="C59" s="10" t="n">
-        <v>472.05</v>
+        <v>981</v>
       </c>
       <c r="D59" s="13" t="n">
-        <v>480.4</v>
+        <v>509</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>479.75</v>
+        <v>508.15</v>
       </c>
       <c r="F59" s="16" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>474.25</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="60">
@@ -2105,22 +2105,22 @@
         </is>
       </c>
       <c r="B60" s="8" t="n">
-        <v>4499</v>
+        <v>998.8</v>
       </c>
       <c r="C60" s="10" t="n">
-        <v>4420.7</v>
+        <v>981</v>
       </c>
       <c r="D60" s="13" t="n">
-        <v>4470</v>
+        <v>4620</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>4476.85</v>
+        <v>4618.95</v>
       </c>
       <c r="F60" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>4475</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="61">
@@ -2130,22 +2130,22 @@
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>1727.95</v>
+        <v>998.8</v>
       </c>
       <c r="C61" s="10" t="n">
-        <v>1702.2</v>
+        <v>981</v>
       </c>
       <c r="D61" s="13" t="n">
-        <v>1721.45</v>
+        <v>1703.5</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>1718</v>
+        <v>1704.7</v>
       </c>
       <c r="F61" s="16" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>1704.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="62">
@@ -2155,22 +2155,22 @@
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>1872.3</v>
+        <v>998.8</v>
       </c>
       <c r="C62" s="10" t="n">
-        <v>1844.15</v>
+        <v>981</v>
       </c>
       <c r="D62" s="13" t="n">
-        <v>1850</v>
+        <v>1909.95</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>1848.05</v>
+        <v>1909.9</v>
       </c>
       <c r="F62" s="16" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>1845.05</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="63">
@@ -2180,22 +2180,22 @@
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>4235.75</v>
+        <v>998.8</v>
       </c>
       <c r="C63" s="10" t="n">
-        <v>4188</v>
+        <v>981</v>
       </c>
       <c r="D63" s="13" t="n">
-        <v>4209.25</v>
+        <v>4459.75</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>4204.25</v>
+        <v>4469.15</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4214.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="64">
@@ -2205,22 +2205,22 @@
         </is>
       </c>
       <c r="B64" s="8" t="n">
-        <v>666</v>
+        <v>998.8</v>
       </c>
       <c r="C64" s="10" t="n">
-        <v>651.3</v>
+        <v>981</v>
       </c>
       <c r="D64" s="13" t="n">
-        <v>656</v>
+        <v>641.7</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>657.75</v>
+        <v>641.8</v>
       </c>
       <c r="F64" s="16" t="n">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>664.35</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="65">
@@ -2230,22 +2230,22 @@
         </is>
       </c>
       <c r="B65" s="8" t="n">
-        <v>658.6</v>
+        <v>998.8</v>
       </c>
       <c r="C65" s="10" t="n">
-        <v>649.1</v>
+        <v>981</v>
       </c>
       <c r="D65" s="13" t="n">
-        <v>657</v>
+        <v>670.3</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>656.2</v>
+        <v>670.9</v>
       </c>
       <c r="F65" s="16" t="n">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>650.45</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="66">
@@ -2255,22 +2255,22 @@
         </is>
       </c>
       <c r="B66" s="8" t="n">
-        <v>278.45</v>
+        <v>998.8</v>
       </c>
       <c r="C66" s="10" t="n">
-        <v>271.7</v>
+        <v>981</v>
       </c>
       <c r="D66" s="13" t="n">
-        <v>275.4</v>
+        <v>290.1</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>276</v>
+        <v>292.5</v>
       </c>
       <c r="F66" s="16" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>273.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="67">
@@ -2280,22 +2280,22 @@
         </is>
       </c>
       <c r="B67" s="8" t="n">
-        <v>1888.55</v>
+        <v>998.8</v>
       </c>
       <c r="C67" s="10" t="n">
-        <v>1846.05</v>
+        <v>981</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>1860.1</v>
+        <v>1963</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1861.85</v>
+        <v>1962.2</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>1886.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="68">
@@ -2305,22 +2305,22 @@
         </is>
       </c>
       <c r="B68" s="8" t="n">
-        <v>701.1</v>
+        <v>998.8</v>
       </c>
       <c r="C68" s="10" t="n">
-        <v>687.6</v>
+        <v>981</v>
       </c>
       <c r="D68" s="13" t="n">
-        <v>698.6</v>
+        <v>676.55</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>699.65</v>
+        <v>676.2</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>699</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="69">
@@ -2330,22 +2330,22 @@
         </is>
       </c>
       <c r="B69" s="8" t="n">
-        <v>177.91</v>
+        <v>998.8</v>
       </c>
       <c r="C69" s="10" t="n">
-        <v>173.29</v>
+        <v>981</v>
       </c>
       <c r="D69" s="13" t="n">
-        <v>176.1</v>
+        <v>184.4</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>176.19</v>
+        <v>184.13</v>
       </c>
       <c r="F69" s="16" t="n">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>175.2</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="70">
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="B70" s="8" t="n">
-        <v>331.65</v>
+        <v>998.8</v>
       </c>
       <c r="C70" s="10" t="n">
-        <v>313.45</v>
+        <v>981</v>
       </c>
       <c r="D70" s="13" t="n">
-        <v>330</v>
+        <v>386.65</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>327.05</v>
+        <v>385.55</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>319.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="71">
@@ -2380,22 +2380,22 @@
         </is>
       </c>
       <c r="B71" s="8" t="n">
-        <v>801.7</v>
+        <v>998.8</v>
       </c>
       <c r="C71" s="10" t="n">
-        <v>780</v>
+        <v>981</v>
       </c>
       <c r="D71" s="13" t="n">
-        <v>794.45</v>
+        <v>835.25</v>
       </c>
       <c r="E71" s="5" t="n">
-        <v>793.35</v>
+        <v>837.2</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>780.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="72">
@@ -2405,22 +2405,22 @@
         </is>
       </c>
       <c r="B72" s="8" t="n">
-        <v>366.9</v>
+        <v>998.8</v>
       </c>
       <c r="C72" s="10" t="n">
-        <v>360.5</v>
+        <v>981</v>
       </c>
       <c r="D72" s="13" t="n">
-        <v>366.9</v>
+        <v>345.4</v>
       </c>
       <c r="E72" s="5" t="n">
-        <v>365.8</v>
+        <v>345.75</v>
       </c>
       <c r="F72" s="16" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>362.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="73">
@@ -2430,22 +2430,22 @@
         </is>
       </c>
       <c r="B73" s="8" t="n">
-        <v>2355</v>
+        <v>998.8</v>
       </c>
       <c r="C73" s="10" t="n">
-        <v>2323.05</v>
+        <v>981</v>
       </c>
       <c r="D73" s="13" t="n">
-        <v>2347</v>
+        <v>2370</v>
       </c>
       <c r="E73" s="5" t="n">
-        <v>2344.9</v>
+        <v>2371.15</v>
       </c>
       <c r="F73" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>2337.05</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="74">
@@ -2455,22 +2455,22 @@
         </is>
       </c>
       <c r="B74" s="8" t="n">
-        <v>4400</v>
+        <v>998.8</v>
       </c>
       <c r="C74" s="10" t="n">
-        <v>4326.3</v>
+        <v>981</v>
       </c>
       <c r="D74" s="13" t="n">
-        <v>4380</v>
+        <v>4487.85</v>
       </c>
       <c r="E74" s="5" t="n">
-        <v>4378.9</v>
+        <v>4489.45</v>
       </c>
       <c r="F74" s="16" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>4332.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="75">
@@ -2480,22 +2480,22 @@
         </is>
       </c>
       <c r="B75" s="8" t="n">
-        <v>999.5</v>
+        <v>998.8</v>
       </c>
       <c r="C75" s="10" t="n">
-        <v>987.3</v>
+        <v>981</v>
       </c>
       <c r="D75" s="13" t="n">
-        <v>994.45</v>
+        <v>982.75</v>
       </c>
       <c r="E75" s="5" t="n">
-        <v>995.85</v>
+        <v>982.6</v>
       </c>
       <c r="F75" s="16" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>994.25</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="76">
@@ -2505,22 +2505,22 @@
         </is>
       </c>
       <c r="B76" s="8" t="n">
-        <v>352.5</v>
+        <v>998.8</v>
       </c>
       <c r="C76" s="10" t="n">
-        <v>345.5</v>
+        <v>981</v>
       </c>
       <c r="D76" s="13" t="n">
-        <v>349.25</v>
+        <v>361.75</v>
       </c>
       <c r="E76" s="5" t="n">
-        <v>349.35</v>
+        <v>362.15</v>
       </c>
       <c r="F76" s="16" t="n">
-        <v>46</v>
+        <v>143</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>350.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="77">
@@ -2530,22 +2530,22 @@
         </is>
       </c>
       <c r="B77" s="8" t="n">
-        <v>721</v>
+        <v>998.8</v>
       </c>
       <c r="C77" s="10" t="n">
-        <v>693</v>
+        <v>981</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>715.45</v>
+        <v>793</v>
       </c>
       <c r="E77" s="5" t="n">
-        <v>717</v>
+        <v>793.15</v>
       </c>
       <c r="F77" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>708.75</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="78">
@@ -2555,22 +2555,22 @@
         </is>
       </c>
       <c r="B78" s="8" t="n">
-        <v>1545.25</v>
+        <v>998.8</v>
       </c>
       <c r="C78" s="10" t="n">
-        <v>1520.05</v>
+        <v>981</v>
       </c>
       <c r="D78" s="13" t="n">
-        <v>1544.45</v>
+        <v>1524.65</v>
       </c>
       <c r="E78" s="5" t="n">
-        <v>1542.55</v>
+        <v>1523.75</v>
       </c>
       <c r="F78" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>1523.2</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="79">
@@ -2580,22 +2580,22 @@
         </is>
       </c>
       <c r="B79" s="8" t="n">
-        <v>912.5</v>
+        <v>998.8</v>
       </c>
       <c r="C79" s="10" t="n">
-        <v>892</v>
+        <v>981</v>
       </c>
       <c r="D79" s="13" t="n">
-        <v>907</v>
+        <v>968</v>
       </c>
       <c r="E79" s="5" t="n">
-        <v>906.45</v>
+        <v>967.2</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>895.25</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="80">
@@ -2605,22 +2605,22 @@
         </is>
       </c>
       <c r="B80" s="8" t="n">
-        <v>4300.2</v>
+        <v>998.8</v>
       </c>
       <c r="C80" s="10" t="n">
-        <v>4145.05</v>
+        <v>981</v>
       </c>
       <c r="D80" s="13" t="n">
-        <v>4255.05</v>
+        <v>4570</v>
       </c>
       <c r="E80" s="5" t="n">
-        <v>4278.25</v>
+        <v>4562.95</v>
       </c>
       <c r="F80" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>4160.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="81">
@@ -2630,22 +2630,22 @@
         </is>
       </c>
       <c r="B81" s="8" t="n">
-        <v>971.7</v>
+        <v>998.8</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>956.15</v>
+        <v>981</v>
       </c>
       <c r="D81" s="13" t="n">
-        <v>965.2</v>
+        <v>1012</v>
       </c>
       <c r="E81" s="5" t="n">
-        <v>966</v>
+        <v>1011.9</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>957.35</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="82">
@@ -2655,22 +2655,22 @@
         </is>
       </c>
       <c r="B82" s="8" t="n">
-        <v>650.65</v>
+        <v>998.8</v>
       </c>
       <c r="C82" s="10" t="n">
-        <v>639.6</v>
+        <v>981</v>
       </c>
       <c r="D82" s="13" t="n">
-        <v>643.15</v>
+        <v>695</v>
       </c>
       <c r="E82" s="5" t="n">
-        <v>644.55</v>
+        <v>694.7</v>
       </c>
       <c r="F82" s="16" t="n">
         <v>13</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>640.2</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="83">
@@ -2680,22 +2680,22 @@
         </is>
       </c>
       <c r="B83" s="8" t="n">
-        <v>1773.6</v>
+        <v>998.8</v>
       </c>
       <c r="C83" s="10" t="n">
-        <v>1758.8</v>
+        <v>981</v>
       </c>
       <c r="D83" s="13" t="n">
-        <v>1761.25</v>
+        <v>1786.95</v>
       </c>
       <c r="E83" s="5" t="n">
-        <v>1765.25</v>
+        <v>1786.25</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>1768.15</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="84">
@@ -2705,22 +2705,22 @@
         </is>
       </c>
       <c r="B84" s="8" t="n">
-        <v>3014</v>
+        <v>998.8</v>
       </c>
       <c r="C84" s="10" t="n">
-        <v>2981</v>
+        <v>981</v>
       </c>
       <c r="D84" s="13" t="n">
-        <v>3002.5</v>
+        <v>3146.9</v>
       </c>
       <c r="E84" s="5" t="n">
-        <v>3002.9</v>
+        <v>3136.8</v>
       </c>
       <c r="F84" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G84" s="4" t="n">
-        <v>2993.75</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="85">
@@ -2730,22 +2730,22 @@
         </is>
       </c>
       <c r="B85" s="8" t="n">
-        <v>570</v>
+        <v>998.8</v>
       </c>
       <c r="C85" s="10" t="n">
-        <v>558.55</v>
+        <v>981</v>
       </c>
       <c r="D85" s="13" t="n">
-        <v>568</v>
+        <v>570.6</v>
       </c>
       <c r="E85" s="5" t="n">
-        <v>567.15</v>
+        <v>571.9</v>
       </c>
       <c r="F85" s="16" t="n">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="G85" s="4" t="n">
-        <v>562.3</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="86">
@@ -2755,22 +2755,22 @@
         </is>
       </c>
       <c r="B86" s="8" t="n">
-        <v>639.95</v>
+        <v>998.8</v>
       </c>
       <c r="C86" s="10" t="n">
-        <v>630.95</v>
+        <v>981</v>
       </c>
       <c r="D86" s="13" t="n">
-        <v>637.3</v>
+        <v>630.45</v>
       </c>
       <c r="E86" s="5" t="n">
-        <v>638.8</v>
+        <v>630.15</v>
       </c>
       <c r="F86" s="16" t="n">
         <v>8</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>636.45</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="87">
@@ -2780,22 +2780,22 @@
         </is>
       </c>
       <c r="B87" s="8" t="n">
-        <v>6250</v>
+        <v>998.8</v>
       </c>
       <c r="C87" s="10" t="n">
-        <v>6141.25</v>
+        <v>981</v>
       </c>
       <c r="D87" s="13" t="n">
-        <v>6170.2</v>
+        <v>6396.4</v>
       </c>
       <c r="E87" s="5" t="n">
-        <v>6172.4</v>
+        <v>6389.05</v>
       </c>
       <c r="F87" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G87" s="4" t="n">
-        <v>6146.25</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="88">
@@ -2805,22 +2805,22 @@
         </is>
       </c>
       <c r="B88" s="8" t="n">
-        <v>5325</v>
+        <v>998.8</v>
       </c>
       <c r="C88" s="10" t="n">
-        <v>5254.3</v>
+        <v>981</v>
       </c>
       <c r="D88" s="13" t="n">
-        <v>5280</v>
+        <v>5356</v>
       </c>
       <c r="E88" s="5" t="n">
-        <v>5285.2</v>
+        <v>5348.9</v>
       </c>
       <c r="F88" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>5264.3</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="89">
@@ -2830,22 +2830,22 @@
         </is>
       </c>
       <c r="B89" s="8" t="n">
-        <v>2059.55</v>
+        <v>998.8</v>
       </c>
       <c r="C89" s="10" t="n">
-        <v>2013.05</v>
+        <v>981</v>
       </c>
       <c r="D89" s="13" t="n">
-        <v>2052</v>
+        <v>2110</v>
       </c>
       <c r="E89" s="5" t="n">
-        <v>2050.75</v>
+        <v>2104.7</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>2016.45</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="90">
@@ -2855,22 +2855,22 @@
         </is>
       </c>
       <c r="B90" s="8" t="n">
-        <v>274.85</v>
+        <v>998.8</v>
       </c>
       <c r="C90" s="10" t="n">
-        <v>269.35</v>
+        <v>981</v>
       </c>
       <c r="D90" s="13" t="n">
-        <v>273.85</v>
+        <v>279.5</v>
       </c>
       <c r="E90" s="5" t="n">
-        <v>273.4</v>
+        <v>279.15</v>
       </c>
       <c r="F90" s="16" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>271.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="91">
@@ -2880,22 +2880,22 @@
         </is>
       </c>
       <c r="B91" s="8" t="n">
-        <v>156.94</v>
+        <v>998.8</v>
       </c>
       <c r="C91" s="10" t="n">
-        <v>154.5</v>
+        <v>981</v>
       </c>
       <c r="D91" s="13" t="n">
-        <v>156.4</v>
+        <v>172</v>
       </c>
       <c r="E91" s="5" t="n">
-        <v>156.26</v>
+        <v>170.29</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>156.73</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="92">
@@ -2905,22 +2905,22 @@
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>651.3</v>
+        <v>998.8</v>
       </c>
       <c r="C92" s="10" t="n">
-        <v>630.7</v>
+        <v>981</v>
       </c>
       <c r="D92" s="13" t="n">
-        <v>642.55</v>
+        <v>610.35</v>
       </c>
       <c r="E92" s="5" t="n">
-        <v>644.95</v>
+        <v>607.75</v>
       </c>
       <c r="F92" s="16" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G92" s="4" t="n">
-        <v>632.05</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="93">
@@ -2930,22 +2930,22 @@
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>1541.95</v>
+        <v>998.8</v>
       </c>
       <c r="C93" s="10" t="n">
-        <v>1508.45</v>
+        <v>981</v>
       </c>
       <c r="D93" s="13" t="n">
-        <v>1531</v>
+        <v>1508.6</v>
       </c>
       <c r="E93" s="5" t="n">
-        <v>1529.1</v>
+        <v>1506.25</v>
       </c>
       <c r="F93" s="16" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G93" s="4" t="n">
-        <v>1509.25</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="94">
@@ -2955,22 +2955,22 @@
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>6235</v>
+        <v>998.8</v>
       </c>
       <c r="C94" s="10" t="n">
-        <v>6116.9</v>
+        <v>981</v>
       </c>
       <c r="D94" s="13" t="n">
-        <v>6199.95</v>
+        <v>6870</v>
       </c>
       <c r="E94" s="5" t="n">
-        <v>6185.35</v>
+        <v>6849.4</v>
       </c>
       <c r="F94" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G94" s="4" t="n">
-        <v>6150</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="95">
@@ -2980,22 +2980,22 @@
         </is>
       </c>
       <c r="B95" s="8" t="n">
-        <v>2153.6</v>
+        <v>998.8</v>
       </c>
       <c r="C95" s="10" t="n">
-        <v>2111</v>
+        <v>981</v>
       </c>
       <c r="D95" s="13" t="n">
-        <v>2150.15</v>
+        <v>2210.1</v>
       </c>
       <c r="E95" s="5" t="n">
-        <v>2141.6</v>
+        <v>2190.45</v>
       </c>
       <c r="F95" s="16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G95" s="4" t="n">
-        <v>2142</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="96">
@@ -3005,22 +3005,22 @@
         </is>
       </c>
       <c r="B96" s="8" t="n">
-        <v>1148.4</v>
+        <v>998.8</v>
       </c>
       <c r="C96" s="10" t="n">
-        <v>1125.55</v>
+        <v>981</v>
       </c>
       <c r="D96" s="13" t="n">
-        <v>1129.55</v>
+        <v>1186.5</v>
       </c>
       <c r="E96" s="5" t="n">
-        <v>1133.95</v>
+        <v>1186.15</v>
       </c>
       <c r="F96" s="16" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>1147.9</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="97">
@@ -3030,22 +3030,22 @@
         </is>
       </c>
       <c r="B97" s="8" t="n">
-        <v>1203</v>
+        <v>998.8</v>
       </c>
       <c r="C97" s="10" t="n">
-        <v>1172.15</v>
+        <v>981</v>
       </c>
       <c r="D97" s="13" t="n">
-        <v>1201.45</v>
+        <v>1282.95</v>
       </c>
       <c r="E97" s="5" t="n">
-        <v>1191.75</v>
+        <v>1279.35</v>
       </c>
       <c r="F97" s="16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G97" s="4" t="n">
-        <v>1182.15</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="98">
@@ -3055,22 +3055,22 @@
         </is>
       </c>
       <c r="B98" s="8" t="n">
-        <v>2992.2</v>
+        <v>998.8</v>
       </c>
       <c r="C98" s="10" t="n">
-        <v>2956.85</v>
+        <v>981</v>
       </c>
       <c r="D98" s="13" t="n">
-        <v>2971.9</v>
+        <v>3116</v>
       </c>
       <c r="E98" s="5" t="n">
-        <v>2974.55</v>
+        <v>3104.6</v>
       </c>
       <c r="F98" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G98" s="4" t="n">
-        <v>2960.95</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="99">
@@ -3080,22 +3080,22 @@
         </is>
       </c>
       <c r="B99" s="8" t="n">
-        <v>1924.25</v>
+        <v>998.8</v>
       </c>
       <c r="C99" s="10" t="n">
-        <v>1903</v>
+        <v>981</v>
       </c>
       <c r="D99" s="13" t="n">
-        <v>1920</v>
+        <v>1990.2</v>
       </c>
       <c r="E99" s="5" t="n">
-        <v>1917.05</v>
+        <v>1991.3</v>
       </c>
       <c r="F99" s="16" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>1907.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="100">
@@ -3105,22 +3105,22 @@
         </is>
       </c>
       <c r="B100" s="8" t="n">
-        <v>690.95</v>
+        <v>998.8</v>
       </c>
       <c r="C100" s="10" t="n">
-        <v>678.5</v>
+        <v>981</v>
       </c>
       <c r="D100" s="13" t="n">
-        <v>683.95</v>
+        <v>734.5</v>
       </c>
       <c r="E100" s="5" t="n">
-        <v>685.5</v>
+        <v>734.55</v>
       </c>
       <c r="F100" s="16" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>690.6</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="101">
@@ -3130,22 +3130,22 @@
         </is>
       </c>
       <c r="B101" s="8" t="n">
-        <v>8297.65</v>
+        <v>998.8</v>
       </c>
       <c r="C101" s="10" t="n">
-        <v>8113.2</v>
+        <v>981</v>
       </c>
       <c r="D101" s="13" t="n">
-        <v>8270</v>
+        <v>8431.549999999999</v>
       </c>
       <c r="E101" s="5" t="n">
-        <v>8255.299999999999</v>
+        <v>8418.85</v>
       </c>
       <c r="F101" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>8157.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="102">
@@ -3155,22 +3155,22 @@
         </is>
       </c>
       <c r="B102" s="8" t="n">
-        <v>3520</v>
+        <v>998.8</v>
       </c>
       <c r="C102" s="10" t="n">
-        <v>3470.6</v>
+        <v>981</v>
       </c>
       <c r="D102" s="13" t="n">
-        <v>3506</v>
+        <v>3533</v>
       </c>
       <c r="E102" s="5" t="n">
-        <v>3507.9</v>
+        <v>3533.1</v>
       </c>
       <c r="F102" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>3474.05</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="103">
@@ -3180,22 +3180,22 @@
         </is>
       </c>
       <c r="B103" s="8" t="n">
-        <v>232.19</v>
+        <v>998.8</v>
       </c>
       <c r="C103" s="10" t="n">
-        <v>227.51</v>
+        <v>981</v>
       </c>
       <c r="D103" s="13" t="n">
-        <v>230</v>
+        <v>241.5</v>
       </c>
       <c r="E103" s="5" t="n">
-        <v>230.07</v>
+        <v>241.53</v>
       </c>
       <c r="F103" s="16" t="n">
-        <v>93</v>
+        <v>131</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>227.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="104">
@@ -3205,22 +3205,22 @@
         </is>
       </c>
       <c r="B104" s="8" t="n">
-        <v>364.75</v>
+        <v>998.8</v>
       </c>
       <c r="C104" s="10" t="n">
-        <v>360.2</v>
+        <v>981</v>
       </c>
       <c r="D104" s="13" t="n">
-        <v>363</v>
+        <v>369.45</v>
       </c>
       <c r="E104" s="5" t="n">
-        <v>363.65</v>
+        <v>369.85</v>
       </c>
       <c r="F104" s="16" t="n">
-        <v>142</v>
+        <v>108</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>362</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="105">
@@ -3230,22 +3230,22 @@
         </is>
       </c>
       <c r="B105" s="8" t="n">
-        <v>2011.95</v>
+        <v>998.8</v>
       </c>
       <c r="C105" s="10" t="n">
-        <v>1955.6</v>
+        <v>981</v>
       </c>
       <c r="D105" s="13" t="n">
-        <v>1999.65</v>
+        <v>2137.7</v>
       </c>
       <c r="E105" s="5" t="n">
-        <v>2007.35</v>
+        <v>2139.9</v>
       </c>
       <c r="F105" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>1984</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="106">
@@ -3255,22 +3255,22 @@
         </is>
       </c>
       <c r="B106" s="8" t="n">
-        <v>258.65</v>
+        <v>998.8</v>
       </c>
       <c r="C106" s="10" t="n">
-        <v>252.4</v>
+        <v>981</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>256.95</v>
+        <v>258.75</v>
       </c>
       <c r="E106" s="5" t="n">
-        <v>256.7</v>
+        <v>258.9</v>
       </c>
       <c r="F106" s="16" t="n">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>252.95</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="107">
@@ -3280,22 +3280,22 @@
         </is>
       </c>
       <c r="B107" s="8" t="n">
-        <v>1191.65</v>
+        <v>998.8</v>
       </c>
       <c r="C107" s="10" t="n">
-        <v>1170</v>
+        <v>981</v>
       </c>
       <c r="D107" s="13" t="n">
-        <v>1184.9</v>
+        <v>1240.95</v>
       </c>
       <c r="E107" s="5" t="n">
-        <v>1185</v>
+        <v>1241.1</v>
       </c>
       <c r="F107" s="16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>1183.85</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="108">
@@ -3305,22 +3305,22 @@
         </is>
       </c>
       <c r="B108" s="8" t="n">
-        <v>5933.95</v>
+        <v>998.8</v>
       </c>
       <c r="C108" s="10" t="n">
-        <v>5827.5</v>
+        <v>981</v>
       </c>
       <c r="D108" s="13" t="n">
-        <v>5897.45</v>
+        <v>6235</v>
       </c>
       <c r="E108" s="5" t="n">
-        <v>5905.65</v>
+        <v>6234.25</v>
       </c>
       <c r="F108" s="16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>5831.3</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="109">
@@ -3330,22 +3330,22 @@
         </is>
       </c>
       <c r="B109" s="8" t="n">
-        <v>337</v>
+        <v>998.8</v>
       </c>
       <c r="C109" s="10" t="n">
-        <v>325.8</v>
+        <v>981</v>
       </c>
       <c r="D109" s="13" t="n">
-        <v>337</v>
+        <v>335.1</v>
       </c>
       <c r="E109" s="5" t="n">
-        <v>333.1</v>
+        <v>335.1</v>
       </c>
       <c r="F109" s="16" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G109" s="4" t="n">
-        <v>328.2</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="110">
@@ -3355,22 +3355,22 @@
         </is>
       </c>
       <c r="B110" s="8" t="n">
-        <v>3074.85</v>
+        <v>998.8</v>
       </c>
       <c r="C110" s="10" t="n">
-        <v>3037.95</v>
+        <v>981</v>
       </c>
       <c r="D110" s="13" t="n">
-        <v>3069.95</v>
+        <v>3160</v>
       </c>
       <c r="E110" s="5" t="n">
-        <v>3066.2</v>
+        <v>3160.75</v>
       </c>
       <c r="F110" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>3038.05</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="111">
@@ -3380,22 +3380,22 @@
         </is>
       </c>
       <c r="B111" s="8" t="n">
-        <v>7320</v>
+        <v>998.8</v>
       </c>
       <c r="C111" s="10" t="n">
-        <v>7154.75</v>
+        <v>981</v>
       </c>
       <c r="D111" s="13" t="n">
-        <v>7310.1</v>
+        <v>7434</v>
       </c>
       <c r="E111" s="5" t="n">
-        <v>7297.9</v>
+        <v>7438.4</v>
       </c>
       <c r="F111" s="16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>7182.8</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="112">
@@ -3405,22 +3405,22 @@
         </is>
       </c>
       <c r="B112" s="8" t="n">
-        <v>331.9</v>
+        <v>998.8</v>
       </c>
       <c r="C112" s="10" t="n">
-        <v>326.5</v>
+        <v>981</v>
       </c>
       <c r="D112" s="13" t="n">
-        <v>329.15</v>
+        <v>329.45</v>
       </c>
       <c r="E112" s="5" t="n">
-        <v>329.4</v>
+        <v>329.1</v>
       </c>
       <c r="F112" s="16" t="n">
-        <v>138</v>
+        <v>93</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>328.35</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="113">
@@ -3430,22 +3430,22 @@
         </is>
       </c>
       <c r="B113" s="8" t="n">
-        <v>154.09</v>
+        <v>998.8</v>
       </c>
       <c r="C113" s="10" t="n">
-        <v>150.9</v>
+        <v>981</v>
       </c>
       <c r="D113" s="13" t="n">
-        <v>153.65</v>
+        <v>187.61</v>
       </c>
       <c r="E113" s="5" t="n">
-        <v>153.74</v>
+        <v>187.1</v>
       </c>
       <c r="F113" s="16" t="n">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="G113" s="4" t="n">
-        <v>152.5</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="114">
@@ -3455,22 +3455,22 @@
         </is>
       </c>
       <c r="B114" s="8" t="n">
-        <v>1022.25</v>
+        <v>998.8</v>
       </c>
       <c r="C114" s="10" t="n">
-        <v>978.5</v>
+        <v>981</v>
       </c>
       <c r="D114" s="13" t="n">
-        <v>1010.1</v>
+        <v>1016.45</v>
       </c>
       <c r="E114" s="5" t="n">
-        <v>1014.8</v>
+        <v>1014.45</v>
       </c>
       <c r="F114" s="16" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="G114" s="4" t="n">
-        <v>981.85</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="115">
@@ -3480,22 +3480,22 @@
         </is>
       </c>
       <c r="B115" s="8" t="n">
-        <v>158.33</v>
+        <v>998.8</v>
       </c>
       <c r="C115" s="10" t="n">
-        <v>152.31</v>
+        <v>981</v>
       </c>
       <c r="D115" s="13" t="n">
-        <v>154.95</v>
+        <v>171.3</v>
       </c>
       <c r="E115" s="5" t="n">
-        <v>154.98</v>
+        <v>171.36</v>
       </c>
       <c r="F115" s="16" t="n">
-        <v>74</v>
+        <v>189</v>
       </c>
       <c r="G115" s="4" t="n">
-        <v>157.91</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="116">
@@ -3505,22 +3505,22 @@
         </is>
       </c>
       <c r="B116" s="8" t="n">
-        <v>535.4</v>
+        <v>998.8</v>
       </c>
       <c r="C116" s="10" t="n">
-        <v>525.85</v>
+        <v>981</v>
       </c>
       <c r="D116" s="13" t="n">
-        <v>533</v>
+        <v>563</v>
       </c>
       <c r="E116" s="5" t="n">
-        <v>532.6</v>
+        <v>563.7</v>
       </c>
       <c r="F116" s="16" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>526.05</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="117">
@@ -3530,22 +3530,22 @@
         </is>
       </c>
       <c r="B117" s="8" t="n">
-        <v>708.8</v>
+        <v>998.8</v>
       </c>
       <c r="C117" s="10" t="n">
-        <v>699</v>
+        <v>981</v>
       </c>
       <c r="D117" s="13" t="n">
-        <v>700</v>
+        <v>719.5</v>
       </c>
       <c r="E117" s="5" t="n">
-        <v>700.6</v>
+        <v>719.65</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>704.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="118">
@@ -3555,22 +3555,22 @@
         </is>
       </c>
       <c r="B118" s="8" t="n">
-        <v>1442.1</v>
+        <v>998.8</v>
       </c>
       <c r="C118" s="10" t="n">
-        <v>1396.65</v>
+        <v>981</v>
       </c>
       <c r="D118" s="13" t="n">
-        <v>1436</v>
+        <v>1467.85</v>
       </c>
       <c r="E118" s="5" t="n">
-        <v>1437.75</v>
+        <v>1469.3</v>
       </c>
       <c r="F118" s="16" t="n">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>1437</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="119">
@@ -3580,22 +3580,22 @@
         </is>
       </c>
       <c r="B119" s="8" t="n">
-        <v>7633</v>
+        <v>998.8</v>
       </c>
       <c r="C119" s="10" t="n">
-        <v>7435.1</v>
+        <v>981</v>
       </c>
       <c r="D119" s="13" t="n">
-        <v>7565</v>
+        <v>7862.3</v>
       </c>
       <c r="E119" s="5" t="n">
-        <v>7560.85</v>
+        <v>7842.05</v>
       </c>
       <c r="F119" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>7480</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="120">
@@ -3605,22 +3605,22 @@
         </is>
       </c>
       <c r="B120" s="8" t="n">
-        <v>2284</v>
+        <v>998.8</v>
       </c>
       <c r="C120" s="10" t="n">
-        <v>2250.55</v>
+        <v>981</v>
       </c>
       <c r="D120" s="13" t="n">
-        <v>2262.2</v>
+        <v>2318.1</v>
       </c>
       <c r="E120" s="5" t="n">
-        <v>2265</v>
+        <v>2302.35</v>
       </c>
       <c r="F120" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>2254.15</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="121">
@@ -3630,22 +3630,22 @@
         </is>
       </c>
       <c r="B121" s="8" t="n">
-        <v>1648.8</v>
+        <v>998.8</v>
       </c>
       <c r="C121" s="10" t="n">
-        <v>1578</v>
+        <v>981</v>
       </c>
       <c r="D121" s="13" t="n">
-        <v>1631</v>
+        <v>716.65</v>
       </c>
       <c r="E121" s="5" t="n">
-        <v>1635.35</v>
+        <v>197.57</v>
       </c>
       <c r="F121" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G121" s="4" t="n">
-        <v>1578.9</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="122">
@@ -3655,22 +3655,22 @@
         </is>
       </c>
       <c r="B122" s="8" t="n">
-        <v>1795.8</v>
+        <v>998.8</v>
       </c>
       <c r="C122" s="10" t="n">
-        <v>1759.55</v>
+        <v>981</v>
       </c>
       <c r="D122" s="13" t="n">
-        <v>1784</v>
+        <v>1807</v>
       </c>
       <c r="E122" s="5" t="n">
-        <v>1780.9</v>
+        <v>1806.65</v>
       </c>
       <c r="F122" s="16" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="G122" s="4" t="n">
-        <v>1767.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="123">
@@ -3680,22 +3680,22 @@
         </is>
       </c>
       <c r="B123" s="8" t="n">
-        <v>943.55</v>
+        <v>998.8</v>
       </c>
       <c r="C123" s="10" t="n">
-        <v>922</v>
+        <v>981</v>
       </c>
       <c r="D123" s="13" t="n">
-        <v>936</v>
+        <v>872.7</v>
       </c>
       <c r="E123" s="5" t="n">
-        <v>940.8</v>
+        <v>867.9</v>
       </c>
       <c r="F123" s="16" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G123" s="4" t="n">
-        <v>924.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="124">
@@ -3705,22 +3705,22 @@
         </is>
       </c>
       <c r="B124" s="8" t="n">
-        <v>1759.1</v>
+        <v>998.8</v>
       </c>
       <c r="C124" s="10" t="n">
-        <v>1733</v>
+        <v>981</v>
       </c>
       <c r="D124" s="13" t="n">
-        <v>1756.75</v>
+        <v>1790.3</v>
       </c>
       <c r="E124" s="5" t="n">
-        <v>1755.1</v>
+        <v>1785.35</v>
       </c>
       <c r="F124" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G124" s="4" t="n">
-        <v>1735.65</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="125">
@@ -3730,22 +3730,22 @@
         </is>
       </c>
       <c r="B125" s="8" t="n">
-        <v>789.4</v>
+        <v>998.8</v>
       </c>
       <c r="C125" s="10" t="n">
-        <v>777.05</v>
+        <v>981</v>
       </c>
       <c r="D125" s="13" t="n">
-        <v>787.35</v>
+        <v>799.7</v>
       </c>
       <c r="E125" s="5" t="n">
-        <v>786.45</v>
+        <v>798.75</v>
       </c>
       <c r="F125" s="16" t="n">
-        <v>103</v>
+        <v>155</v>
       </c>
       <c r="G125" s="4" t="n">
-        <v>778</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="126">
@@ -3755,22 +3755,22 @@
         </is>
       </c>
       <c r="B126" s="8" t="n">
-        <v>4298.7</v>
+        <v>998.8</v>
       </c>
       <c r="C126" s="10" t="n">
-        <v>4212.35</v>
+        <v>981</v>
       </c>
       <c r="D126" s="13" t="n">
-        <v>4266</v>
+        <v>4445.6</v>
       </c>
       <c r="E126" s="5" t="n">
-        <v>4270.85</v>
+        <v>4452.15</v>
       </c>
       <c r="F126" s="16" t="n">
         <v>20</v>
       </c>
       <c r="G126" s="4" t="n">
-        <v>4216.85</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="127">
@@ -3780,22 +3780,22 @@
         </is>
       </c>
       <c r="B127" s="8" t="n">
-        <v>1730</v>
+        <v>998.8</v>
       </c>
       <c r="C127" s="10" t="n">
-        <v>1702.65</v>
+        <v>981</v>
       </c>
       <c r="D127" s="13" t="n">
-        <v>1713</v>
+        <v>1777.25</v>
       </c>
       <c r="E127" s="5" t="n">
-        <v>1712.3</v>
+        <v>1777.85</v>
       </c>
       <c r="F127" s="16" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G127" s="4" t="n">
-        <v>1705</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="128">
@@ -3805,22 +3805,22 @@
         </is>
       </c>
       <c r="B128" s="8" t="n">
-        <v>3260</v>
+        <v>998.8</v>
       </c>
       <c r="C128" s="10" t="n">
-        <v>3221.3</v>
+        <v>981</v>
       </c>
       <c r="D128" s="13" t="n">
-        <v>3245</v>
+        <v>3466.5</v>
       </c>
       <c r="E128" s="5" t="n">
-        <v>3249</v>
+        <v>3468.2</v>
       </c>
       <c r="F128" s="16" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G128" s="4" t="n">
-        <v>3233</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="129">
@@ -3830,22 +3830,22 @@
         </is>
       </c>
       <c r="B129" s="8" t="n">
-        <v>3333.1</v>
+        <v>998.8</v>
       </c>
       <c r="C129" s="10" t="n">
-        <v>3224.5</v>
+        <v>981</v>
       </c>
       <c r="D129" s="13" t="n">
-        <v>3330</v>
+        <v>3344</v>
       </c>
       <c r="E129" s="5" t="n">
-        <v>3324.2</v>
+        <v>3335.7</v>
       </c>
       <c r="F129" s="16" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G129" s="4" t="n">
-        <v>3229.55</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="130">
@@ -3855,22 +3855,22 @@
         </is>
       </c>
       <c r="B130" s="8" t="n">
-        <v>1556.95</v>
+        <v>998.8</v>
       </c>
       <c r="C130" s="10" t="n">
-        <v>1502.2</v>
+        <v>981</v>
       </c>
       <c r="D130" s="13" t="n">
-        <v>1507</v>
+        <v>1649</v>
       </c>
       <c r="E130" s="5" t="n">
-        <v>1510.7</v>
+        <v>1645.95</v>
       </c>
       <c r="F130" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G130" s="4" t="n">
-        <v>1510.8</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="131">
@@ -3880,22 +3880,22 @@
         </is>
       </c>
       <c r="B131" s="8" t="n">
-        <v>6820</v>
+        <v>998.8</v>
       </c>
       <c r="C131" s="10" t="n">
-        <v>6728.1</v>
+        <v>981</v>
       </c>
       <c r="D131" s="13" t="n">
-        <v>6790.8</v>
+        <v>6925</v>
       </c>
       <c r="E131" s="5" t="n">
-        <v>6795.4</v>
+        <v>6949.7</v>
       </c>
       <c r="F131" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>6765</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="132">
@@ -3905,22 +3905,22 @@
         </is>
       </c>
       <c r="B132" s="8" t="n">
-        <v>2445</v>
+        <v>998.8</v>
       </c>
       <c r="C132" s="10" t="n">
-        <v>2406</v>
+        <v>981</v>
       </c>
       <c r="D132" s="13" t="n">
-        <v>2433</v>
+        <v>2497</v>
       </c>
       <c r="E132" s="5" t="n">
-        <v>2434.45</v>
+        <v>2488.85</v>
       </c>
       <c r="F132" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>2406</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="133">
@@ -3930,22 +3930,22 @@
         </is>
       </c>
       <c r="B133" s="8" t="n">
-        <v>1955.95</v>
+        <v>998.8</v>
       </c>
       <c r="C133" s="10" t="n">
-        <v>1932.5</v>
+        <v>981</v>
       </c>
       <c r="D133" s="13" t="n">
-        <v>1950</v>
+        <v>1955</v>
       </c>
       <c r="E133" s="5" t="n">
-        <v>1950.5</v>
+        <v>1958.35</v>
       </c>
       <c r="F133" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G133" s="4" t="n">
-        <v>1941.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="134">
@@ -3955,22 +3955,22 @@
         </is>
       </c>
       <c r="B134" s="8" t="n">
-        <v>11233</v>
+        <v>998.8</v>
       </c>
       <c r="C134" s="10" t="n">
-        <v>11020</v>
+        <v>981</v>
       </c>
       <c r="D134" s="13" t="n">
-        <v>11188</v>
+        <v>11795.2</v>
       </c>
       <c r="E134" s="5" t="n">
-        <v>11202.15</v>
+        <v>11814.8</v>
       </c>
       <c r="F134" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G134" s="4" t="n">
-        <v>11047.05</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="135">
@@ -3980,22 +3980,22 @@
         </is>
       </c>
       <c r="B135" s="8" t="n">
-        <v>546.4</v>
+        <v>998.8</v>
       </c>
       <c r="C135" s="10" t="n">
-        <v>538.25</v>
+        <v>981</v>
       </c>
       <c r="D135" s="13" t="n">
-        <v>544.55</v>
+        <v>555</v>
       </c>
       <c r="E135" s="5" t="n">
-        <v>545</v>
+        <v>555.4</v>
       </c>
       <c r="F135" s="16" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G135" s="4" t="n">
-        <v>540.7</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="136">
@@ -4005,22 +4005,22 @@
         </is>
       </c>
       <c r="B136" s="8" t="n">
-        <v>457.8</v>
+        <v>998.8</v>
       </c>
       <c r="C136" s="10" t="n">
-        <v>449.05</v>
+        <v>981</v>
       </c>
       <c r="D136" s="13" t="n">
-        <v>453.7</v>
+        <v>496.25</v>
       </c>
       <c r="E136" s="5" t="n">
-        <v>453.5</v>
+        <v>497.05</v>
       </c>
       <c r="F136" s="16" t="n">
-        <v>68</v>
+        <v>115</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>450.1</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="137">
@@ -4030,22 +4030,22 @@
         </is>
       </c>
       <c r="B137" s="8" t="n">
-        <v>1666.9</v>
+        <v>998.8</v>
       </c>
       <c r="C137" s="10" t="n">
-        <v>1640.2</v>
+        <v>981</v>
       </c>
       <c r="D137" s="13" t="n">
-        <v>1658</v>
+        <v>1762.95</v>
       </c>
       <c r="E137" s="5" t="n">
-        <v>1658.25</v>
+        <v>1764.35</v>
       </c>
       <c r="F137" s="16" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>1654.15</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="138">
@@ -4055,22 +4055,22 @@
         </is>
       </c>
       <c r="B138" s="8" t="n">
-        <v>132.69</v>
+        <v>998.8</v>
       </c>
       <c r="C138" s="10" t="n">
-        <v>127.5</v>
+        <v>981</v>
       </c>
       <c r="D138" s="13" t="n">
-        <v>129.1</v>
+        <v>140.86</v>
       </c>
       <c r="E138" s="5" t="n">
-        <v>129.16</v>
+        <v>141.29</v>
       </c>
       <c r="F138" s="16" t="n">
-        <v>466</v>
+        <v>97</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>129.82</v>
+        <v>997.65</v>
       </c>
     </row>
     <row r="139" ht="15.75" customHeight="1" thickBot="1">
@@ -4080,22 +4080,22 @@
         </is>
       </c>
       <c r="B139" s="18" t="n">
-        <v>972.75</v>
+        <v>998.8</v>
       </c>
       <c r="C139" s="11" t="n">
-        <v>955</v>
+        <v>981</v>
       </c>
       <c r="D139" s="14" t="n">
-        <v>965.2</v>
+        <v>985</v>
       </c>
       <c r="E139" s="6" t="n">
-        <v>965.95</v>
+        <v>982.45</v>
       </c>
       <c r="F139" s="17" t="n">
         <v>11</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>961.65</v>
+        <v>997.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed GLS to alvius and added a mid run save point for csh and algo so that the high lows get saved in case theres an error in the close extraction
</commit_message>
<xml_diff>
--- a/algo high low.xlsx
+++ b/algo high low.xlsx
@@ -514,7 +514,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -650,12 +650,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -675,6 +688,19 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -1010,1523 +1036,3179 @@
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="4"/>
+      <c r="B2" s="7">
+        <v>446.5</v>
+      </c>
+      <c r="C2" s="9">
+        <v>438.6</v>
+      </c>
+      <c r="D2" s="12">
+        <v>446.5</v>
+      </c>
+      <c r="E2" s="19">
+        <v>444.7</v>
+      </c>
+      <c r="F2" s="15">
+        <v>26</v>
+      </c>
+      <c r="G2" s="4">
+        <v>442</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="4"/>
+      <c r="B3" s="8">
+        <v>5947.85</v>
+      </c>
+      <c r="C3" s="10">
+        <v>5778.6</v>
+      </c>
+      <c r="D3" s="13">
+        <v>5891.35</v>
+      </c>
+      <c r="E3" s="20">
+        <v>5874.65</v>
+      </c>
+      <c r="F3" s="16">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
+        <v>5831.9</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="4"/>
+      <c r="B4" s="8">
+        <v>181.6</v>
+      </c>
+      <c r="C4" s="10">
+        <v>175.91</v>
+      </c>
+      <c r="D4" s="13">
+        <v>179.02</v>
+      </c>
+      <c r="E4" s="20">
+        <v>179.39</v>
+      </c>
+      <c r="F4" s="16">
+        <v>26</v>
+      </c>
+      <c r="G4" s="4">
+        <v>176.25</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="4"/>
+      <c r="B5" s="8">
+        <v>274.75</v>
+      </c>
+      <c r="C5" s="10">
+        <v>270.5</v>
+      </c>
+      <c r="D5" s="13">
+        <v>273.7</v>
+      </c>
+      <c r="E5" s="20">
+        <v>273.85000000000002</v>
+      </c>
+      <c r="F5" s="16">
+        <v>18</v>
+      </c>
+      <c r="G5" s="4">
+        <v>272.5</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="4"/>
+      <c r="B6" s="8">
+        <v>2314.9499999999998</v>
+      </c>
+      <c r="C6" s="10">
+        <v>2238.4</v>
+      </c>
+      <c r="D6" s="13">
+        <v>2297</v>
+      </c>
+      <c r="E6" s="20">
+        <v>2287.8000000000002</v>
+      </c>
+      <c r="F6" s="16">
+        <v>20</v>
+      </c>
+      <c r="G6" s="4">
+        <v>2241.6999999999998</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="4"/>
+      <c r="B7" s="8">
+        <v>1109.25</v>
+      </c>
+      <c r="C7" s="10">
+        <v>1083.3499999999999</v>
+      </c>
+      <c r="D7" s="13">
+        <v>1099</v>
+      </c>
+      <c r="E7" s="20">
+        <v>1099.3499999999999</v>
+      </c>
+      <c r="F7" s="16">
+        <v>46</v>
+      </c>
+      <c r="G7" s="4">
+        <v>1087</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="4"/>
+      <c r="B8" s="8">
+        <v>5087.95</v>
+      </c>
+      <c r="C8" s="10">
+        <v>5010.1000000000004</v>
+      </c>
+      <c r="D8" s="13">
+        <v>5060</v>
+      </c>
+      <c r="E8" s="20">
+        <v>5063.05</v>
+      </c>
+      <c r="F8" s="16">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>5051.3500000000004</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="4"/>
+      <c r="B9" s="8">
+        <v>518.29999999999995</v>
+      </c>
+      <c r="C9" s="10">
+        <v>510.95</v>
+      </c>
+      <c r="D9" s="13">
+        <v>513.15</v>
+      </c>
+      <c r="E9" s="20">
+        <v>512.79999999999995</v>
+      </c>
+      <c r="F9" s="16">
+        <v>23</v>
+      </c>
+      <c r="G9" s="4">
+        <v>513</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="4"/>
+      <c r="B10" s="8">
+        <v>6880</v>
+      </c>
+      <c r="C10" s="10">
+        <v>6798</v>
+      </c>
+      <c r="D10" s="13">
+        <v>6832</v>
+      </c>
+      <c r="E10" s="20">
+        <v>6810.5</v>
+      </c>
+      <c r="F10" s="16">
+        <v>1</v>
+      </c>
+      <c r="G10" s="4">
+        <v>6808.85</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="4"/>
+      <c r="B11" s="8">
+        <v>439.1</v>
+      </c>
+      <c r="C11" s="10">
+        <v>431.8</v>
+      </c>
+      <c r="D11" s="13">
+        <v>437.05</v>
+      </c>
+      <c r="E11" s="20">
+        <v>437.3</v>
+      </c>
+      <c r="F11" s="16">
+        <v>11</v>
+      </c>
+      <c r="G11" s="4">
+        <v>433.8</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="4"/>
+      <c r="B12" s="8">
+        <v>219</v>
+      </c>
+      <c r="C12" s="10">
+        <v>211.31</v>
+      </c>
+      <c r="D12" s="13">
+        <v>217.48</v>
+      </c>
+      <c r="E12" s="20">
+        <v>216.83</v>
+      </c>
+      <c r="F12" s="16">
+        <v>65</v>
+      </c>
+      <c r="G12" s="4">
+        <v>212</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="4"/>
+      <c r="B13" s="8">
+        <v>1531</v>
+      </c>
+      <c r="C13" s="10">
+        <v>1498.7</v>
+      </c>
+      <c r="D13" s="13">
+        <v>1506.15</v>
+      </c>
+      <c r="E13" s="20">
+        <v>1507.3</v>
+      </c>
+      <c r="F13" s="16">
+        <v>10</v>
+      </c>
+      <c r="G13" s="4">
+        <v>1510.45</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="4"/>
+      <c r="B14" s="8">
+        <v>6354.7</v>
+      </c>
+      <c r="C14" s="10">
+        <v>6209.95</v>
+      </c>
+      <c r="D14" s="13">
+        <v>6286</v>
+      </c>
+      <c r="E14" s="20">
+        <v>6285.7</v>
+      </c>
+      <c r="F14" s="16">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>6339.25</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="4"/>
+      <c r="B15" s="8">
+        <v>603.5</v>
+      </c>
+      <c r="C15" s="10">
+        <v>590.1</v>
+      </c>
+      <c r="D15" s="13">
+        <v>603</v>
+      </c>
+      <c r="E15" s="20">
+        <v>600.95000000000005</v>
+      </c>
+      <c r="F15" s="16">
+        <v>27</v>
+      </c>
+      <c r="G15" s="4">
+        <v>592.5</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="4"/>
+      <c r="B16" s="8">
+        <v>1189</v>
+      </c>
+      <c r="C16" s="10">
+        <v>1162.0999999999999</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1170.4000000000001</v>
+      </c>
+      <c r="E16" s="20">
+        <v>1171.9000000000001</v>
+      </c>
+      <c r="F16" s="16">
+        <v>9</v>
+      </c>
+      <c r="G16" s="4">
+        <v>1183.9000000000001</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="4"/>
+      <c r="B17" s="8">
+        <v>8959.9</v>
+      </c>
+      <c r="C17" s="10">
+        <v>8755.25</v>
+      </c>
+      <c r="D17" s="13">
+        <v>8876</v>
+      </c>
+      <c r="E17" s="20">
+        <v>8847.7999999999993</v>
+      </c>
+      <c r="F17" s="16">
+        <v>3</v>
+      </c>
+      <c r="G17" s="4">
+        <v>8762.0499999999993</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="4"/>
+      <c r="B18" s="8">
+        <v>1753.7</v>
+      </c>
+      <c r="C18" s="10">
+        <v>1698.2</v>
+      </c>
+      <c r="D18" s="13">
+        <v>1742.35</v>
+      </c>
+      <c r="E18" s="20">
+        <v>1736.1</v>
+      </c>
+      <c r="F18" s="16">
+        <v>19</v>
+      </c>
+      <c r="G18" s="4">
+        <v>1720.2</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="4"/>
+      <c r="B19" s="8">
+        <v>7980.65</v>
+      </c>
+      <c r="C19" s="10">
+        <v>7791</v>
+      </c>
+      <c r="D19" s="13">
+        <v>7898.75</v>
+      </c>
+      <c r="E19" s="20">
+        <v>7885.1</v>
+      </c>
+      <c r="F19" s="16">
+        <v>18</v>
+      </c>
+      <c r="G19" s="4">
+        <v>7860.6</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="4"/>
+      <c r="B20" s="8">
+        <v>2785.05</v>
+      </c>
+      <c r="C20" s="10">
+        <v>2748.6</v>
+      </c>
+      <c r="D20" s="13">
+        <v>2770</v>
+      </c>
+      <c r="E20" s="20">
+        <v>2771.25</v>
+      </c>
+      <c r="F20" s="16">
+        <v>1</v>
+      </c>
+      <c r="G20" s="4">
+        <v>2772.8</v>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="4"/>
+      <c r="B21" s="8">
+        <v>488.95</v>
+      </c>
+      <c r="C21" s="10">
+        <v>471</v>
+      </c>
+      <c r="D21" s="13">
+        <v>484.6</v>
+      </c>
+      <c r="E21" s="20">
+        <v>487.35</v>
+      </c>
+      <c r="F21" s="16">
+        <v>3</v>
+      </c>
+      <c r="G21" s="4">
+        <v>472.6</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="4"/>
+      <c r="B22" s="8">
+        <v>152.59</v>
+      </c>
+      <c r="C22" s="10">
+        <v>147.35</v>
+      </c>
+      <c r="D22" s="13">
+        <v>151.6</v>
+      </c>
+      <c r="E22" s="20">
+        <v>151.38</v>
+      </c>
+      <c r="F22" s="16">
+        <v>67</v>
+      </c>
+      <c r="G22" s="4">
+        <v>148.25</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="4"/>
+      <c r="B23" s="8">
+        <v>217.13</v>
+      </c>
+      <c r="C23" s="10">
+        <v>211.05</v>
+      </c>
+      <c r="D23" s="13">
+        <v>213.61</v>
+      </c>
+      <c r="E23" s="20">
+        <v>213.39</v>
+      </c>
+      <c r="F23" s="16">
+        <v>508</v>
+      </c>
+      <c r="G23" s="4">
+        <v>214.88</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="4"/>
+      <c r="B24" s="8">
+        <v>1299.95</v>
+      </c>
+      <c r="C24" s="10">
+        <v>1280.5</v>
+      </c>
+      <c r="D24" s="13">
+        <v>1295.3</v>
+      </c>
+      <c r="E24" s="20">
+        <v>1296.8</v>
+      </c>
+      <c r="F24" s="16">
+        <v>2</v>
+      </c>
+      <c r="G24" s="4">
+        <v>1285.9000000000001</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="4"/>
+      <c r="B25" s="8">
+        <v>294.2</v>
+      </c>
+      <c r="C25" s="10">
+        <v>282.85000000000002</v>
+      </c>
+      <c r="D25" s="13">
+        <v>294</v>
+      </c>
+      <c r="E25" s="20">
+        <v>292.64999999999998</v>
+      </c>
+      <c r="F25" s="16">
+        <v>502</v>
+      </c>
+      <c r="G25" s="4">
+        <v>286.64999999999998</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="4"/>
+      <c r="B26" s="8">
+        <v>1238</v>
+      </c>
+      <c r="C26" s="10">
+        <v>1188.5</v>
+      </c>
+      <c r="D26" s="13">
+        <v>1238</v>
+      </c>
+      <c r="E26" s="20">
+        <v>1224.05</v>
+      </c>
+      <c r="F26" s="16">
+        <v>6</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1194.8</v>
+      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="4"/>
+      <c r="B27" s="8">
+        <v>208.68</v>
+      </c>
+      <c r="C27" s="10">
+        <v>198.16</v>
+      </c>
+      <c r="D27" s="13">
+        <v>208.4</v>
+      </c>
+      <c r="E27" s="20">
+        <v>208.09</v>
+      </c>
+      <c r="F27" s="16">
+        <v>211</v>
+      </c>
+      <c r="G27" s="4">
+        <v>199.58</v>
+      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="4"/>
+      <c r="B28" s="8">
+        <v>370.2</v>
+      </c>
+      <c r="C28" s="10">
+        <v>358.55</v>
+      </c>
+      <c r="D28" s="13">
+        <v>361.65</v>
+      </c>
+      <c r="E28" s="20">
+        <v>362.55</v>
+      </c>
+      <c r="F28" s="16">
+        <v>73</v>
+      </c>
+      <c r="G28" s="4">
+        <v>368.6</v>
+      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="4"/>
+      <c r="B29" s="8">
+        <v>5170</v>
+      </c>
+      <c r="C29" s="10">
+        <v>5048.1000000000004</v>
+      </c>
+      <c r="D29" s="13">
+        <v>5129.05</v>
+      </c>
+      <c r="E29" s="20">
+        <v>5129.6499999999996</v>
+      </c>
+      <c r="F29" s="16">
+        <v>3</v>
+      </c>
+      <c r="G29" s="4">
+        <v>5054.45</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="4"/>
+      <c r="B30" s="8">
+        <v>536.95000000000005</v>
+      </c>
+      <c r="C30" s="10">
+        <v>530.35</v>
+      </c>
+      <c r="D30" s="13">
+        <v>535.95000000000005</v>
+      </c>
+      <c r="E30" s="20">
+        <v>534.6</v>
+      </c>
+      <c r="F30" s="16">
+        <v>4</v>
+      </c>
+      <c r="G30" s="4">
+        <v>534.1</v>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="4"/>
+      <c r="B31" s="8">
+        <v>94</v>
+      </c>
+      <c r="C31" s="10">
+        <v>90.75</v>
+      </c>
+      <c r="D31" s="13">
+        <v>93.29</v>
+      </c>
+      <c r="E31" s="20">
+        <v>93.27</v>
+      </c>
+      <c r="F31" s="16">
+        <v>334</v>
+      </c>
+      <c r="G31" s="4">
+        <v>91.8</v>
+      </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="4"/>
+      <c r="B32" s="8">
+        <v>671.5</v>
+      </c>
+      <c r="C32" s="10">
+        <v>652</v>
+      </c>
+      <c r="D32" s="13">
+        <v>667</v>
+      </c>
+      <c r="E32" s="20">
+        <v>667.7</v>
+      </c>
+      <c r="F32" s="16">
+        <v>5</v>
+      </c>
+      <c r="G32" s="4">
+        <v>656.9</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="8"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="4"/>
+      <c r="B33" s="8">
+        <v>507</v>
+      </c>
+      <c r="C33" s="10">
+        <v>494</v>
+      </c>
+      <c r="D33" s="13">
+        <v>504</v>
+      </c>
+      <c r="E33" s="20">
+        <v>504.1</v>
+      </c>
+      <c r="F33" s="16">
+        <v>14</v>
+      </c>
+      <c r="G33" s="4">
+        <v>496.7</v>
+      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="4"/>
+      <c r="B34" s="8">
+        <v>1321.8</v>
+      </c>
+      <c r="C34" s="10">
+        <v>1247.45</v>
+      </c>
+      <c r="D34" s="13">
+        <v>1291.1500000000001</v>
+      </c>
+      <c r="E34" s="20">
+        <v>1285.8499999999999</v>
+      </c>
+      <c r="F34" s="16">
+        <v>34</v>
+      </c>
+      <c r="G34" s="4">
+        <v>1280.8499999999999</v>
+      </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="4"/>
+      <c r="B35" s="8">
+        <v>1491</v>
+      </c>
+      <c r="C35" s="10">
+        <v>1452.1</v>
+      </c>
+      <c r="D35" s="13">
+        <v>1481</v>
+      </c>
+      <c r="E35" s="20">
+        <v>1479.4</v>
+      </c>
+      <c r="F35" s="16">
+        <v>20</v>
+      </c>
+      <c r="G35" s="4">
+        <v>1473.2</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B36" s="8"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="4"/>
+      <c r="B36" s="8">
+        <v>8395</v>
+      </c>
+      <c r="C36" s="10">
+        <v>8205.1</v>
+      </c>
+      <c r="D36" s="13">
+        <v>8258.7000000000007</v>
+      </c>
+      <c r="E36" s="20">
+        <v>8263.85</v>
+      </c>
+      <c r="F36" s="16">
+        <v>3</v>
+      </c>
+      <c r="G36" s="4">
+        <v>8372.4500000000007</v>
+      </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="8"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="4"/>
+      <c r="B37" s="8">
+        <v>786</v>
+      </c>
+      <c r="C37" s="10">
+        <v>719</v>
+      </c>
+      <c r="D37" s="13">
+        <v>778.3</v>
+      </c>
+      <c r="E37" s="20">
+        <v>780.1</v>
+      </c>
+      <c r="F37" s="16">
+        <v>47</v>
+      </c>
+      <c r="G37" s="4">
+        <v>733.25</v>
+      </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="8"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="4"/>
+      <c r="B38" s="8">
+        <v>1829.9</v>
+      </c>
+      <c r="C38" s="10">
+        <v>1802.85</v>
+      </c>
+      <c r="D38" s="13">
+        <v>1810</v>
+      </c>
+      <c r="E38" s="20">
+        <v>1809.55</v>
+      </c>
+      <c r="F38" s="16">
+        <v>4</v>
+      </c>
+      <c r="G38" s="4">
+        <v>1814.8</v>
+      </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="4"/>
+      <c r="B39" s="8">
+        <v>348.95</v>
+      </c>
+      <c r="C39" s="10">
+        <v>340.2</v>
+      </c>
+      <c r="D39" s="13">
+        <v>342.35</v>
+      </c>
+      <c r="E39" s="20">
+        <v>343.4</v>
+      </c>
+      <c r="F39" s="16">
+        <v>17</v>
+      </c>
+      <c r="G39" s="4">
+        <v>344.15</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B40" s="8"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="16"/>
-      <c r="G40" s="4"/>
+      <c r="B40" s="8">
+        <v>2943</v>
+      </c>
+      <c r="C40" s="10">
+        <v>2872.15</v>
+      </c>
+      <c r="D40" s="13">
+        <v>2935</v>
+      </c>
+      <c r="E40" s="20">
+        <v>2914.05</v>
+      </c>
+      <c r="F40" s="16">
+        <v>4</v>
+      </c>
+      <c r="G40" s="4">
+        <v>2900.15</v>
+      </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="16"/>
-      <c r="G41" s="4"/>
+      <c r="B41" s="8">
+        <v>542.79999999999995</v>
+      </c>
+      <c r="C41" s="10">
+        <v>525.5</v>
+      </c>
+      <c r="D41" s="13">
+        <v>529.65</v>
+      </c>
+      <c r="E41" s="20">
+        <v>529.85</v>
+      </c>
+      <c r="F41" s="16">
+        <v>43</v>
+      </c>
+      <c r="G41" s="4">
+        <v>528</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B42" s="8"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="16"/>
-      <c r="G42" s="4"/>
+      <c r="B42" s="8">
+        <v>1872.7</v>
+      </c>
+      <c r="C42" s="10">
+        <v>1848.55</v>
+      </c>
+      <c r="D42" s="13">
+        <v>1863.55</v>
+      </c>
+      <c r="E42" s="20">
+        <v>1866.35</v>
+      </c>
+      <c r="F42" s="16">
+        <v>1</v>
+      </c>
+      <c r="G42" s="4">
+        <v>1849</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B43" s="8"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="16"/>
-      <c r="G43" s="4"/>
+      <c r="B43" s="8">
+        <v>1157.5</v>
+      </c>
+      <c r="C43" s="10">
+        <v>1121</v>
+      </c>
+      <c r="D43" s="13">
+        <v>1135</v>
+      </c>
+      <c r="E43" s="20">
+        <v>1135.8499999999999</v>
+      </c>
+      <c r="F43" s="16">
+        <v>19</v>
+      </c>
+      <c r="G43" s="4">
+        <v>1141.25</v>
+      </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B44" s="8"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="16"/>
-      <c r="G44" s="4"/>
+      <c r="B44" s="8">
+        <v>2334.9499999999998</v>
+      </c>
+      <c r="C44" s="10">
+        <v>2280.1</v>
+      </c>
+      <c r="D44" s="13">
+        <v>2325</v>
+      </c>
+      <c r="E44" s="20">
+        <v>2325.6</v>
+      </c>
+      <c r="F44" s="16">
+        <v>1</v>
+      </c>
+      <c r="G44" s="4">
+        <v>2297.85</v>
+      </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B45" s="8"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="16"/>
-      <c r="G45" s="4"/>
+      <c r="B45" s="8">
+        <v>102</v>
+      </c>
+      <c r="C45" s="10">
+        <v>99.7</v>
+      </c>
+      <c r="D45" s="13">
+        <v>101.98</v>
+      </c>
+      <c r="E45" s="20">
+        <v>101.86</v>
+      </c>
+      <c r="F45" s="16">
+        <v>11</v>
+      </c>
+      <c r="G45" s="4">
+        <v>100.05</v>
+      </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B46" s="8"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="16"/>
-      <c r="G46" s="4"/>
+      <c r="B46" s="8">
+        <v>5707.45</v>
+      </c>
+      <c r="C46" s="10">
+        <v>5548.9</v>
+      </c>
+      <c r="D46" s="13">
+        <v>5550</v>
+      </c>
+      <c r="E46" s="20">
+        <v>5577.7</v>
+      </c>
+      <c r="F46" s="16">
+        <v>4</v>
+      </c>
+      <c r="G46" s="4">
+        <v>5689.25</v>
+      </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="16"/>
-      <c r="G47" s="4"/>
+      <c r="B47" s="8">
+        <v>15036.65</v>
+      </c>
+      <c r="C47" s="10">
+        <v>14407.7</v>
+      </c>
+      <c r="D47" s="13">
+        <v>15018.65</v>
+      </c>
+      <c r="E47" s="20">
+        <v>14985.95</v>
+      </c>
+      <c r="F47" s="16">
+        <v>2</v>
+      </c>
+      <c r="G47" s="4">
+        <v>14816.9</v>
+      </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B48" s="8"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="16"/>
-      <c r="G48" s="4"/>
+      <c r="B48" s="8">
+        <v>754</v>
+      </c>
+      <c r="C48" s="10">
+        <v>738</v>
+      </c>
+      <c r="D48" s="13">
+        <v>745</v>
+      </c>
+      <c r="E48" s="20">
+        <v>745.05</v>
+      </c>
+      <c r="F48" s="16">
+        <v>33</v>
+      </c>
+      <c r="G48" s="4">
+        <v>744</v>
+      </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B49" s="8"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="16"/>
-      <c r="G49" s="4"/>
+      <c r="B49" s="8">
+        <v>1221</v>
+      </c>
+      <c r="C49" s="10">
+        <v>1197.5</v>
+      </c>
+      <c r="D49" s="13">
+        <v>1215.45</v>
+      </c>
+      <c r="E49" s="20">
+        <v>1217.3499999999999</v>
+      </c>
+      <c r="F49" s="16">
+        <v>15</v>
+      </c>
+      <c r="G49" s="4">
+        <v>1198.75</v>
+      </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B50" s="8"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="16"/>
-      <c r="G50" s="4"/>
+      <c r="B50" s="8">
+        <v>3656</v>
+      </c>
+      <c r="C50" s="10">
+        <v>3571.3</v>
+      </c>
+      <c r="D50" s="13">
+        <v>3656</v>
+      </c>
+      <c r="E50" s="20">
+        <v>3623.45</v>
+      </c>
+      <c r="F50" s="16">
+        <v>1</v>
+      </c>
+      <c r="G50" s="4">
+        <v>3582.05</v>
+      </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B51" s="8"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="16"/>
-      <c r="G51" s="4"/>
+      <c r="B51" s="8">
+        <v>375.9</v>
+      </c>
+      <c r="C51" s="10">
+        <v>364.75</v>
+      </c>
+      <c r="D51" s="13">
+        <v>375.7</v>
+      </c>
+      <c r="E51" s="20">
+        <v>374.5</v>
+      </c>
+      <c r="F51" s="16">
+        <v>29</v>
+      </c>
+      <c r="G51" s="4">
+        <v>367.3</v>
+      </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="16"/>
-      <c r="G52" s="4"/>
+      <c r="B52" s="8">
+        <v>1477.25</v>
+      </c>
+      <c r="C52" s="10">
+        <v>1443.55</v>
+      </c>
+      <c r="D52" s="13">
+        <v>1448.75</v>
+      </c>
+      <c r="E52" s="20">
+        <v>1453.2</v>
+      </c>
+      <c r="F52" s="16">
+        <v>3</v>
+      </c>
+      <c r="G52" s="4">
+        <v>1453.6</v>
+      </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B53" s="8"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="16"/>
-      <c r="G53" s="4"/>
+      <c r="B53" s="8">
+        <v>1214.4000000000001</v>
+      </c>
+      <c r="C53" s="10">
+        <v>1188</v>
+      </c>
+      <c r="D53" s="13">
+        <v>1198</v>
+      </c>
+      <c r="E53" s="20">
+        <v>1200.25</v>
+      </c>
+      <c r="F53" s="16">
+        <v>0</v>
+      </c>
+      <c r="G53" s="4">
+        <v>1189.3</v>
+      </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B54" s="8"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="16"/>
-      <c r="G54" s="4"/>
+      <c r="B54" s="8">
+        <v>556.20000000000005</v>
+      </c>
+      <c r="C54" s="10">
+        <v>543</v>
+      </c>
+      <c r="D54" s="13">
+        <v>554.1</v>
+      </c>
+      <c r="E54" s="20">
+        <v>554.45000000000005</v>
+      </c>
+      <c r="F54" s="16">
+        <v>5</v>
+      </c>
+      <c r="G54" s="4">
+        <v>547.75</v>
+      </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B55" s="8"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="16"/>
-      <c r="G55" s="4"/>
+      <c r="B55" s="8">
+        <v>1136.3</v>
+      </c>
+      <c r="C55" s="10">
+        <v>1114</v>
+      </c>
+      <c r="D55" s="13">
+        <v>1118.0999999999999</v>
+      </c>
+      <c r="E55" s="20">
+        <v>1121.25</v>
+      </c>
+      <c r="F55" s="16">
+        <v>23</v>
+      </c>
+      <c r="G55" s="4">
+        <v>1119.5</v>
+      </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B56" s="8"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="13"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="16"/>
-      <c r="G56" s="4"/>
+      <c r="B56" s="8">
+        <v>2346.4499999999998</v>
+      </c>
+      <c r="C56" s="10">
+        <v>2290.75</v>
+      </c>
+      <c r="D56" s="13">
+        <v>2328.4499999999998</v>
+      </c>
+      <c r="E56" s="20">
+        <v>2329.4499999999998</v>
+      </c>
+      <c r="F56" s="16">
+        <v>6</v>
+      </c>
+      <c r="G56" s="4">
+        <v>2296</v>
+      </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B57" s="8"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="16"/>
-      <c r="G57" s="4"/>
+      <c r="B57" s="8">
+        <v>567.65</v>
+      </c>
+      <c r="C57" s="10">
+        <v>551.04999999999995</v>
+      </c>
+      <c r="D57" s="13">
+        <v>555.65</v>
+      </c>
+      <c r="E57" s="20">
+        <v>556.35</v>
+      </c>
+      <c r="F57" s="16">
+        <v>9</v>
+      </c>
+      <c r="G57" s="4">
+        <v>565.45000000000005</v>
+      </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B58" s="8"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="16"/>
-      <c r="G58" s="4"/>
+      <c r="B58" s="8">
+        <v>2518.3000000000002</v>
+      </c>
+      <c r="C58" s="10">
+        <v>2479.3000000000002</v>
+      </c>
+      <c r="D58" s="13">
+        <v>2506.9499999999998</v>
+      </c>
+      <c r="E58" s="20">
+        <v>2508.85</v>
+      </c>
+      <c r="F58" s="16">
+        <v>4</v>
+      </c>
+      <c r="G58" s="4">
+        <v>2481.1</v>
+      </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B59" s="8"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="13"/>
-      <c r="E59" s="5"/>
-      <c r="F59" s="16"/>
-      <c r="G59" s="4"/>
+      <c r="B59" s="8">
+        <v>486.85</v>
+      </c>
+      <c r="C59" s="10">
+        <v>478.3</v>
+      </c>
+      <c r="D59" s="13">
+        <v>486</v>
+      </c>
+      <c r="E59" s="20">
+        <v>486</v>
+      </c>
+      <c r="F59" s="16">
+        <v>2</v>
+      </c>
+      <c r="G59" s="4">
+        <v>480.7</v>
+      </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B60" s="8"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="13"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="16"/>
-      <c r="G60" s="4"/>
+      <c r="B60" s="8">
+        <v>3969</v>
+      </c>
+      <c r="C60" s="10">
+        <v>3836.9</v>
+      </c>
+      <c r="D60" s="13">
+        <v>3963</v>
+      </c>
+      <c r="E60" s="20">
+        <v>3936.8</v>
+      </c>
+      <c r="F60" s="16">
+        <v>19</v>
+      </c>
+      <c r="G60" s="4">
+        <v>3848.45</v>
+      </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B61" s="8"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="13"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="16"/>
-      <c r="G61" s="4"/>
+      <c r="B61" s="8">
+        <v>1569.4</v>
+      </c>
+      <c r="C61" s="10">
+        <v>1528.15</v>
+      </c>
+      <c r="D61" s="13">
+        <v>1565</v>
+      </c>
+      <c r="E61" s="20">
+        <v>1566.2</v>
+      </c>
+      <c r="F61" s="16">
+        <v>6</v>
+      </c>
+      <c r="G61" s="4">
+        <v>1546.4</v>
+      </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B62" s="8"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="13"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="16"/>
-      <c r="G62" s="4"/>
+      <c r="B62" s="8">
+        <v>1738.2</v>
+      </c>
+      <c r="C62" s="10">
+        <v>1713</v>
+      </c>
+      <c r="D62" s="13">
+        <v>1730</v>
+      </c>
+      <c r="E62" s="20">
+        <v>1725.45</v>
+      </c>
+      <c r="F62" s="16">
+        <v>20</v>
+      </c>
+      <c r="G62" s="4">
+        <v>1726.05</v>
+      </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B63" s="8"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="13"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="16"/>
-      <c r="G63" s="4"/>
+      <c r="B63" s="8">
+        <v>4000</v>
+      </c>
+      <c r="C63" s="10">
+        <v>3822.8</v>
+      </c>
+      <c r="D63" s="13">
+        <v>4000</v>
+      </c>
+      <c r="E63" s="20">
+        <v>3869.9</v>
+      </c>
+      <c r="F63" s="16">
+        <v>3</v>
+      </c>
+      <c r="G63" s="4">
+        <v>3828.5</v>
+      </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B64" s="8"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="13"/>
-      <c r="E64" s="5"/>
-      <c r="F64" s="16"/>
-      <c r="G64" s="4"/>
+      <c r="B64" s="8">
+        <v>641</v>
+      </c>
+      <c r="C64" s="10">
+        <v>634.1</v>
+      </c>
+      <c r="D64" s="13">
+        <v>638.85</v>
+      </c>
+      <c r="E64" s="20">
+        <v>638.04999999999995</v>
+      </c>
+      <c r="F64" s="16">
+        <v>10</v>
+      </c>
+      <c r="G64" s="4">
+        <v>635.9</v>
+      </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B65" s="8"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="13"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="16"/>
-      <c r="G65" s="4"/>
+      <c r="B65" s="8">
+        <v>596.4</v>
+      </c>
+      <c r="C65" s="10">
+        <v>585.1</v>
+      </c>
+      <c r="D65" s="13">
+        <v>593.75</v>
+      </c>
+      <c r="E65" s="20">
+        <v>594.29999999999995</v>
+      </c>
+      <c r="F65" s="16">
+        <v>37</v>
+      </c>
+      <c r="G65" s="4">
+        <v>587.5</v>
+      </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B66" s="8"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="13"/>
-      <c r="E66" s="5"/>
-      <c r="F66" s="16"/>
-      <c r="G66" s="4"/>
+      <c r="B66" s="8">
+        <v>240.58</v>
+      </c>
+      <c r="C66" s="10">
+        <v>228.98</v>
+      </c>
+      <c r="D66" s="13">
+        <v>238</v>
+      </c>
+      <c r="E66" s="20">
+        <v>238.98</v>
+      </c>
+      <c r="F66" s="16">
+        <v>46</v>
+      </c>
+      <c r="G66" s="4">
+        <v>229.48</v>
+      </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B67" s="8"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="13"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="16"/>
-      <c r="G67" s="4"/>
+      <c r="B67" s="8">
+        <v>1880.1</v>
+      </c>
+      <c r="C67" s="10">
+        <v>1851.5</v>
+      </c>
+      <c r="D67" s="13">
+        <v>1864.85</v>
+      </c>
+      <c r="E67" s="20">
+        <v>1858.5</v>
+      </c>
+      <c r="F67" s="16">
+        <v>5</v>
+      </c>
+      <c r="G67" s="4">
+        <v>1861.6</v>
+      </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B68" s="8"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="13"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="16"/>
-      <c r="G68" s="4"/>
+      <c r="B68" s="8">
+        <v>620.95000000000005</v>
+      </c>
+      <c r="C68" s="10">
+        <v>610.5</v>
+      </c>
+      <c r="D68" s="13">
+        <v>617.04999999999995</v>
+      </c>
+      <c r="E68" s="20">
+        <v>616</v>
+      </c>
+      <c r="F68" s="16">
+        <v>5</v>
+      </c>
+      <c r="G68" s="4">
+        <v>615.6</v>
+      </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B69" s="8"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="13"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="16"/>
-      <c r="G69" s="4"/>
+      <c r="B69" s="8">
+        <v>177.4</v>
+      </c>
+      <c r="C69" s="10">
+        <v>173.5</v>
+      </c>
+      <c r="D69" s="13">
+        <v>174.64</v>
+      </c>
+      <c r="E69" s="20">
+        <v>174.6</v>
+      </c>
+      <c r="F69" s="16">
+        <v>42</v>
+      </c>
+      <c r="G69" s="4">
+        <v>173.78</v>
+      </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B70" s="8"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="13"/>
-      <c r="E70" s="5"/>
-      <c r="F70" s="16"/>
-      <c r="G70" s="4"/>
+      <c r="B70" s="8">
+        <v>203.45</v>
+      </c>
+      <c r="C70" s="10">
+        <v>196.35</v>
+      </c>
+      <c r="D70" s="13">
+        <v>202.2</v>
+      </c>
+      <c r="E70" s="20">
+        <v>201.8</v>
+      </c>
+      <c r="F70" s="16">
+        <v>58</v>
+      </c>
+      <c r="G70" s="4">
+        <v>197.75</v>
+      </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B71" s="8"/>
-      <c r="C71" s="10"/>
-      <c r="D71" s="13"/>
-      <c r="E71" s="5"/>
-      <c r="F71" s="16"/>
-      <c r="G71" s="4"/>
+      <c r="B71" s="8">
+        <v>771.35</v>
+      </c>
+      <c r="C71" s="10">
+        <v>763</v>
+      </c>
+      <c r="D71" s="13">
+        <v>765</v>
+      </c>
+      <c r="E71" s="20">
+        <v>764.7</v>
+      </c>
+      <c r="F71" s="16">
+        <v>25</v>
+      </c>
+      <c r="G71" s="4">
+        <v>766.6</v>
+      </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B72" s="8"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="13"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="16"/>
-      <c r="G72" s="4"/>
+      <c r="B72" s="8">
+        <v>271.75</v>
+      </c>
+      <c r="C72" s="10">
+        <v>261</v>
+      </c>
+      <c r="D72" s="13">
+        <v>265</v>
+      </c>
+      <c r="E72" s="20">
+        <v>264.10000000000002</v>
+      </c>
+      <c r="F72" s="16">
+        <v>8</v>
+      </c>
+      <c r="G72" s="4">
+        <v>264.5</v>
+      </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B73" s="8"/>
-      <c r="C73" s="10"/>
-      <c r="D73" s="13"/>
-      <c r="E73" s="5"/>
-      <c r="F73" s="16"/>
-      <c r="G73" s="4"/>
+      <c r="B73" s="8">
+        <v>2083.6999999999998</v>
+      </c>
+      <c r="C73" s="10">
+        <v>2057.6</v>
+      </c>
+      <c r="D73" s="13">
+        <v>2072.6</v>
+      </c>
+      <c r="E73" s="20">
+        <v>2066.4</v>
+      </c>
+      <c r="F73" s="16">
+        <v>3</v>
+      </c>
+      <c r="G73" s="4">
+        <v>2081.3000000000002</v>
+      </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B74" s="8"/>
-      <c r="C74" s="10"/>
-      <c r="D74" s="13"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="16"/>
-      <c r="G74" s="4"/>
+      <c r="B74" s="8">
+        <v>4344.8500000000004</v>
+      </c>
+      <c r="C74" s="10">
+        <v>4226.25</v>
+      </c>
+      <c r="D74" s="13">
+        <v>4334.8</v>
+      </c>
+      <c r="E74" s="20">
+        <v>4324.3500000000004</v>
+      </c>
+      <c r="F74" s="16">
+        <v>5</v>
+      </c>
+      <c r="G74" s="4">
+        <v>4237.05</v>
+      </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B75" s="8"/>
-      <c r="C75" s="10"/>
-      <c r="D75" s="13"/>
-      <c r="E75" s="5"/>
-      <c r="F75" s="16"/>
-      <c r="G75" s="4"/>
+      <c r="B75" s="8">
+        <v>999.3</v>
+      </c>
+      <c r="C75" s="10">
+        <v>953.85</v>
+      </c>
+      <c r="D75" s="13">
+        <v>995.2</v>
+      </c>
+      <c r="E75" s="20">
+        <v>991.2</v>
+      </c>
+      <c r="F75" s="16">
+        <v>53</v>
+      </c>
+      <c r="G75" s="4">
+        <v>962.75</v>
+      </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B76" s="8"/>
-      <c r="C76" s="10"/>
-      <c r="D76" s="13"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="16"/>
-      <c r="G76" s="4"/>
+      <c r="B76" s="8">
+        <v>348.9</v>
+      </c>
+      <c r="C76" s="10">
+        <v>342.4</v>
+      </c>
+      <c r="D76" s="13">
+        <v>346.25</v>
+      </c>
+      <c r="E76" s="20">
+        <v>347.2</v>
+      </c>
+      <c r="F76" s="16">
+        <v>64</v>
+      </c>
+      <c r="G76" s="4">
+        <v>345.85</v>
+      </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B77" s="8"/>
-      <c r="C77" s="10"/>
-      <c r="D77" s="13"/>
-      <c r="E77" s="5"/>
-      <c r="F77" s="16"/>
-      <c r="G77" s="4"/>
+      <c r="B77" s="8">
+        <v>824.8</v>
+      </c>
+      <c r="C77" s="10">
+        <v>775.45</v>
+      </c>
+      <c r="D77" s="13">
+        <v>809</v>
+      </c>
+      <c r="E77" s="20">
+        <v>811</v>
+      </c>
+      <c r="F77" s="16">
+        <v>14</v>
+      </c>
+      <c r="G77" s="4">
+        <v>778.1</v>
+      </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B78" s="8"/>
-      <c r="C78" s="10"/>
-      <c r="D78" s="13"/>
-      <c r="E78" s="5"/>
-      <c r="F78" s="16"/>
-      <c r="G78" s="4"/>
+      <c r="B78" s="8">
+        <v>1470.9</v>
+      </c>
+      <c r="C78" s="10">
+        <v>1428.95</v>
+      </c>
+      <c r="D78" s="13">
+        <v>1443</v>
+      </c>
+      <c r="E78" s="20">
+        <v>1443.3</v>
+      </c>
+      <c r="F78" s="16">
+        <v>2</v>
+      </c>
+      <c r="G78" s="4">
+        <v>1460.4</v>
+      </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B79" s="8"/>
-      <c r="C79" s="10"/>
-      <c r="D79" s="13"/>
-      <c r="E79" s="5"/>
-      <c r="F79" s="16"/>
-      <c r="G79" s="4"/>
+      <c r="B79" s="8">
+        <v>796.8</v>
+      </c>
+      <c r="C79" s="10">
+        <v>723.35</v>
+      </c>
+      <c r="D79" s="13">
+        <v>787.7</v>
+      </c>
+      <c r="E79" s="20">
+        <v>791.55</v>
+      </c>
+      <c r="F79" s="16">
+        <v>226</v>
+      </c>
+      <c r="G79" s="4">
+        <v>756.05</v>
+      </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B80" s="8"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="13"/>
-      <c r="E80" s="5"/>
-      <c r="F80" s="16"/>
-      <c r="G80" s="4"/>
+      <c r="B80" s="8">
+        <v>4848</v>
+      </c>
+      <c r="C80" s="10">
+        <v>4755</v>
+      </c>
+      <c r="D80" s="13">
+        <v>4801.25</v>
+      </c>
+      <c r="E80" s="20">
+        <v>4834.8500000000004</v>
+      </c>
+      <c r="F80" s="16">
+        <v>0</v>
+      </c>
+      <c r="G80" s="4">
+        <v>4801.55</v>
+      </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B81" s="8"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="13"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="16"/>
-      <c r="G81" s="4"/>
+      <c r="B81" s="8">
+        <v>959.9</v>
+      </c>
+      <c r="C81" s="10">
+        <v>940.55</v>
+      </c>
+      <c r="D81" s="13">
+        <v>944.7</v>
+      </c>
+      <c r="E81" s="20">
+        <v>945</v>
+      </c>
+      <c r="F81" s="16">
+        <v>20</v>
+      </c>
+      <c r="G81" s="4">
+        <v>948.1</v>
+      </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B82" s="8"/>
-      <c r="C82" s="10"/>
-      <c r="D82" s="13"/>
-      <c r="E82" s="5"/>
-      <c r="F82" s="16"/>
-      <c r="G82" s="4"/>
+      <c r="B82" s="8">
+        <v>710.95</v>
+      </c>
+      <c r="C82" s="10">
+        <v>698.1</v>
+      </c>
+      <c r="D82" s="13">
+        <v>702.1</v>
+      </c>
+      <c r="E82" s="20">
+        <v>703.9</v>
+      </c>
+      <c r="F82" s="16">
+        <v>13</v>
+      </c>
+      <c r="G82" s="4">
+        <v>703.9</v>
+      </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B83" s="8"/>
-      <c r="C83" s="10"/>
-      <c r="D83" s="13"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="16"/>
-      <c r="G83" s="4"/>
+      <c r="B83" s="8">
+        <v>1906.9</v>
+      </c>
+      <c r="C83" s="10">
+        <v>1889.6</v>
+      </c>
+      <c r="D83" s="13">
+        <v>1900</v>
+      </c>
+      <c r="E83" s="20">
+        <v>1901.3</v>
+      </c>
+      <c r="F83" s="16">
+        <v>23</v>
+      </c>
+      <c r="G83" s="4">
+        <v>1895.95</v>
+      </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B84" s="8"/>
-      <c r="C84" s="10"/>
-      <c r="D84" s="13"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="16"/>
-      <c r="G84" s="4"/>
+      <c r="B84" s="8">
+        <v>2919.95</v>
+      </c>
+      <c r="C84" s="10">
+        <v>2822.05</v>
+      </c>
+      <c r="D84" s="13">
+        <v>2840</v>
+      </c>
+      <c r="E84" s="20">
+        <v>2853.05</v>
+      </c>
+      <c r="F84" s="16">
+        <v>2</v>
+      </c>
+      <c r="G84" s="4">
+        <v>2912.2</v>
+      </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B85" s="8"/>
-      <c r="C85" s="10"/>
-      <c r="D85" s="13"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="16"/>
-      <c r="G85" s="4"/>
+      <c r="B85" s="8">
+        <v>592.45000000000005</v>
+      </c>
+      <c r="C85" s="10">
+        <v>578</v>
+      </c>
+      <c r="D85" s="13">
+        <v>585</v>
+      </c>
+      <c r="E85" s="20">
+        <v>584.04999999999995</v>
+      </c>
+      <c r="F85" s="16">
+        <v>28</v>
+      </c>
+      <c r="G85" s="4">
+        <v>587.79999999999995</v>
+      </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B86" s="8"/>
-      <c r="C86" s="10"/>
-      <c r="D86" s="13"/>
-      <c r="E86" s="5"/>
-      <c r="F86" s="16"/>
-      <c r="G86" s="4"/>
+      <c r="B86" s="8">
+        <v>601.45000000000005</v>
+      </c>
+      <c r="C86" s="10">
+        <v>570.25</v>
+      </c>
+      <c r="D86" s="13">
+        <v>600</v>
+      </c>
+      <c r="E86" s="20">
+        <v>598.1</v>
+      </c>
+      <c r="F86" s="16">
+        <v>30</v>
+      </c>
+      <c r="G86" s="4">
+        <v>582.9</v>
+      </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B87" s="8"/>
-      <c r="C87" s="10"/>
-      <c r="D87" s="13"/>
-      <c r="E87" s="5"/>
-      <c r="F87" s="16"/>
-      <c r="G87" s="4"/>
+      <c r="B87" s="8">
+        <v>5955</v>
+      </c>
+      <c r="C87" s="10">
+        <v>5823.25</v>
+      </c>
+      <c r="D87" s="13">
+        <v>5933</v>
+      </c>
+      <c r="E87" s="20">
+        <v>5914.15</v>
+      </c>
+      <c r="F87" s="16">
+        <v>2</v>
+      </c>
+      <c r="G87" s="4">
+        <v>5911.55</v>
+      </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B88" s="8"/>
-      <c r="C88" s="10"/>
-      <c r="D88" s="13"/>
-      <c r="E88" s="5"/>
-      <c r="F88" s="16"/>
-      <c r="G88" s="4"/>
+      <c r="B88" s="8">
+        <v>5463.8</v>
+      </c>
+      <c r="C88" s="10">
+        <v>5325</v>
+      </c>
+      <c r="D88" s="13">
+        <v>5422.6</v>
+      </c>
+      <c r="E88" s="20">
+        <v>5449.35</v>
+      </c>
+      <c r="F88" s="16">
+        <v>0</v>
+      </c>
+      <c r="G88" s="4">
+        <v>5403.95</v>
+      </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B89" s="8"/>
-      <c r="C89" s="10"/>
-      <c r="D89" s="13"/>
-      <c r="E89" s="5"/>
-      <c r="F89" s="16"/>
-      <c r="G89" s="4"/>
+      <c r="B89" s="8">
+        <v>2109.4</v>
+      </c>
+      <c r="C89" s="10">
+        <v>2066</v>
+      </c>
+      <c r="D89" s="13">
+        <v>2089.0500000000002</v>
+      </c>
+      <c r="E89" s="20">
+        <v>2080.4499999999998</v>
+      </c>
+      <c r="F89" s="16">
+        <v>8</v>
+      </c>
+      <c r="G89" s="4">
+        <v>2094.4499999999998</v>
+      </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B90" s="8"/>
-      <c r="C90" s="10"/>
-      <c r="D90" s="13"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="16"/>
-      <c r="G90" s="4"/>
+      <c r="B90" s="8">
+        <v>285.8</v>
+      </c>
+      <c r="C90" s="10">
+        <v>277</v>
+      </c>
+      <c r="D90" s="13">
+        <v>285.10000000000002</v>
+      </c>
+      <c r="E90" s="20">
+        <v>284.95</v>
+      </c>
+      <c r="F90" s="16">
+        <v>13</v>
+      </c>
+      <c r="G90" s="4">
+        <v>278.10000000000002</v>
+      </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B91" s="8"/>
-      <c r="C91" s="10"/>
-      <c r="D91" s="13"/>
-      <c r="E91" s="5"/>
-      <c r="F91" s="16"/>
-      <c r="G91" s="4"/>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B91" s="8">
+        <v>199.95</v>
+      </c>
+      <c r="C91" s="10">
+        <v>195.24</v>
+      </c>
+      <c r="D91" s="13">
+        <v>196.18</v>
+      </c>
+      <c r="E91" s="20">
+        <v>196.03</v>
+      </c>
+      <c r="F91" s="16">
+        <v>47</v>
+      </c>
+      <c r="G91" s="4">
+        <v>199.57</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B92" s="8"/>
-      <c r="C92" s="10"/>
-      <c r="D92" s="13"/>
-      <c r="E92" s="5"/>
-      <c r="F92" s="16"/>
-      <c r="G92" s="4"/>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B92" s="8">
+        <v>686.55</v>
+      </c>
+      <c r="C92" s="10">
+        <v>655.04999999999995</v>
+      </c>
+      <c r="D92" s="13">
+        <v>670.85</v>
+      </c>
+      <c r="E92" s="22">
+        <v>670.65</v>
+      </c>
+      <c r="F92" s="16">
+        <v>36</v>
+      </c>
+      <c r="G92" s="4">
+        <v>673.75</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B93" s="8"/>
-      <c r="C93" s="10"/>
-      <c r="D93" s="13"/>
-      <c r="E93" s="5"/>
-      <c r="F93" s="16"/>
-      <c r="G93" s="4"/>
+      <c r="B93" s="8">
+        <v>1437.95</v>
+      </c>
+      <c r="C93" s="10">
+        <v>1417.2</v>
+      </c>
+      <c r="D93" s="13">
+        <v>1424</v>
+      </c>
+      <c r="E93" s="23">
+        <v>1424</v>
+      </c>
+      <c r="F93" s="16">
+        <v>6</v>
+      </c>
+      <c r="G93" s="4">
+        <v>1434.9</v>
+      </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B94" s="8"/>
-      <c r="C94" s="10"/>
-      <c r="D94" s="13"/>
-      <c r="E94" s="5"/>
-      <c r="F94" s="16"/>
-      <c r="G94" s="4"/>
+      <c r="B94" s="8">
+        <v>5757</v>
+      </c>
+      <c r="C94" s="10">
+        <v>5594.25</v>
+      </c>
+      <c r="D94" s="13">
+        <v>5730</v>
+      </c>
+      <c r="E94" s="19">
+        <v>5732.95</v>
+      </c>
+      <c r="F94" s="16">
+        <v>2</v>
+      </c>
+      <c r="G94" s="4">
+        <v>5618.5</v>
+      </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B95" s="8"/>
-      <c r="C95" s="10"/>
-      <c r="D95" s="13"/>
-      <c r="E95" s="5"/>
-      <c r="F95" s="16"/>
-      <c r="G95" s="4"/>
+      <c r="B95" s="8">
+        <v>1811.95</v>
+      </c>
+      <c r="C95" s="10">
+        <v>1773.8</v>
+      </c>
+      <c r="D95" s="13">
+        <v>1792.8</v>
+      </c>
+      <c r="E95" s="20">
+        <v>1796.9</v>
+      </c>
+      <c r="F95" s="16">
+        <v>0</v>
+      </c>
+      <c r="G95" s="4">
+        <v>1803.6</v>
+      </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B96" s="8"/>
-      <c r="C96" s="10"/>
-      <c r="D96" s="13"/>
-      <c r="E96" s="5"/>
-      <c r="F96" s="16"/>
-      <c r="G96" s="4"/>
+      <c r="B96" s="8">
+        <v>1119.95</v>
+      </c>
+      <c r="C96" s="10">
+        <v>1083.25</v>
+      </c>
+      <c r="D96" s="13">
+        <v>1118.7</v>
+      </c>
+      <c r="E96" s="20">
+        <v>1115.75</v>
+      </c>
+      <c r="F96" s="16">
+        <v>3</v>
+      </c>
+      <c r="G96" s="4">
+        <v>1084.7</v>
+      </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B97" s="8"/>
-      <c r="C97" s="10"/>
-      <c r="D97" s="13"/>
-      <c r="E97" s="5"/>
-      <c r="F97" s="16"/>
-      <c r="G97" s="4"/>
+      <c r="B97" s="8">
+        <v>1385.45</v>
+      </c>
+      <c r="C97" s="10">
+        <v>1332.25</v>
+      </c>
+      <c r="D97" s="13">
+        <v>1378</v>
+      </c>
+      <c r="E97" s="20">
+        <v>1379.85</v>
+      </c>
+      <c r="F97" s="16">
+        <v>15</v>
+      </c>
+      <c r="G97" s="4">
+        <v>1336</v>
+      </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B98" s="8"/>
-      <c r="C98" s="10"/>
-      <c r="D98" s="13"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="16"/>
-      <c r="G98" s="4"/>
+      <c r="B98" s="8">
+        <v>2901.4</v>
+      </c>
+      <c r="C98" s="10">
+        <v>2853.35</v>
+      </c>
+      <c r="D98" s="13">
+        <v>2865.05</v>
+      </c>
+      <c r="E98" s="20">
+        <v>2867.95</v>
+      </c>
+      <c r="F98" s="16">
+        <v>4</v>
+      </c>
+      <c r="G98" s="4">
+        <v>2884.75</v>
+      </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B99" s="8"/>
-      <c r="C99" s="10"/>
-      <c r="D99" s="13"/>
-      <c r="E99" s="5"/>
-      <c r="F99" s="16"/>
-      <c r="G99" s="4"/>
+      <c r="B99" s="8">
+        <v>2269.25</v>
+      </c>
+      <c r="C99" s="10">
+        <v>2218</v>
+      </c>
+      <c r="D99" s="13">
+        <v>2250</v>
+      </c>
+      <c r="E99" s="20">
+        <v>2258.8000000000002</v>
+      </c>
+      <c r="F99" s="16">
+        <v>5</v>
+      </c>
+      <c r="G99" s="4">
+        <v>2225.65</v>
+      </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="B100" s="8"/>
-      <c r="C100" s="10"/>
-      <c r="D100" s="13"/>
-      <c r="E100" s="5"/>
-      <c r="F100" s="16"/>
-      <c r="G100" s="4"/>
+      <c r="B100" s="8">
+        <v>590.6</v>
+      </c>
+      <c r="C100" s="10">
+        <v>572</v>
+      </c>
+      <c r="D100" s="13">
+        <v>583</v>
+      </c>
+      <c r="E100" s="20">
+        <v>583.79999999999995</v>
+      </c>
+      <c r="F100" s="16">
+        <v>8</v>
+      </c>
+      <c r="G100" s="4">
+        <v>581.70000000000005</v>
+      </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B101" s="8"/>
-      <c r="C101" s="10"/>
-      <c r="D101" s="13"/>
-      <c r="E101" s="5"/>
-      <c r="F101" s="16"/>
-      <c r="G101" s="4"/>
+      <c r="B101" s="8">
+        <v>7750</v>
+      </c>
+      <c r="C101" s="10">
+        <v>7675</v>
+      </c>
+      <c r="D101" s="13">
+        <v>7730</v>
+      </c>
+      <c r="E101" s="20">
+        <v>7723.7</v>
+      </c>
+      <c r="F101" s="16">
+        <v>2</v>
+      </c>
+      <c r="G101" s="4">
+        <v>7683.85</v>
+      </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B102" s="8"/>
-      <c r="C102" s="10"/>
-      <c r="D102" s="13"/>
-      <c r="E102" s="5"/>
-      <c r="F102" s="16"/>
-      <c r="G102" s="4"/>
+      <c r="B102" s="8">
+        <v>4299.05</v>
+      </c>
+      <c r="C102" s="10">
+        <v>4128.55</v>
+      </c>
+      <c r="D102" s="13">
+        <v>4145</v>
+      </c>
+      <c r="E102" s="20">
+        <v>4148.7</v>
+      </c>
+      <c r="F102" s="16">
+        <v>24</v>
+      </c>
+      <c r="G102" s="4">
+        <v>4179.7</v>
+      </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B103" s="8"/>
-      <c r="C103" s="10"/>
-      <c r="D103" s="13"/>
-      <c r="E103" s="5"/>
-      <c r="F103" s="16"/>
-      <c r="G103" s="4"/>
+      <c r="B103" s="8">
+        <v>66.3</v>
+      </c>
+      <c r="C103" s="10">
+        <v>64.540000000000006</v>
+      </c>
+      <c r="D103" s="13">
+        <v>66.08</v>
+      </c>
+      <c r="E103" s="20">
+        <v>66.099999999999994</v>
+      </c>
+      <c r="F103" s="16">
+        <v>159</v>
+      </c>
+      <c r="G103" s="4">
+        <v>64.91</v>
+      </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B104" s="8"/>
-      <c r="C104" s="10"/>
-      <c r="D104" s="13"/>
-      <c r="E104" s="5"/>
-      <c r="F104" s="16"/>
-      <c r="G104" s="4"/>
+      <c r="B104" s="8">
+        <v>326.25</v>
+      </c>
+      <c r="C104" s="10">
+        <v>319.10000000000002</v>
+      </c>
+      <c r="D104" s="13">
+        <v>325.14999999999998</v>
+      </c>
+      <c r="E104" s="20">
+        <v>324</v>
+      </c>
+      <c r="F104" s="16">
+        <v>131</v>
+      </c>
+      <c r="G104" s="4">
+        <v>319.8</v>
+      </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B105" s="8"/>
-      <c r="C105" s="10"/>
-      <c r="D105" s="13"/>
-      <c r="E105" s="5"/>
-      <c r="F105" s="16"/>
-      <c r="G105" s="4"/>
+      <c r="B105" s="8">
+        <v>1842.95</v>
+      </c>
+      <c r="C105" s="10">
+        <v>1775.5</v>
+      </c>
+      <c r="D105" s="13">
+        <v>1813.45</v>
+      </c>
+      <c r="E105" s="20">
+        <v>1812.65</v>
+      </c>
+      <c r="F105" s="16">
+        <v>13</v>
+      </c>
+      <c r="G105" s="4">
+        <v>1777.1</v>
+      </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B106" s="8"/>
-      <c r="C106" s="10"/>
-      <c r="D106" s="13"/>
-      <c r="E106" s="5"/>
-      <c r="F106" s="16"/>
-      <c r="G106" s="4"/>
+      <c r="B106" s="8">
+        <v>263.49</v>
+      </c>
+      <c r="C106" s="10">
+        <v>256.3</v>
+      </c>
+      <c r="D106" s="13">
+        <v>262.8</v>
+      </c>
+      <c r="E106" s="20">
+        <v>262.61</v>
+      </c>
+      <c r="F106" s="16">
+        <v>88</v>
+      </c>
+      <c r="G106" s="4">
+        <v>257.2</v>
+      </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B107" s="8"/>
-      <c r="C107" s="10"/>
-      <c r="D107" s="13"/>
-      <c r="E107" s="5"/>
-      <c r="F107" s="16"/>
-      <c r="G107" s="4"/>
+      <c r="B107" s="8">
+        <v>1026.45</v>
+      </c>
+      <c r="C107" s="10">
+        <v>974.25</v>
+      </c>
+      <c r="D107" s="13">
+        <v>1022</v>
+      </c>
+      <c r="E107" s="20">
+        <v>1023.1</v>
+      </c>
+      <c r="F107" s="16">
+        <v>5</v>
+      </c>
+      <c r="G107" s="4">
+        <v>976</v>
+      </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B108" s="8"/>
-      <c r="C108" s="10"/>
-      <c r="D108" s="13"/>
-      <c r="E108" s="5"/>
-      <c r="F108" s="16"/>
-      <c r="G108" s="4"/>
+      <c r="B108" s="8">
+        <v>6137.2</v>
+      </c>
+      <c r="C108" s="10">
+        <v>5964</v>
+      </c>
+      <c r="D108" s="13">
+        <v>6058.1</v>
+      </c>
+      <c r="E108" s="20">
+        <v>6032.6</v>
+      </c>
+      <c r="F108" s="16">
+        <v>3</v>
+      </c>
+      <c r="G108" s="4">
+        <v>6119.4</v>
+      </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B109" s="8"/>
-      <c r="C109" s="10"/>
-      <c r="D109" s="13"/>
-      <c r="E109" s="5"/>
-      <c r="F109" s="16"/>
-      <c r="G109" s="4"/>
+      <c r="B109" s="8">
+        <v>317</v>
+      </c>
+      <c r="C109" s="10">
+        <v>303.95</v>
+      </c>
+      <c r="D109" s="13">
+        <v>316.10000000000002</v>
+      </c>
+      <c r="E109" s="20">
+        <v>316.2</v>
+      </c>
+      <c r="F109" s="16">
+        <v>17</v>
+      </c>
+      <c r="G109" s="4">
+        <v>304.10000000000002</v>
+      </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B110" s="8"/>
-      <c r="C110" s="10"/>
-      <c r="D110" s="13"/>
-      <c r="E110" s="5"/>
-      <c r="F110" s="16"/>
-      <c r="G110" s="4"/>
+      <c r="B110" s="8">
+        <v>2901.3</v>
+      </c>
+      <c r="C110" s="10">
+        <v>2845</v>
+      </c>
+      <c r="D110" s="13">
+        <v>2882</v>
+      </c>
+      <c r="E110" s="20">
+        <v>2871.7</v>
+      </c>
+      <c r="F110" s="16">
+        <v>3</v>
+      </c>
+      <c r="G110" s="4">
+        <v>2881.75</v>
+      </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B111" s="8"/>
-      <c r="C111" s="10"/>
-      <c r="D111" s="13"/>
-      <c r="E111" s="5"/>
-      <c r="F111" s="16"/>
-      <c r="G111" s="4"/>
+      <c r="B111" s="8">
+        <v>6053.6</v>
+      </c>
+      <c r="C111" s="10">
+        <v>5877.2</v>
+      </c>
+      <c r="D111" s="13">
+        <v>6032.9</v>
+      </c>
+      <c r="E111" s="20">
+        <v>6037.95</v>
+      </c>
+      <c r="F111" s="16">
+        <v>6</v>
+      </c>
+      <c r="G111" s="4">
+        <v>5920</v>
+      </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B112" s="8"/>
-      <c r="C112" s="10"/>
-      <c r="D112" s="13"/>
-      <c r="E112" s="5"/>
-      <c r="F112" s="16"/>
-      <c r="G112" s="4"/>
+      <c r="B112" s="8">
+        <v>303.45</v>
+      </c>
+      <c r="C112" s="10">
+        <v>298.55</v>
+      </c>
+      <c r="D112" s="13">
+        <v>302</v>
+      </c>
+      <c r="E112" s="20">
+        <v>301.64999999999998</v>
+      </c>
+      <c r="F112" s="16">
+        <v>141</v>
+      </c>
+      <c r="G112" s="4">
+        <v>299.5</v>
+      </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B113" s="8"/>
-      <c r="C113" s="10"/>
-      <c r="D113" s="13"/>
-      <c r="E113" s="5"/>
-      <c r="F113" s="16"/>
-      <c r="G113" s="4"/>
+      <c r="B113" s="8">
+        <v>146</v>
+      </c>
+      <c r="C113" s="10">
+        <v>141.74</v>
+      </c>
+      <c r="D113" s="13">
+        <v>145</v>
+      </c>
+      <c r="E113" s="20">
+        <v>144.91</v>
+      </c>
+      <c r="F113" s="16">
+        <v>9</v>
+      </c>
+      <c r="G113" s="4">
+        <v>143.59</v>
+      </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B114" s="8"/>
-      <c r="C114" s="10"/>
-      <c r="D114" s="13"/>
-      <c r="E114" s="5"/>
-      <c r="F114" s="16"/>
-      <c r="G114" s="4"/>
+      <c r="B114" s="8">
+        <v>933</v>
+      </c>
+      <c r="C114" s="10">
+        <v>910.75</v>
+      </c>
+      <c r="D114" s="13">
+        <v>914.4</v>
+      </c>
+      <c r="E114" s="20">
+        <v>917.5</v>
+      </c>
+      <c r="F114" s="16">
+        <v>2</v>
+      </c>
+      <c r="G114" s="4">
+        <v>925</v>
+      </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B115" s="8"/>
-      <c r="C115" s="10"/>
-      <c r="D115" s="13"/>
-      <c r="E115" s="5"/>
-      <c r="F115" s="16"/>
-      <c r="G115" s="4"/>
+      <c r="B115" s="8">
+        <v>166.6</v>
+      </c>
+      <c r="C115" s="10">
+        <v>162.66</v>
+      </c>
+      <c r="D115" s="13">
+        <v>165.18</v>
+      </c>
+      <c r="E115" s="20">
+        <v>164.77</v>
+      </c>
+      <c r="F115" s="16">
+        <v>87</v>
+      </c>
+      <c r="G115" s="4">
+        <v>163.44999999999999</v>
+      </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B116" s="8"/>
-      <c r="C116" s="10"/>
-      <c r="D116" s="13"/>
-      <c r="E116" s="5"/>
-      <c r="F116" s="16"/>
-      <c r="G116" s="4"/>
+      <c r="B116" s="8">
+        <v>454.65</v>
+      </c>
+      <c r="C116" s="10">
+        <v>444.75</v>
+      </c>
+      <c r="D116" s="13">
+        <v>452.1</v>
+      </c>
+      <c r="E116" s="20">
+        <v>449.85</v>
+      </c>
+      <c r="F116" s="16">
+        <v>72</v>
+      </c>
+      <c r="G116" s="4">
+        <v>449.2</v>
+      </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B117" s="8"/>
-      <c r="C117" s="10"/>
-      <c r="D117" s="13"/>
-      <c r="E117" s="5"/>
-      <c r="F117" s="16"/>
-      <c r="G117" s="4"/>
+      <c r="B117" s="8">
+        <v>782</v>
+      </c>
+      <c r="C117" s="10">
+        <v>772.05</v>
+      </c>
+      <c r="D117" s="13">
+        <v>780.4</v>
+      </c>
+      <c r="E117" s="20">
+        <v>778.2</v>
+      </c>
+      <c r="F117" s="16">
+        <v>12</v>
+      </c>
+      <c r="G117" s="4">
+        <v>776.85</v>
+      </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B118" s="8"/>
-      <c r="C118" s="10"/>
-      <c r="D118" s="13"/>
-      <c r="E118" s="5"/>
-      <c r="F118" s="16"/>
-      <c r="G118" s="4"/>
+      <c r="B118" s="8">
+        <v>1490</v>
+      </c>
+      <c r="C118" s="10">
+        <v>1467</v>
+      </c>
+      <c r="D118" s="13">
+        <v>1485</v>
+      </c>
+      <c r="E118" s="20">
+        <v>1483.6</v>
+      </c>
+      <c r="F118" s="16">
+        <v>8</v>
+      </c>
+      <c r="G118" s="4">
+        <v>1480.1</v>
+      </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B119" s="8"/>
-      <c r="C119" s="10"/>
-      <c r="D119" s="13"/>
-      <c r="E119" s="5"/>
-      <c r="F119" s="16"/>
-      <c r="G119" s="4"/>
+      <c r="B119" s="8">
+        <v>6100</v>
+      </c>
+      <c r="C119" s="10">
+        <v>5944.7</v>
+      </c>
+      <c r="D119" s="13">
+        <v>6080</v>
+      </c>
+      <c r="E119" s="20">
+        <v>6073.35</v>
+      </c>
+      <c r="F119" s="16">
+        <v>4</v>
+      </c>
+      <c r="G119" s="4">
+        <v>5978.2</v>
+      </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B120" s="8"/>
-      <c r="C120" s="10"/>
-      <c r="D120" s="13"/>
-      <c r="E120" s="5"/>
-      <c r="F120" s="16"/>
-      <c r="G120" s="4"/>
+      <c r="B120" s="8">
+        <v>2884.45</v>
+      </c>
+      <c r="C120" s="10">
+        <v>2782</v>
+      </c>
+      <c r="D120" s="13">
+        <v>2822.9</v>
+      </c>
+      <c r="E120" s="20">
+        <v>2809.85</v>
+      </c>
+      <c r="F120" s="16">
+        <v>16</v>
+      </c>
+      <c r="G120" s="4">
+        <v>2852.05</v>
+      </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B121" s="8"/>
-      <c r="C121" s="10"/>
-      <c r="D121" s="13"/>
-      <c r="E121" s="5"/>
-      <c r="F121" s="16"/>
-      <c r="G121" s="4"/>
+      <c r="B121" s="8">
+        <v>215.9</v>
+      </c>
+      <c r="C121" s="10">
+        <v>208.92</v>
+      </c>
+      <c r="D121" s="13">
+        <v>685</v>
+      </c>
+      <c r="E121" s="20">
+        <v>685.5</v>
+      </c>
+      <c r="F121" s="16">
+        <v>4</v>
+      </c>
+      <c r="G121" s="4">
+        <v>209.05</v>
+      </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B122" s="8"/>
-      <c r="C122" s="10"/>
-      <c r="D122" s="13"/>
-      <c r="E122" s="5"/>
-      <c r="F122" s="16"/>
-      <c r="G122" s="4"/>
+      <c r="B122" s="8">
+        <v>1769.85</v>
+      </c>
+      <c r="C122" s="10">
+        <v>1706.05</v>
+      </c>
+      <c r="D122" s="13">
+        <v>1752.85</v>
+      </c>
+      <c r="E122" s="20">
+        <v>1743.95</v>
+      </c>
+      <c r="F122" s="16">
+        <v>42</v>
+      </c>
+      <c r="G122" s="4">
+        <v>1745.35</v>
+      </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B123" s="8"/>
-      <c r="C123" s="10"/>
-      <c r="D123" s="13"/>
-      <c r="E123" s="5"/>
-      <c r="F123" s="16"/>
-      <c r="G123" s="4"/>
+      <c r="B123" s="8">
+        <v>765.85</v>
+      </c>
+      <c r="C123" s="10">
+        <v>739.05</v>
+      </c>
+      <c r="D123" s="13">
+        <v>745.35</v>
+      </c>
+      <c r="E123" s="20">
+        <v>746.65</v>
+      </c>
+      <c r="F123" s="16">
+        <v>6</v>
+      </c>
+      <c r="G123" s="4">
+        <v>760.65</v>
+      </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B124" s="8"/>
-      <c r="C124" s="10"/>
-      <c r="D124" s="13"/>
-      <c r="E124" s="5"/>
-      <c r="F124" s="16"/>
-      <c r="G124" s="4"/>
+      <c r="B124" s="8">
+        <v>1638.75</v>
+      </c>
+      <c r="C124" s="10">
+        <v>1584.3</v>
+      </c>
+      <c r="D124" s="13">
+        <v>1631.85</v>
+      </c>
+      <c r="E124" s="20">
+        <v>1633</v>
+      </c>
+      <c r="F124" s="16">
+        <v>2</v>
+      </c>
+      <c r="G124" s="4">
+        <v>1588.35</v>
+      </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B125" s="8"/>
-      <c r="C125" s="10"/>
-      <c r="D125" s="13"/>
-      <c r="E125" s="5"/>
-      <c r="F125" s="16"/>
-      <c r="G125" s="4"/>
+      <c r="B125" s="8">
+        <v>717</v>
+      </c>
+      <c r="C125" s="10">
+        <v>699.55</v>
+      </c>
+      <c r="D125" s="13">
+        <v>715.7</v>
+      </c>
+      <c r="E125" s="20">
+        <v>716.1</v>
+      </c>
+      <c r="F125" s="16">
+        <v>191</v>
+      </c>
+      <c r="G125" s="4">
+        <v>703.65</v>
+      </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B126" s="8"/>
-      <c r="C126" s="10"/>
-      <c r="D126" s="13"/>
-      <c r="E126" s="5"/>
-      <c r="F126" s="16"/>
-      <c r="G126" s="4"/>
+      <c r="B126" s="8">
+        <v>4128.45</v>
+      </c>
+      <c r="C126" s="10">
+        <v>4085.25</v>
+      </c>
+      <c r="D126" s="13">
+        <v>4114.1499999999996</v>
+      </c>
+      <c r="E126" s="20">
+        <v>4112.3999999999996</v>
+      </c>
+      <c r="F126" s="16">
+        <v>14</v>
+      </c>
+      <c r="G126" s="4">
+        <v>4112.45</v>
+      </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B127" s="8"/>
-      <c r="C127" s="10"/>
-      <c r="D127" s="13"/>
-      <c r="E127" s="5"/>
-      <c r="F127" s="16"/>
-      <c r="G127" s="4"/>
+      <c r="B127" s="8">
+        <v>1695</v>
+      </c>
+      <c r="C127" s="10">
+        <v>1665.25</v>
+      </c>
+      <c r="D127" s="13">
+        <v>1675.8</v>
+      </c>
+      <c r="E127" s="20">
+        <v>1674.45</v>
+      </c>
+      <c r="F127" s="16">
+        <v>10</v>
+      </c>
+      <c r="G127" s="4">
+        <v>1680.7</v>
+      </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B128" s="8"/>
-      <c r="C128" s="10"/>
-      <c r="D128" s="13"/>
-      <c r="E128" s="5"/>
-      <c r="F128" s="16"/>
-      <c r="G128" s="4"/>
+      <c r="B128" s="8">
+        <v>3527.45</v>
+      </c>
+      <c r="C128" s="10">
+        <v>3440.5</v>
+      </c>
+      <c r="D128" s="13">
+        <v>3491.3</v>
+      </c>
+      <c r="E128" s="20">
+        <v>3490.25</v>
+      </c>
+      <c r="F128" s="16">
+        <v>12</v>
+      </c>
+      <c r="G128" s="4">
+        <v>3464</v>
+      </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="B129" s="8"/>
-      <c r="C129" s="10"/>
-      <c r="D129" s="13"/>
-      <c r="E129" s="5"/>
-      <c r="F129" s="16"/>
-      <c r="G129" s="4"/>
+      <c r="B129" s="8">
+        <v>3363.1</v>
+      </c>
+      <c r="C129" s="10">
+        <v>3251.55</v>
+      </c>
+      <c r="D129" s="13">
+        <v>3273</v>
+      </c>
+      <c r="E129" s="20">
+        <v>3269.1</v>
+      </c>
+      <c r="F129" s="16">
+        <v>4</v>
+      </c>
+      <c r="G129" s="4">
+        <v>3341.35</v>
+      </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B130" s="8"/>
-      <c r="C130" s="10"/>
-      <c r="D130" s="13"/>
-      <c r="E130" s="5"/>
-      <c r="F130" s="16"/>
-      <c r="G130" s="4"/>
+      <c r="B130" s="8">
+        <v>1485.7</v>
+      </c>
+      <c r="C130" s="10">
+        <v>1442.45</v>
+      </c>
+      <c r="D130" s="13">
+        <v>1463</v>
+      </c>
+      <c r="E130" s="20">
+        <v>1463.45</v>
+      </c>
+      <c r="F130" s="16">
+        <v>4</v>
+      </c>
+      <c r="G130" s="4">
+        <v>1482</v>
+      </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B131" s="8"/>
-      <c r="C131" s="10"/>
-      <c r="D131" s="13"/>
-      <c r="E131" s="5"/>
-      <c r="F131" s="16"/>
-      <c r="G131" s="4"/>
+      <c r="B131" s="8">
+        <v>5817.65</v>
+      </c>
+      <c r="C131" s="10">
+        <v>5629</v>
+      </c>
+      <c r="D131" s="13">
+        <v>5765</v>
+      </c>
+      <c r="E131" s="20">
+        <v>5753.2</v>
+      </c>
+      <c r="F131" s="16">
+        <v>10</v>
+      </c>
+      <c r="G131" s="4">
+        <v>5668.55</v>
+      </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="B132" s="8"/>
-      <c r="C132" s="10"/>
-      <c r="D132" s="13"/>
-      <c r="E132" s="5"/>
-      <c r="F132" s="16"/>
-      <c r="G132" s="4"/>
+      <c r="B132" s="8">
+        <v>2492.5</v>
+      </c>
+      <c r="C132" s="10">
+        <v>2440.5500000000002</v>
+      </c>
+      <c r="D132" s="13">
+        <v>2454.75</v>
+      </c>
+      <c r="E132" s="20">
+        <v>2457.9</v>
+      </c>
+      <c r="F132" s="16">
+        <v>6</v>
+      </c>
+      <c r="G132" s="4">
+        <v>2458.9499999999998</v>
+      </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B133" s="8"/>
-      <c r="C133" s="10"/>
-      <c r="D133" s="13"/>
-      <c r="E133" s="5"/>
-      <c r="F133" s="16"/>
-      <c r="G133" s="4"/>
+      <c r="B133" s="8">
+        <v>2164.65</v>
+      </c>
+      <c r="C133" s="10">
+        <v>2115.6999999999998</v>
+      </c>
+      <c r="D133" s="13">
+        <v>2147.6</v>
+      </c>
+      <c r="E133" s="20">
+        <v>2146</v>
+      </c>
+      <c r="F133" s="16">
+        <v>2</v>
+      </c>
+      <c r="G133" s="4">
+        <v>2137.6999999999998</v>
+      </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="B134" s="8"/>
-      <c r="C134" s="10"/>
-      <c r="D134" s="13"/>
-      <c r="E134" s="5"/>
-      <c r="F134" s="16"/>
-      <c r="G134" s="4"/>
+      <c r="B134" s="8">
+        <v>11599</v>
+      </c>
+      <c r="C134" s="10">
+        <v>11414.45</v>
+      </c>
+      <c r="D134" s="13">
+        <v>11599</v>
+      </c>
+      <c r="E134" s="20">
+        <v>11487.45</v>
+      </c>
+      <c r="F134" s="16">
+        <v>3</v>
+      </c>
+      <c r="G134" s="4">
+        <v>11434</v>
+      </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="B135" s="8"/>
-      <c r="C135" s="10"/>
-      <c r="D135" s="13"/>
-      <c r="E135" s="5"/>
-      <c r="F135" s="16"/>
-      <c r="G135" s="4"/>
+      <c r="B135" s="8">
+        <v>617.79999999999995</v>
+      </c>
+      <c r="C135" s="10">
+        <v>567.75</v>
+      </c>
+      <c r="D135" s="13">
+        <v>604.9</v>
+      </c>
+      <c r="E135" s="20">
+        <v>603.75</v>
+      </c>
+      <c r="F135" s="16">
+        <v>86</v>
+      </c>
+      <c r="G135" s="4">
+        <v>570.6</v>
+      </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B136" s="8"/>
-      <c r="C136" s="10"/>
-      <c r="D136" s="13"/>
-      <c r="E136" s="5"/>
-      <c r="F136" s="16"/>
-      <c r="G136" s="4"/>
+      <c r="B136" s="8">
+        <v>443.8</v>
+      </c>
+      <c r="C136" s="10">
+        <v>426.9</v>
+      </c>
+      <c r="D136" s="13">
+        <v>440.4</v>
+      </c>
+      <c r="E136" s="20">
+        <v>441.4</v>
+      </c>
+      <c r="F136" s="16">
+        <v>112</v>
+      </c>
+      <c r="G136" s="4">
+        <v>433.4</v>
+      </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B137" s="8"/>
-      <c r="C137" s="10"/>
-      <c r="D137" s="13"/>
-      <c r="E137" s="5"/>
-      <c r="F137" s="16"/>
-      <c r="G137" s="4"/>
+      <c r="B137" s="8">
+        <v>1283.5999999999999</v>
+      </c>
+      <c r="C137" s="10">
+        <v>1239.05</v>
+      </c>
+      <c r="D137" s="13">
+        <v>1261.8499999999999</v>
+      </c>
+      <c r="E137" s="20">
+        <v>1260.8499999999999</v>
+      </c>
+      <c r="F137" s="16">
+        <v>50</v>
+      </c>
+      <c r="G137" s="4">
+        <v>1265.4000000000001</v>
+      </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B138" s="8"/>
-      <c r="C138" s="10"/>
-      <c r="D138" s="13"/>
-      <c r="E138" s="5"/>
-      <c r="F138" s="16"/>
-      <c r="G138" s="4"/>
+      <c r="B138" s="8">
+        <v>106.45</v>
+      </c>
+      <c r="C138" s="10">
+        <v>104.65</v>
+      </c>
+      <c r="D138" s="13">
+        <v>105.65</v>
+      </c>
+      <c r="E138" s="20">
+        <v>105.59</v>
+      </c>
+      <c r="F138" s="16">
+        <v>93</v>
+      </c>
+      <c r="G138" s="4">
+        <v>104.87</v>
+      </c>
     </row>
     <row r="139" spans="1:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="B139" s="18"/>
-      <c r="C139" s="11"/>
-      <c r="D139" s="14"/>
-      <c r="E139" s="6"/>
-      <c r="F139" s="17"/>
-      <c r="G139" s="4"/>
+      <c r="B139" s="18">
+        <v>975</v>
+      </c>
+      <c r="C139" s="11">
+        <v>957.15</v>
+      </c>
+      <c r="D139" s="14">
+        <v>970</v>
+      </c>
+      <c r="E139" s="21">
+        <v>970.25</v>
+      </c>
+      <c r="F139" s="17">
+        <v>11</v>
+      </c>
+      <c r="G139" s="4">
+        <v>957.15</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
updated cash and algo xpath
</commit_message>
<xml_diff>
--- a/algo high low.xlsx
+++ b/algo high low.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -681,22 +681,22 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>361.95</v>
+        <v>492.25</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>354.2</v>
+        <v>482.4</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>357.85</v>
+        <v>0</v>
       </c>
       <c r="E2" s="19" t="n">
-        <v>357.75</v>
+        <v>0</v>
       </c>
       <c r="F2" s="15" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>360.65</v>
+        <v>484.15</v>
       </c>
     </row>
     <row r="3">
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>5078.9</v>
+        <v>5895</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>4970</v>
+        <v>5824</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>5040</v>
+        <v>0</v>
       </c>
       <c r="E3" s="20" t="n">
-        <v>5036.2</v>
+        <v>0</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>5015.35</v>
+        <v>5885</v>
       </c>
     </row>
     <row r="4">
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>185.49</v>
+        <v>218.6</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>180.4</v>
+        <v>213.98</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>181.81</v>
+        <v>0</v>
       </c>
       <c r="E4" s="20" t="n">
-        <v>181.95</v>
+        <v>0</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>183.46</v>
+        <v>217.96</v>
       </c>
     </row>
     <row r="5">
@@ -756,22 +756,22 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>248.75</v>
+        <v>295.7</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>242.1</v>
+        <v>278.65</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>245.6</v>
+        <v>0</v>
       </c>
       <c r="E5" s="20" t="n">
-        <v>246.3</v>
+        <v>0</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>14</v>
+        <v>115</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>247.25</v>
+        <v>280.85</v>
       </c>
     </row>
     <row r="6">
@@ -781,22 +781,22 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>2266.15</v>
+        <v>2578.8</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>2215.2</v>
+        <v>2536</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>2243.45</v>
+        <v>0</v>
       </c>
       <c r="E6" s="20" t="n">
-        <v>2236.9</v>
+        <v>0</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2261</v>
+        <v>2566.8</v>
       </c>
     </row>
     <row r="7">
@@ -806,22 +806,22 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1135.6</v>
+        <v>1409.1</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>1112</v>
+        <v>1392</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>1135</v>
+        <v>0</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>1131.8</v>
+        <v>0</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1122.65</v>
+        <v>1406.2</v>
       </c>
     </row>
     <row r="8">
@@ -831,22 +831,22 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>4852.5</v>
+        <v>5400</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>4787.4</v>
+        <v>5200.5</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>4837.5</v>
+        <v>0</v>
       </c>
       <c r="E8" s="20" t="n">
-        <v>4838.85</v>
+        <v>0</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>4796.35</v>
+        <v>5213</v>
       </c>
     </row>
     <row r="9">
@@ -856,22 +856,22 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>552.3</v>
+        <v>569.55</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>531.15</v>
+        <v>559.35</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>542.65</v>
+        <v>0</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>547.8</v>
+        <v>0</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>533.6</v>
+        <v>562.75</v>
       </c>
     </row>
     <row r="10">
@@ -881,22 +881,22 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>6851.45</v>
+        <v>7061</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>6729.3</v>
+        <v>6965.5</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>6840.85</v>
+        <v>0</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>6834.1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>6751.45</v>
+        <v>7029</v>
       </c>
     </row>
     <row r="11">
@@ -906,22 +906,22 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>409.3</v>
+        <v>498.3</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>395.65</v>
+        <v>487.65</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>409.25</v>
+        <v>0</v>
       </c>
       <c r="E11" s="20" t="n">
-        <v>407.8</v>
+        <v>0</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>397.1</v>
+        <v>495.8</v>
       </c>
     </row>
     <row r="12">
@@ -931,22 +931,22 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>205.85</v>
+        <v>243.25</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>199.5</v>
+        <v>237.01</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>204.5</v>
+        <v>0</v>
       </c>
       <c r="E12" s="20" t="n">
-        <v>204.68</v>
+        <v>0</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>201.06</v>
+        <v>237.65</v>
       </c>
     </row>
     <row r="13">
@@ -956,22 +956,22 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>1273.6</v>
+        <v>1428.9</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>1252.4</v>
+        <v>1362.6</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>1264.55</v>
+        <v>0</v>
       </c>
       <c r="E13" s="20" t="n">
-        <v>1265.9</v>
+        <v>0</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>1263</v>
+        <v>1372.6</v>
       </c>
     </row>
     <row r="14">
@@ -981,22 +981,22 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>5389.8</v>
+        <v>6912</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>5101</v>
+        <v>6750.5</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>5199.5</v>
+        <v>0</v>
       </c>
       <c r="E14" s="20" t="n">
-        <v>5196.6</v>
+        <v>0</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>5304.35</v>
+        <v>6771</v>
       </c>
     </row>
     <row r="15">
@@ -1006,22 +1006,22 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>557.85</v>
+        <v>690.5</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>540.95</v>
+        <v>683.65</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>554</v>
+        <v>0</v>
       </c>
       <c r="E15" s="20" t="n">
-        <v>554.3</v>
+        <v>0</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>545.25</v>
+        <v>689.95</v>
       </c>
     </row>
     <row r="16">
@@ -1031,22 +1031,22 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>1076.5</v>
+        <v>1225.9</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>1046.3</v>
+        <v>1201.4</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1055</v>
+        <v>0</v>
       </c>
       <c r="E16" s="20" t="n">
-        <v>1058</v>
+        <v>0</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>1068.6</v>
+        <v>1205.9</v>
       </c>
     </row>
     <row r="17">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>7631.3</v>
+        <v>8861.5</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>7460.5</v>
+        <v>8615</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>7576.45</v>
+        <v>0</v>
       </c>
       <c r="E17" s="20" t="n">
-        <v>7572.3</v>
+        <v>0</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7516.55</v>
+        <v>8630</v>
       </c>
     </row>
     <row r="18">
@@ -1081,22 +1081,22 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>1918.3</v>
+        <v>2053</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>1878</v>
+        <v>2035.5</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1900</v>
+        <v>0</v>
       </c>
       <c r="E18" s="20" t="n">
-        <v>1895.7</v>
+        <v>0</v>
       </c>
       <c r="F18" s="16" t="n">
         <v>13</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>1902.55</v>
+        <v>2046.9</v>
       </c>
     </row>
     <row r="19">
@@ -1106,22 +1106,22 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>8842</v>
+        <v>9275</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>8625</v>
+        <v>9211</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>8745</v>
+        <v>0</v>
       </c>
       <c r="E19" s="20" t="n">
-        <v>8735.799999999999</v>
+        <v>0</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>8761.4</v>
+        <v>9244.5</v>
       </c>
     </row>
     <row r="20">
@@ -1131,22 +1131,22 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>2307.3</v>
+        <v>2764</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>2231.55</v>
+        <v>2681</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>2280.05</v>
+        <v>0</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>2280.6</v>
+        <v>0</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>2298.95</v>
+        <v>2727.5</v>
       </c>
     </row>
     <row r="21">
@@ -1156,22 +1156,22 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>526.5</v>
+        <v>573.25</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>511.55</v>
+        <v>550.1</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>521</v>
+        <v>0</v>
       </c>
       <c r="E21" s="20" t="n">
-        <v>520.65</v>
+        <v>0</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>525.45</v>
+        <v>558.1</v>
       </c>
     </row>
     <row r="22">
@@ -1181,22 +1181,22 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>148.77</v>
+        <v>173.2</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>143.28</v>
+        <v>169.94</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>146.8</v>
+        <v>0</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>146.86</v>
+        <v>0</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>148.47</v>
+        <v>171.28</v>
       </c>
     </row>
     <row r="23">
@@ -1206,22 +1206,22 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>235</v>
+        <v>242.8</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>229.05</v>
+        <v>236.2</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="E23" s="20" t="n">
-        <v>230.21</v>
+        <v>0</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>234.85</v>
+        <v>236.75</v>
       </c>
     </row>
     <row r="24">
@@ -1231,22 +1231,22 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>1236.9</v>
+        <v>1258.5</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>1201.75</v>
+        <v>1240.3</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>1229.95</v>
+        <v>0</v>
       </c>
       <c r="E24" s="20" t="n">
-        <v>1227.75</v>
+        <v>0</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>1209.65</v>
+        <v>1254.4</v>
       </c>
     </row>
     <row r="25">
@@ -1256,22 +1256,22 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>282.8</v>
+        <v>373.5</v>
       </c>
       <c r="C25" s="10" t="n">
-        <v>276.6</v>
+        <v>362.55</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>281</v>
+        <v>0</v>
       </c>
       <c r="E25" s="20" t="n">
-        <v>280.15</v>
+        <v>0</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>113</v>
+        <v>520</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>278.15</v>
+        <v>371.5</v>
       </c>
     </row>
     <row r="26">
@@ -1281,22 +1281,22 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>972.7</v>
+        <v>1279</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>940.75</v>
+        <v>1251.6</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>969</v>
+        <v>0</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>969.85</v>
+        <v>0</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>945.45</v>
+        <v>1275.9</v>
       </c>
     </row>
     <row r="27">
@@ -1306,22 +1306,22 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>214.2</v>
+        <v>252.25</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>205.19</v>
+        <v>243.2</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>211.95</v>
+        <v>0</v>
       </c>
       <c r="E27" s="20" t="n">
-        <v>211.81</v>
+        <v>0</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>101</v>
+        <v>157</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>206.8</v>
+        <v>252.07</v>
       </c>
     </row>
     <row r="28">
@@ -1331,22 +1331,22 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>313.3</v>
+        <v>345.15</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>305</v>
+        <v>338.5</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>305.6</v>
+        <v>0</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>306.3</v>
+        <v>0</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>313.2</v>
+        <v>341.8</v>
       </c>
     </row>
     <row r="29">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>5352.1</v>
+        <v>5547.5</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>5210</v>
+        <v>5470.5</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>5330</v>
+        <v>0</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>5339.45</v>
+        <v>0</v>
       </c>
       <c r="F29" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>5226.7</v>
+        <v>5505.5</v>
       </c>
     </row>
     <row r="30">
@@ -1381,22 +1381,22 @@
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>360.5</v>
+        <v>434</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>346.9</v>
+        <v>423.8</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>355.85</v>
+        <v>0</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>356.7</v>
+        <v>0</v>
       </c>
       <c r="F30" s="16" t="n">
         <v>11</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>350.25</v>
+        <v>431.3</v>
       </c>
     </row>
     <row r="31">
@@ -1406,22 +1406,22 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>89.5</v>
+        <v>109.5</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>87.15000000000001</v>
+        <v>107.76</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>88.34999999999999</v>
+        <v>0</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>88.42</v>
+        <v>0</v>
       </c>
       <c r="F31" s="16" t="n">
-        <v>218</v>
+        <v>261</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>88.90000000000001</v>
+        <v>108.2</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>662.25</v>
+        <v>754.3</v>
       </c>
       <c r="C32" s="10" t="n">
-        <v>652.25</v>
+        <v>736</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>655</v>
+        <v>0</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>656.85</v>
+        <v>0</v>
       </c>
       <c r="F32" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>659.8</v>
+        <v>747.4</v>
       </c>
     </row>
     <row r="33">
@@ -1456,22 +1456,22 @@
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>642.5</v>
+        <v>631.9</v>
       </c>
       <c r="C33" s="10" t="n">
-        <v>622.3</v>
+        <v>619.45</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>636</v>
+        <v>0</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>638.05</v>
+        <v>0</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>634.6</v>
+        <v>630.4</v>
       </c>
     </row>
     <row r="34">
@@ -1481,22 +1481,22 @@
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>1464.8</v>
+        <v>1639.5</v>
       </c>
       <c r="C34" s="10" t="n">
-        <v>1390</v>
+        <v>1619.6</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>1433.45</v>
+        <v>0</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>1430.6</v>
+        <v>0</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>1462.1</v>
+        <v>1629.5</v>
       </c>
     </row>
     <row r="35">
@@ -1506,22 +1506,22 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>1423</v>
+        <v>1511.7</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>1405.3</v>
+        <v>1489</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>1416</v>
+        <v>0</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>1415.6</v>
+        <v>0</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>1415.65</v>
+        <v>1496.5</v>
       </c>
     </row>
     <row r="36">
@@ -1531,22 +1531,22 @@
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>6363.9</v>
+        <v>8400</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>6175</v>
+        <v>8252.5</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>6290</v>
+        <v>0</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6323.65</v>
+        <v>0</v>
       </c>
       <c r="F36" s="16" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>6294.4</v>
+        <v>8367.5</v>
       </c>
     </row>
     <row r="37">
@@ -1556,22 +1556,22 @@
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>687.2</v>
+        <v>756.35</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>658.5</v>
+        <v>726.5</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>684.2</v>
+        <v>0</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>685.2</v>
+        <v>0</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>663.5</v>
+        <v>732.65</v>
       </c>
     </row>
     <row r="38">
@@ -1581,22 +1581,22 @@
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>2050</v>
+        <v>2509</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>1981.05</v>
+        <v>2420</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>2020.95</v>
+        <v>0</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>2004.7</v>
+        <v>0</v>
       </c>
       <c r="F38" s="16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>2044.75</v>
+        <v>2456.5</v>
       </c>
     </row>
     <row r="39">
@@ -1606,22 +1606,22 @@
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>333.6</v>
+        <v>362.75</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>325.6</v>
+        <v>349.1</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>328.85</v>
+        <v>0</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>328.8</v>
+        <v>0</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>331.35</v>
+        <v>362.25</v>
       </c>
     </row>
     <row r="40">
@@ -1631,22 +1631,22 @@
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>2789.65</v>
+        <v>3062.2</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>2690</v>
+        <v>2981.3</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>2767.05</v>
+        <v>0</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>2781.45</v>
+        <v>0</v>
       </c>
       <c r="F40" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>2716.75</v>
+        <v>3052.7</v>
       </c>
     </row>
     <row r="41">
@@ -1656,22 +1656,22 @@
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>468.45</v>
+        <v>484.5</v>
       </c>
       <c r="C41" s="10" t="n">
-        <v>461</v>
+        <v>478.65</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>465</v>
+        <v>0</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>465.25</v>
+        <v>0</v>
       </c>
       <c r="F41" s="16" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>462.15</v>
+        <v>479.4</v>
       </c>
     </row>
     <row r="42">
@@ -1681,22 +1681,22 @@
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>1835</v>
+        <v>2096</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>1776.85</v>
+        <v>2061.3</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>1825</v>
+        <v>0</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>1825.9</v>
+        <v>0</v>
       </c>
       <c r="F42" s="16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>1804</v>
+        <v>2084.1</v>
       </c>
     </row>
     <row r="43">
@@ -1706,22 +1706,22 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>1164.4</v>
+        <v>1390</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>1100</v>
+        <v>1340.8</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>1149</v>
+        <v>0</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>1158.6</v>
+        <v>0</v>
       </c>
       <c r="F43" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>1108.1</v>
+        <v>1366.2</v>
       </c>
     </row>
     <row r="44">
@@ -1731,22 +1731,22 @@
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>1821.15</v>
+        <v>2174</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>1785.95</v>
+        <v>2113.4</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>1806.5</v>
+        <v>0</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>1807.35</v>
+        <v>0</v>
       </c>
       <c r="F44" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>1817.85</v>
+        <v>2149.9</v>
       </c>
     </row>
     <row r="45">
@@ -1756,22 +1756,22 @@
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>79.15000000000001</v>
+        <v>95.75</v>
       </c>
       <c r="C45" s="10" t="n">
-        <v>78.09999999999999</v>
+        <v>93.33</v>
       </c>
       <c r="D45" s="13" t="n">
-        <v>78.97</v>
+        <v>0</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>78.95999999999999</v>
+        <v>0</v>
       </c>
       <c r="F45" s="16" t="n">
         <v>12</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>78.92</v>
+        <v>94.78</v>
       </c>
     </row>
     <row r="46">
@@ -1781,22 +1781,22 @@
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>5429.6</v>
+        <v>6705</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>5319</v>
+        <v>6415</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>5408.9</v>
+        <v>0</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>5386.15</v>
+        <v>0</v>
       </c>
       <c r="F46" s="16" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>5335.15</v>
+        <v>6462</v>
       </c>
     </row>
     <row r="47">
@@ -1806,22 +1806,22 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>13313.9</v>
+        <v>16727</v>
       </c>
       <c r="C47" s="10" t="n">
-        <v>12755</v>
+        <v>16420</v>
       </c>
       <c r="D47" s="13" t="n">
-        <v>13251.05</v>
+        <v>0</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>13282.45</v>
+        <v>0</v>
       </c>
       <c r="F47" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>13035</v>
+        <v>16674</v>
       </c>
     </row>
     <row r="48">
@@ -1831,22 +1831,22 @@
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>621.25</v>
+        <v>739</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>607.05</v>
+        <v>722.35</v>
       </c>
       <c r="D48" s="13" t="n">
-        <v>613</v>
+        <v>0</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>612.85</v>
+        <v>0</v>
       </c>
       <c r="F48" s="16" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>618.5</v>
+        <v>724.45</v>
       </c>
     </row>
     <row r="49">
@@ -1856,22 +1856,22 @@
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>1103.25</v>
+        <v>1241.8</v>
       </c>
       <c r="C49" s="10" t="n">
-        <v>1076.15</v>
+        <v>1214.2</v>
       </c>
       <c r="D49" s="13" t="n">
-        <v>1093.25</v>
+        <v>0</v>
       </c>
       <c r="E49" s="20" t="n">
-        <v>1094.05</v>
+        <v>0</v>
       </c>
       <c r="F49" s="16" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>1086.4</v>
+        <v>1227.5</v>
       </c>
     </row>
     <row r="50">
@@ -1881,22 +1881,22 @@
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>3170</v>
+        <v>3556.4</v>
       </c>
       <c r="C50" s="10" t="n">
-        <v>3092</v>
+        <v>3508.1</v>
       </c>
       <c r="D50" s="13" t="n">
-        <v>3126</v>
+        <v>0</v>
       </c>
       <c r="E50" s="20" t="n">
-        <v>3128.75</v>
+        <v>0</v>
       </c>
       <c r="F50" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>3097.2</v>
+        <v>3545.9</v>
       </c>
     </row>
     <row r="51">
@@ -1906,22 +1906,22 @@
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>366.9</v>
+        <v>396.65</v>
       </c>
       <c r="C51" s="10" t="n">
-        <v>352.35</v>
+        <v>390.65</v>
       </c>
       <c r="D51" s="13" t="n">
-        <v>364</v>
+        <v>0</v>
       </c>
       <c r="E51" s="20" t="n">
-        <v>364.35</v>
+        <v>0</v>
       </c>
       <c r="F51" s="16" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>354.2</v>
+        <v>396.25</v>
       </c>
     </row>
     <row r="52">
@@ -1931,22 +1931,22 @@
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>1428.65</v>
+        <v>1471.1</v>
       </c>
       <c r="C52" s="10" t="n">
-        <v>1339.9</v>
+        <v>1425</v>
       </c>
       <c r="D52" s="13" t="n">
-        <v>1375.95</v>
+        <v>0</v>
       </c>
       <c r="E52" s="20" t="n">
-        <v>1376.3</v>
+        <v>0</v>
       </c>
       <c r="F52" s="16" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>1420</v>
+        <v>1444.8</v>
       </c>
     </row>
     <row r="53">
@@ -1956,22 +1956,22 @@
         </is>
       </c>
       <c r="B53" s="8" t="n">
-        <v>989.05</v>
+        <v>1155.2</v>
       </c>
       <c r="C53" s="10" t="n">
-        <v>933.4</v>
+        <v>1115</v>
       </c>
       <c r="D53" s="13" t="n">
-        <v>938.05</v>
+        <v>0</v>
       </c>
       <c r="E53" s="20" t="n">
-        <v>940.95</v>
+        <v>0</v>
       </c>
       <c r="F53" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>984.45</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="54">
@@ -1981,22 +1981,22 @@
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>477.95</v>
+        <v>519.3</v>
       </c>
       <c r="C54" s="10" t="n">
-        <v>472.1</v>
+        <v>507.05</v>
       </c>
       <c r="D54" s="13" t="n">
-        <v>476.5</v>
+        <v>0</v>
       </c>
       <c r="E54" s="20" t="n">
-        <v>476.2</v>
+        <v>0</v>
       </c>
       <c r="F54" s="16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>475.6</v>
+        <v>517.75</v>
       </c>
     </row>
     <row r="55">
@@ -2006,22 +2006,22 @@
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>1249</v>
+        <v>1308.2</v>
       </c>
       <c r="C55" s="10" t="n">
-        <v>1199.4</v>
+        <v>1290</v>
       </c>
       <c r="D55" s="13" t="n">
-        <v>1238</v>
+        <v>0</v>
       </c>
       <c r="E55" s="20" t="n">
-        <v>1242.35</v>
+        <v>0</v>
       </c>
       <c r="F55" s="16" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>1204.15</v>
+        <v>1305.7</v>
       </c>
     </row>
     <row r="56">
@@ -2031,22 +2031,22 @@
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>1998</v>
+        <v>2269.1</v>
       </c>
       <c r="C56" s="10" t="n">
-        <v>1925.8</v>
+        <v>2176.1</v>
       </c>
       <c r="D56" s="13" t="n">
-        <v>1965.1</v>
+        <v>0</v>
       </c>
       <c r="E56" s="20" t="n">
-        <v>1973.3</v>
+        <v>0</v>
       </c>
       <c r="F56" s="16" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>1966.55</v>
+        <v>2181.5</v>
       </c>
     </row>
     <row r="57">
@@ -2056,22 +2056,22 @@
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>441.15</v>
+        <v>521.1</v>
       </c>
       <c r="C57" s="10" t="n">
-        <v>422</v>
+        <v>507.55</v>
       </c>
       <c r="D57" s="13" t="n">
-        <v>430</v>
+        <v>0</v>
       </c>
       <c r="E57" s="20" t="n">
-        <v>431.1</v>
+        <v>0</v>
       </c>
       <c r="F57" s="16" t="n">
         <v>10</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>436.3</v>
+        <v>513.2</v>
       </c>
     </row>
     <row r="58">
@@ -2081,22 +2081,22 @@
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>2583.3</v>
+        <v>2791.9</v>
       </c>
       <c r="C58" s="10" t="n">
-        <v>2529.45</v>
+        <v>2721</v>
       </c>
       <c r="D58" s="13" t="n">
-        <v>2568</v>
+        <v>0</v>
       </c>
       <c r="E58" s="20" t="n">
-        <v>2557.75</v>
+        <v>0</v>
       </c>
       <c r="F58" s="16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>2578.15</v>
+        <v>2788.2</v>
       </c>
     </row>
     <row r="59">
@@ -2106,22 +2106,22 @@
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>407.6</v>
+        <v>474.75</v>
       </c>
       <c r="C59" s="10" t="n">
-        <v>393.7</v>
+        <v>465.25</v>
       </c>
       <c r="D59" s="13" t="n">
-        <v>405.65</v>
+        <v>0</v>
       </c>
       <c r="E59" s="20" t="n">
-        <v>404.3</v>
+        <v>0</v>
       </c>
       <c r="F59" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>396.4</v>
+        <v>474.75</v>
       </c>
     </row>
     <row r="60">
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="B60" s="8" t="n">
-        <v>4070</v>
+        <v>5140.9</v>
       </c>
       <c r="C60" s="10" t="n">
-        <v>3965.85</v>
+        <v>4972</v>
       </c>
       <c r="D60" s="13" t="n">
-        <v>4040.1</v>
+        <v>0</v>
       </c>
       <c r="E60" s="20" t="n">
-        <v>4030.7</v>
+        <v>0</v>
       </c>
       <c r="F60" s="16" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>3994.85</v>
+        <v>5135.1</v>
       </c>
     </row>
     <row r="61">
@@ -2156,22 +2156,22 @@
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>1479.1</v>
+        <v>1600.8</v>
       </c>
       <c r="C61" s="10" t="n">
-        <v>1451.1</v>
+        <v>1579.2</v>
       </c>
       <c r="D61" s="13" t="n">
-        <v>1465.6</v>
+        <v>0</v>
       </c>
       <c r="E61" s="20" t="n">
-        <v>1469.7</v>
+        <v>0</v>
       </c>
       <c r="F61" s="16" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>1459.05</v>
+        <v>1593.9</v>
       </c>
     </row>
     <row r="62">
@@ -2181,22 +2181,22 @@
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>1388.7</v>
+        <v>1658</v>
       </c>
       <c r="C62" s="10" t="n">
-        <v>1365.75</v>
+        <v>1642.6</v>
       </c>
       <c r="D62" s="13" t="n">
-        <v>1380.7</v>
+        <v>0</v>
       </c>
       <c r="E62" s="20" t="n">
-        <v>1380</v>
+        <v>0</v>
       </c>
       <c r="F62" s="16" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>1374.4</v>
+        <v>1651.4</v>
       </c>
     </row>
     <row r="63">
@@ -2206,22 +2206,22 @@
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>3850</v>
+        <v>4845</v>
       </c>
       <c r="C63" s="10" t="n">
-        <v>3781.4</v>
+        <v>4800</v>
       </c>
       <c r="D63" s="13" t="n">
-        <v>3789.95</v>
+        <v>0</v>
       </c>
       <c r="E63" s="20" t="n">
-        <v>3799.95</v>
+        <v>0</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>3812.65</v>
+        <v>4812</v>
       </c>
     </row>
     <row r="64">
@@ -2231,22 +2231,22 @@
         </is>
       </c>
       <c r="B64" s="8" t="n">
-        <v>691.6</v>
+        <v>755.5</v>
       </c>
       <c r="C64" s="10" t="n">
-        <v>679.15</v>
+        <v>749</v>
       </c>
       <c r="D64" s="13" t="n">
-        <v>685.5</v>
+        <v>0</v>
       </c>
       <c r="E64" s="20" t="n">
-        <v>684.8</v>
+        <v>0</v>
       </c>
       <c r="F64" s="16" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>685</v>
+        <v>754.5</v>
       </c>
     </row>
     <row r="65">
@@ -2256,22 +2256,22 @@
         </is>
       </c>
       <c r="B65" s="8" t="n">
-        <v>566.65</v>
+        <v>661.75</v>
       </c>
       <c r="C65" s="10" t="n">
-        <v>552.2</v>
+        <v>652</v>
       </c>
       <c r="D65" s="13" t="n">
-        <v>564.25</v>
+        <v>0</v>
       </c>
       <c r="E65" s="20" t="n">
-        <v>564</v>
+        <v>0</v>
       </c>
       <c r="F65" s="16" t="n">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>555.6</v>
+        <v>655.05</v>
       </c>
     </row>
     <row r="66">
@@ -2281,22 +2281,22 @@
         </is>
       </c>
       <c r="B66" s="8" t="n">
-        <v>199.2</v>
+        <v>231.5</v>
       </c>
       <c r="C66" s="10" t="n">
-        <v>187.37</v>
+        <v>225.93</v>
       </c>
       <c r="D66" s="13" t="n">
-        <v>195.8</v>
+        <v>0</v>
       </c>
       <c r="E66" s="20" t="n">
-        <v>196.24</v>
+        <v>0</v>
       </c>
       <c r="F66" s="16" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>189</v>
+        <v>229.39</v>
       </c>
     </row>
     <row r="67">
@@ -2306,22 +2306,22 @@
         </is>
       </c>
       <c r="B67" s="8" t="n">
-        <v>1798.8</v>
+        <v>1901</v>
       </c>
       <c r="C67" s="10" t="n">
-        <v>1776.05</v>
+        <v>1844.4</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>1783.8</v>
+        <v>0</v>
       </c>
       <c r="E67" s="20" t="n">
-        <v>1786.5</v>
+        <v>0</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>1798.7</v>
+        <v>1854.3</v>
       </c>
     </row>
     <row r="68">
@@ -2331,22 +2331,22 @@
         </is>
       </c>
       <c r="B68" s="8" t="n">
-        <v>572</v>
+        <v>627.85</v>
       </c>
       <c r="C68" s="10" t="n">
-        <v>558.9</v>
+        <v>613.2</v>
       </c>
       <c r="D68" s="13" t="n">
-        <v>570.65</v>
+        <v>0</v>
       </c>
       <c r="E68" s="20" t="n">
-        <v>568.85</v>
+        <v>0</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>560.7</v>
+        <v>616.2</v>
       </c>
     </row>
     <row r="69">
@@ -2356,22 +2356,22 @@
         </is>
       </c>
       <c r="B69" s="8" t="n">
-        <v>179.51</v>
+        <v>202.39</v>
       </c>
       <c r="C69" s="10" t="n">
-        <v>173.45</v>
+        <v>197</v>
       </c>
       <c r="D69" s="13" t="n">
-        <v>177.1</v>
+        <v>0</v>
       </c>
       <c r="E69" s="20" t="n">
-        <v>177.4</v>
+        <v>0</v>
       </c>
       <c r="F69" s="16" t="n">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>175.25</v>
+        <v>201.44</v>
       </c>
     </row>
     <row r="70">
@@ -2381,22 +2381,22 @@
         </is>
       </c>
       <c r="B70" s="8" t="n">
-        <v>176.75</v>
+        <v>214.18</v>
       </c>
       <c r="C70" s="10" t="n">
-        <v>172.15</v>
+        <v>208.35</v>
       </c>
       <c r="D70" s="13" t="n">
-        <v>175.08</v>
+        <v>0</v>
       </c>
       <c r="E70" s="20" t="n">
-        <v>174.88</v>
+        <v>0</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>176.1</v>
+        <v>208.75</v>
       </c>
     </row>
     <row r="71">
@@ -2406,22 +2406,22 @@
         </is>
       </c>
       <c r="B71" s="8" t="n">
-        <v>777</v>
+        <v>781.75</v>
       </c>
       <c r="C71" s="10" t="n">
-        <v>754.25</v>
+        <v>769.2</v>
       </c>
       <c r="D71" s="13" t="n">
-        <v>768.95</v>
+        <v>0</v>
       </c>
       <c r="E71" s="20" t="n">
-        <v>768.2</v>
+        <v>0</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>762</v>
+        <v>775.3</v>
       </c>
     </row>
     <row r="72">
@@ -2431,22 +2431,22 @@
         </is>
       </c>
       <c r="B72" s="8" t="n">
-        <v>275.9</v>
+        <v>323.8</v>
       </c>
       <c r="C72" s="10" t="n">
-        <v>268</v>
+        <v>315.05</v>
       </c>
       <c r="D72" s="13" t="n">
-        <v>275.85</v>
+        <v>0</v>
       </c>
       <c r="E72" s="20" t="n">
-        <v>274.15</v>
+        <v>0</v>
       </c>
       <c r="F72" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>269.35</v>
+        <v>318</v>
       </c>
     </row>
     <row r="73">
@@ -2456,22 +2456,22 @@
         </is>
       </c>
       <c r="B73" s="8" t="n">
-        <v>2002.5</v>
+        <v>2389.8</v>
       </c>
       <c r="C73" s="10" t="n">
-        <v>1956.8</v>
+        <v>2340</v>
       </c>
       <c r="D73" s="13" t="n">
-        <v>1996</v>
+        <v>0</v>
       </c>
       <c r="E73" s="20" t="n">
-        <v>1993.8</v>
+        <v>0</v>
       </c>
       <c r="F73" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>1969.8</v>
+        <v>2343</v>
       </c>
     </row>
     <row r="74">
@@ -2481,22 +2481,22 @@
         </is>
       </c>
       <c r="B74" s="8" t="n">
-        <v>5265</v>
+        <v>5665.5</v>
       </c>
       <c r="C74" s="10" t="n">
-        <v>5155.5</v>
+        <v>5557.5</v>
       </c>
       <c r="D74" s="13" t="n">
-        <v>5194.9</v>
+        <v>0</v>
       </c>
       <c r="E74" s="20" t="n">
-        <v>5193.75</v>
+        <v>0</v>
       </c>
       <c r="F74" s="16" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>5157.65</v>
+        <v>5619</v>
       </c>
     </row>
     <row r="75">
@@ -2506,22 +2506,22 @@
         </is>
       </c>
       <c r="B75" s="8" t="n">
-        <v>682.05</v>
+        <v>791.95</v>
       </c>
       <c r="C75" s="10" t="n">
-        <v>670.25</v>
+        <v>771.45</v>
       </c>
       <c r="D75" s="13" t="n">
-        <v>678.3</v>
+        <v>0</v>
       </c>
       <c r="E75" s="20" t="n">
-        <v>678.55</v>
+        <v>0</v>
       </c>
       <c r="F75" s="16" t="n">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>677.55</v>
+        <v>776.5</v>
       </c>
     </row>
     <row r="76">
@@ -2531,22 +2531,22 @@
         </is>
       </c>
       <c r="B76" s="8" t="n">
-        <v>374.4</v>
+        <v>402.15</v>
       </c>
       <c r="C76" s="10" t="n">
-        <v>365.2</v>
+        <v>382</v>
       </c>
       <c r="D76" s="13" t="n">
-        <v>369.5</v>
+        <v>0</v>
       </c>
       <c r="E76" s="20" t="n">
-        <v>370.6</v>
+        <v>0</v>
       </c>
       <c r="F76" s="16" t="n">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>369.3</v>
+        <v>401.3</v>
       </c>
     </row>
     <row r="77">
@@ -2556,22 +2556,22 @@
         </is>
       </c>
       <c r="B77" s="8" t="n">
-        <v>630.75</v>
+        <v>1110</v>
       </c>
       <c r="C77" s="10" t="n">
-        <v>609</v>
+        <v>1045.55</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>613.7</v>
+        <v>0</v>
       </c>
       <c r="E77" s="20" t="n">
-        <v>612.35</v>
+        <v>0</v>
       </c>
       <c r="F77" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>629.35</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="78">
@@ -2581,22 +2581,22 @@
         </is>
       </c>
       <c r="B78" s="8" t="n">
-        <v>1322.7</v>
+        <v>1464.1</v>
       </c>
       <c r="C78" s="10" t="n">
-        <v>1270</v>
+        <v>1404.6</v>
       </c>
       <c r="D78" s="13" t="n">
-        <v>1290</v>
+        <v>0</v>
       </c>
       <c r="E78" s="20" t="n">
-        <v>1294.85</v>
+        <v>0</v>
       </c>
       <c r="F78" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>1319.55</v>
+        <v>1409.1</v>
       </c>
     </row>
     <row r="79">
@@ -2606,22 +2606,22 @@
         </is>
       </c>
       <c r="B79" s="8" t="n">
-        <v>790.25</v>
+        <v>979.65</v>
       </c>
       <c r="C79" s="10" t="n">
-        <v>770</v>
+        <v>955.25</v>
       </c>
       <c r="D79" s="13" t="n">
-        <v>787.7</v>
+        <v>0</v>
       </c>
       <c r="E79" s="20" t="n">
-        <v>786.9</v>
+        <v>0</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>780.8</v>
+        <v>972.2</v>
       </c>
     </row>
     <row r="80">
@@ -2631,22 +2631,22 @@
         </is>
       </c>
       <c r="B80" s="8" t="n">
-        <v>4938.35</v>
+        <v>5287.5</v>
       </c>
       <c r="C80" s="10" t="n">
-        <v>4826.65</v>
+        <v>5207</v>
       </c>
       <c r="D80" s="13" t="n">
-        <v>4890</v>
+        <v>0</v>
       </c>
       <c r="E80" s="20" t="n">
-        <v>4884.9</v>
+        <v>0</v>
       </c>
       <c r="F80" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>4870.15</v>
+        <v>5222.5</v>
       </c>
     </row>
     <row r="81">
@@ -2656,22 +2656,22 @@
         </is>
       </c>
       <c r="B81" s="8" t="n">
-        <v>953.4</v>
+        <v>1030.8</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>938.05</v>
+        <v>1016.7</v>
       </c>
       <c r="D81" s="13" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="E81" s="20" t="n">
-        <v>945.55</v>
+        <v>0</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>943.75</v>
+        <v>1023.5</v>
       </c>
     </row>
     <row r="82">
@@ -2681,22 +2681,22 @@
         </is>
       </c>
       <c r="B82" s="8" t="n">
-        <v>691.5</v>
+        <v>703</v>
       </c>
       <c r="C82" s="10" t="n">
-        <v>671.15</v>
+        <v>665.1</v>
       </c>
       <c r="D82" s="13" t="n">
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="E82" s="20" t="n">
-        <v>685.05</v>
+        <v>0</v>
       </c>
       <c r="F82" s="16" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>675.05</v>
+        <v>672.9</v>
       </c>
     </row>
     <row r="83">
@@ -2706,22 +2706,22 @@
         </is>
       </c>
       <c r="B83" s="8" t="n">
-        <v>2065</v>
+        <v>2124</v>
       </c>
       <c r="C83" s="10" t="n">
-        <v>2042.1</v>
+        <v>2105.3</v>
       </c>
       <c r="D83" s="13" t="n">
-        <v>2058</v>
+        <v>0</v>
       </c>
       <c r="E83" s="20" t="n">
-        <v>2052.7</v>
+        <v>0</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>2056.25</v>
+        <v>2116.9</v>
       </c>
     </row>
     <row r="84">
@@ -2731,22 +2731,22 @@
         </is>
       </c>
       <c r="B84" s="8" t="n">
-        <v>2686</v>
+        <v>2809.4</v>
       </c>
       <c r="C84" s="10" t="n">
-        <v>2520.05</v>
+        <v>2773.2</v>
       </c>
       <c r="D84" s="13" t="n">
-        <v>2650</v>
+        <v>0</v>
       </c>
       <c r="E84" s="20" t="n">
-        <v>2667.75</v>
+        <v>0</v>
       </c>
       <c r="F84" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G84" s="4" t="n">
-        <v>2528.15</v>
+        <v>2802</v>
       </c>
     </row>
     <row r="85">
@@ -2756,22 +2756,22 @@
         </is>
       </c>
       <c r="B85" s="8" t="n">
-        <v>575.2</v>
+        <v>620.35</v>
       </c>
       <c r="C85" s="10" t="n">
-        <v>551</v>
+        <v>604</v>
       </c>
       <c r="D85" s="13" t="n">
-        <v>563.55</v>
+        <v>0</v>
       </c>
       <c r="E85" s="20" t="n">
-        <v>564.25</v>
+        <v>0</v>
       </c>
       <c r="F85" s="16" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G85" s="4" t="n">
-        <v>563.3</v>
+        <v>607.45</v>
       </c>
     </row>
     <row r="86">
@@ -2781,22 +2781,22 @@
         </is>
       </c>
       <c r="B86" s="8" t="n">
-        <v>566.25</v>
+        <v>608.9</v>
       </c>
       <c r="C86" s="10" t="n">
-        <v>544.55</v>
+        <v>599</v>
       </c>
       <c r="D86" s="13" t="n">
-        <v>557</v>
+        <v>0</v>
       </c>
       <c r="E86" s="20" t="n">
-        <v>556.35</v>
+        <v>0</v>
       </c>
       <c r="F86" s="16" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>556.2</v>
+        <v>605.8</v>
       </c>
     </row>
     <row r="87">
@@ -2806,22 +2806,22 @@
         </is>
       </c>
       <c r="B87" s="8" t="n">
-        <v>4155</v>
+        <v>5079.4</v>
       </c>
       <c r="C87" s="10" t="n">
-        <v>4024.75</v>
+        <v>4981.8</v>
       </c>
       <c r="D87" s="13" t="n">
-        <v>4100.65</v>
+        <v>0</v>
       </c>
       <c r="E87" s="20" t="n">
-        <v>4107.85</v>
+        <v>0</v>
       </c>
       <c r="F87" s="16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G87" s="4" t="n">
-        <v>4079</v>
+        <v>5052.2</v>
       </c>
     </row>
     <row r="88">
@@ -2831,22 +2831,22 @@
         </is>
       </c>
       <c r="B88" s="8" t="n">
-        <v>4110.65</v>
+        <v>4555</v>
       </c>
       <c r="C88" s="10" t="n">
-        <v>3991</v>
+        <v>4475.1</v>
       </c>
       <c r="D88" s="13" t="n">
-        <v>4070</v>
+        <v>0</v>
       </c>
       <c r="E88" s="20" t="n">
-        <v>4089.55</v>
+        <v>0</v>
       </c>
       <c r="F88" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>4010.6</v>
+        <v>4512.6</v>
       </c>
     </row>
     <row r="89">
@@ -2856,22 +2856,22 @@
         </is>
       </c>
       <c r="B89" s="8" t="n">
-        <v>1939.25</v>
+        <v>2075.8</v>
       </c>
       <c r="C89" s="10" t="n">
-        <v>1908</v>
+        <v>2025.6</v>
       </c>
       <c r="D89" s="13" t="n">
-        <v>1919.6</v>
+        <v>0</v>
       </c>
       <c r="E89" s="20" t="n">
-        <v>1919.7</v>
+        <v>0</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>1935.4</v>
+        <v>2060.2</v>
       </c>
     </row>
     <row r="90">
@@ -2881,22 +2881,22 @@
         </is>
       </c>
       <c r="B90" s="8" t="n">
-        <v>259.75</v>
+        <v>268.9</v>
       </c>
       <c r="C90" s="10" t="n">
-        <v>251.25</v>
+        <v>264.15</v>
       </c>
       <c r="D90" s="13" t="n">
-        <v>258.6</v>
+        <v>0</v>
       </c>
       <c r="E90" s="20" t="n">
-        <v>257.6</v>
+        <v>0</v>
       </c>
       <c r="F90" s="16" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>258</v>
+        <v>267.2</v>
       </c>
     </row>
     <row r="91">
@@ -2906,22 +2906,22 @@
         </is>
       </c>
       <c r="B91" s="8" t="n">
-        <v>228.2</v>
+        <v>229.8</v>
       </c>
       <c r="C91" s="10" t="n">
-        <v>221.76</v>
+        <v>228.33</v>
       </c>
       <c r="D91" s="13" t="n">
-        <v>224.81</v>
+        <v>0</v>
       </c>
       <c r="E91" s="20" t="n">
-        <v>224.93</v>
+        <v>0</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>145</v>
+        <v>17</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>227.6</v>
+        <v>229.5</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1" thickBot="1">
@@ -2931,22 +2931,22 @@
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>698.4</v>
+        <v>726.8</v>
       </c>
       <c r="C92" s="10" t="n">
-        <v>677.15</v>
+        <v>713.55</v>
       </c>
       <c r="D92" s="13" t="n">
-        <v>692.25</v>
+        <v>0</v>
       </c>
       <c r="E92" s="22" t="n">
-        <v>693.45</v>
+        <v>0</v>
       </c>
       <c r="F92" s="16" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="G92" s="4" t="n">
-        <v>680.65</v>
+        <v>724.35</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1" thickBot="1">
@@ -2956,22 +2956,22 @@
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>1455.95</v>
+        <v>1567.7</v>
       </c>
       <c r="C93" s="10" t="n">
-        <v>1425.5</v>
+        <v>1539</v>
       </c>
       <c r="D93" s="13" t="n">
-        <v>1455</v>
+        <v>0</v>
       </c>
       <c r="E93" s="23" t="n">
-        <v>1451.6</v>
+        <v>0</v>
       </c>
       <c r="F93" s="16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G93" s="4" t="n">
-        <v>1437.4</v>
+        <v>1550.4</v>
       </c>
     </row>
     <row r="94">
@@ -2981,22 +2981,22 @@
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>5249.05</v>
+        <v>6558</v>
       </c>
       <c r="C94" s="10" t="n">
-        <v>5069.85</v>
+        <v>6345.5</v>
       </c>
       <c r="D94" s="13" t="n">
-        <v>5222.6</v>
+        <v>0</v>
       </c>
       <c r="E94" s="19" t="n">
-        <v>5221.05</v>
+        <v>0</v>
       </c>
       <c r="F94" s="16" t="n">
         <v>4</v>
       </c>
       <c r="G94" s="4" t="n">
-        <v>5193.75</v>
+        <v>6490</v>
       </c>
     </row>
     <row r="95">
@@ -3006,22 +3006,22 @@
         </is>
       </c>
       <c r="B95" s="8" t="n">
-        <v>1599.8</v>
+        <v>1665</v>
       </c>
       <c r="C95" s="10" t="n">
-        <v>1511.8</v>
+        <v>1617</v>
       </c>
       <c r="D95" s="13" t="n">
-        <v>1582.4</v>
+        <v>0</v>
       </c>
       <c r="E95" s="20" t="n">
-        <v>1579.15</v>
+        <v>0</v>
       </c>
       <c r="F95" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G95" s="4" t="n">
-        <v>1515.85</v>
+        <v>1637.9</v>
       </c>
     </row>
     <row r="96">
@@ -3031,22 +3031,22 @@
         </is>
       </c>
       <c r="B96" s="8" t="n">
-        <v>1169</v>
+        <v>1398.5</v>
       </c>
       <c r="C96" s="10" t="n">
-        <v>1127.7</v>
+        <v>1357.8</v>
       </c>
       <c r="D96" s="13" t="n">
-        <v>1167.5</v>
+        <v>0</v>
       </c>
       <c r="E96" s="20" t="n">
-        <v>1164.55</v>
+        <v>0</v>
       </c>
       <c r="F96" s="16" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>1135.15</v>
+        <v>1360.1</v>
       </c>
     </row>
     <row r="97">
@@ -3056,22 +3056,22 @@
         </is>
       </c>
       <c r="B97" s="8" t="n">
-        <v>1302.5</v>
+        <v>1434.2</v>
       </c>
       <c r="C97" s="10" t="n">
-        <v>1239.75</v>
+        <v>1397.4</v>
       </c>
       <c r="D97" s="13" t="n">
-        <v>1244.6</v>
+        <v>0</v>
       </c>
       <c r="E97" s="20" t="n">
-        <v>1244.7</v>
+        <v>0</v>
       </c>
       <c r="F97" s="16" t="n">
         <v>5</v>
       </c>
       <c r="G97" s="4" t="n">
-        <v>1297.5</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="98">
@@ -3081,22 +3081,22 @@
         </is>
       </c>
       <c r="B98" s="8" t="n">
-        <v>2150.85</v>
+        <v>2594.3</v>
       </c>
       <c r="C98" s="10" t="n">
-        <v>2059.25</v>
+        <v>2531</v>
       </c>
       <c r="D98" s="13" t="n">
-        <v>2108.75</v>
+        <v>0</v>
       </c>
       <c r="E98" s="20" t="n">
-        <v>2117.6</v>
+        <v>0</v>
       </c>
       <c r="F98" s="16" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G98" s="4" t="n">
-        <v>2063.35</v>
+        <v>2581.3</v>
       </c>
     </row>
     <row r="99">
@@ -3106,22 +3106,22 @@
         </is>
       </c>
       <c r="B99" s="8" t="n">
-        <v>2290.55</v>
+        <v>2103</v>
       </c>
       <c r="C99" s="10" t="n">
-        <v>2011.25</v>
+        <v>2083.5</v>
       </c>
       <c r="D99" s="13" t="n">
-        <v>2137.2</v>
+        <v>0</v>
       </c>
       <c r="E99" s="20" t="n">
-        <v>2139.95</v>
+        <v>0</v>
       </c>
       <c r="F99" s="16" t="n">
-        <v>58</v>
+        <v>8</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>2287.95</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="100">
@@ -3131,22 +3131,22 @@
         </is>
       </c>
       <c r="B100" s="8" t="n">
-        <v>545.05</v>
+        <v>749.8</v>
       </c>
       <c r="C100" s="10" t="n">
-        <v>522</v>
+        <v>723.95</v>
       </c>
       <c r="D100" s="13" t="n">
-        <v>523.05</v>
+        <v>0</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>526.75</v>
+        <v>0</v>
       </c>
       <c r="F100" s="16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>543.2</v>
+        <v>730</v>
       </c>
     </row>
     <row r="101">
@@ -3156,22 +3156,22 @@
         </is>
       </c>
       <c r="B101" s="8" t="n">
-        <v>6483.6</v>
+        <v>1487</v>
       </c>
       <c r="C101" s="10" t="n">
-        <v>6316.15</v>
+        <v>1453</v>
       </c>
       <c r="D101" s="13" t="n">
-        <v>6409</v>
+        <v>0</v>
       </c>
       <c r="E101" s="20" t="n">
-        <v>6406.75</v>
+        <v>0</v>
       </c>
       <c r="F101" s="16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>6428.8</v>
+        <v>1479.5</v>
       </c>
     </row>
     <row r="102">
@@ -3181,22 +3181,22 @@
         </is>
       </c>
       <c r="B102" s="8" t="n">
-        <v>4000.65</v>
+        <v>4323.4</v>
       </c>
       <c r="C102" s="10" t="n">
-        <v>3844</v>
+        <v>4189.4</v>
       </c>
       <c r="D102" s="13" t="n">
-        <v>3980</v>
+        <v>0</v>
       </c>
       <c r="E102" s="20" t="n">
-        <v>3979.4</v>
+        <v>0</v>
       </c>
       <c r="F102" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>3850.65</v>
+        <v>4216.1</v>
       </c>
     </row>
     <row r="103">
@@ -3206,22 +3206,22 @@
         </is>
       </c>
       <c r="B103" s="8" t="n">
-        <v>61.78</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="C103" s="10" t="n">
-        <v>59.53</v>
+        <v>69.55</v>
       </c>
       <c r="D103" s="13" t="n">
-        <v>61.22</v>
+        <v>0</v>
       </c>
       <c r="E103" s="20" t="n">
-        <v>61.31</v>
+        <v>0</v>
       </c>
       <c r="F103" s="16" t="n">
-        <v>405</v>
+        <v>193</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>60.42</v>
+        <v>70.34999999999999</v>
       </c>
     </row>
     <row r="104">
@@ -3231,22 +3231,22 @@
         </is>
       </c>
       <c r="B104" s="8" t="n">
-        <v>354.3</v>
+        <v>347.7</v>
       </c>
       <c r="C104" s="10" t="n">
-        <v>348.2</v>
+        <v>344</v>
       </c>
       <c r="D104" s="13" t="n">
-        <v>350.65</v>
+        <v>0</v>
       </c>
       <c r="E104" s="20" t="n">
-        <v>349.35</v>
+        <v>0</v>
       </c>
       <c r="F104" s="16" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>350.45</v>
+        <v>346.55</v>
       </c>
     </row>
     <row r="105">
@@ -3256,22 +3256,22 @@
         </is>
       </c>
       <c r="B105" s="8" t="n">
-        <v>1506.6</v>
+        <v>1746</v>
       </c>
       <c r="C105" s="10" t="n">
-        <v>1470.45</v>
+        <v>1678.4</v>
       </c>
       <c r="D105" s="13" t="n">
-        <v>1491.5</v>
+        <v>0</v>
       </c>
       <c r="E105" s="20" t="n">
-        <v>1493.2</v>
+        <v>0</v>
       </c>
       <c r="F105" s="16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>1495</v>
+        <v>1687.5</v>
       </c>
     </row>
     <row r="106">
@@ -3281,22 +3281,22 @@
         </is>
       </c>
       <c r="B106" s="8" t="n">
-        <v>224.06</v>
+        <v>249.34</v>
       </c>
       <c r="C106" s="10" t="n">
-        <v>220.26</v>
+        <v>244.91</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>223</v>
+        <v>0</v>
       </c>
       <c r="E106" s="20" t="n">
-        <v>221.94</v>
+        <v>0</v>
       </c>
       <c r="F106" s="16" t="n">
-        <v>168</v>
+        <v>80</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>220.76</v>
+        <v>249.17</v>
       </c>
     </row>
     <row r="107">
@@ -3306,22 +3306,22 @@
         </is>
       </c>
       <c r="B107" s="8" t="n">
-        <v>962.4</v>
+        <v>1146.2</v>
       </c>
       <c r="C107" s="10" t="n">
-        <v>935.35</v>
+        <v>1106.1</v>
       </c>
       <c r="D107" s="13" t="n">
-        <v>945.25</v>
+        <v>0</v>
       </c>
       <c r="E107" s="20" t="n">
-        <v>947.85</v>
+        <v>0</v>
       </c>
       <c r="F107" s="16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>961.4</v>
+        <v>1114.7</v>
       </c>
     </row>
     <row r="108">
@@ -3331,22 +3331,22 @@
         </is>
       </c>
       <c r="B108" s="8" t="n">
-        <v>4492.3</v>
+        <v>5732</v>
       </c>
       <c r="C108" s="10" t="n">
-        <v>4341.45</v>
+        <v>5626</v>
       </c>
       <c r="D108" s="13" t="n">
-        <v>4380</v>
+        <v>0</v>
       </c>
       <c r="E108" s="20" t="n">
-        <v>4402.75</v>
+        <v>0</v>
       </c>
       <c r="F108" s="16" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>4484.15</v>
+        <v>5667</v>
       </c>
     </row>
     <row r="109">
@@ -3356,22 +3356,22 @@
         </is>
       </c>
       <c r="B109" s="8" t="n">
-        <v>289.2</v>
+        <v>324.1</v>
       </c>
       <c r="C109" s="10" t="n">
-        <v>282.6</v>
+        <v>319</v>
       </c>
       <c r="D109" s="13" t="n">
-        <v>285</v>
+        <v>0</v>
       </c>
       <c r="E109" s="20" t="n">
-        <v>286.6</v>
+        <v>0</v>
       </c>
       <c r="F109" s="16" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G109" s="4" t="n">
-        <v>284.9</v>
+        <v>322.65</v>
       </c>
     </row>
     <row r="110">
@@ -3381,22 +3381,22 @@
         </is>
       </c>
       <c r="B110" s="8" t="n">
-        <v>2973.7</v>
+        <v>3105</v>
       </c>
       <c r="C110" s="10" t="n">
-        <v>2913.35</v>
+        <v>3062</v>
       </c>
       <c r="D110" s="13" t="n">
-        <v>2939.3</v>
+        <v>0</v>
       </c>
       <c r="E110" s="20" t="n">
-        <v>2939.8</v>
+        <v>0</v>
       </c>
       <c r="F110" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>2920</v>
+        <v>3104.3</v>
       </c>
     </row>
     <row r="111">
@@ -3406,22 +3406,22 @@
         </is>
       </c>
       <c r="B111" s="8" t="n">
-        <v>5028.3</v>
+        <v>6167</v>
       </c>
       <c r="C111" s="10" t="n">
-        <v>4890</v>
+        <v>6061.5</v>
       </c>
       <c r="D111" s="13" t="n">
-        <v>5006</v>
+        <v>0</v>
       </c>
       <c r="E111" s="20" t="n">
-        <v>5005</v>
+        <v>0</v>
       </c>
       <c r="F111" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>4960</v>
+        <v>6093.5</v>
       </c>
     </row>
     <row r="112">
@@ -3431,22 +3431,22 @@
         </is>
       </c>
       <c r="B112" s="8" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="C112" s="10" t="n">
-        <v>292.15</v>
+        <v>300.8</v>
       </c>
       <c r="D112" s="13" t="n">
-        <v>294.1</v>
+        <v>0</v>
       </c>
       <c r="E112" s="20" t="n">
-        <v>293.4</v>
+        <v>0</v>
       </c>
       <c r="F112" s="16" t="n">
-        <v>213</v>
+        <v>125</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>294.15</v>
+        <v>301.4</v>
       </c>
     </row>
     <row r="113">
@@ -3456,22 +3456,22 @@
         </is>
       </c>
       <c r="B113" s="8" t="n">
-        <v>134.54</v>
+        <v>152.43</v>
       </c>
       <c r="C113" s="10" t="n">
-        <v>132.7</v>
+        <v>148.88</v>
       </c>
       <c r="D113" s="13" t="n">
-        <v>133.6</v>
+        <v>0</v>
       </c>
       <c r="E113" s="20" t="n">
-        <v>133.57</v>
+        <v>0</v>
       </c>
       <c r="F113" s="16" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G113" s="4" t="n">
-        <v>134.4</v>
+        <v>149.47</v>
       </c>
     </row>
     <row r="114">
@@ -3481,22 +3481,22 @@
         </is>
       </c>
       <c r="B114" s="8" t="n">
-        <v>950</v>
+        <v>1011.75</v>
       </c>
       <c r="C114" s="10" t="n">
-        <v>924.2</v>
+        <v>997.15</v>
       </c>
       <c r="D114" s="13" t="n">
-        <v>940</v>
+        <v>0</v>
       </c>
       <c r="E114" s="20" t="n">
-        <v>941.1</v>
+        <v>0</v>
       </c>
       <c r="F114" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G114" s="4" t="n">
-        <v>930.4</v>
+        <v>1004.6</v>
       </c>
     </row>
     <row r="115">
@@ -3506,22 +3506,22 @@
         </is>
       </c>
       <c r="B115" s="8" t="n">
-        <v>170.51</v>
+        <v>216.46</v>
       </c>
       <c r="C115" s="10" t="n">
-        <v>165.05</v>
+        <v>211.25</v>
       </c>
       <c r="D115" s="13" t="n">
-        <v>168.71</v>
+        <v>0</v>
       </c>
       <c r="E115" s="20" t="n">
-        <v>168.67</v>
+        <v>0</v>
       </c>
       <c r="F115" s="16" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G115" s="4" t="n">
-        <v>168.8</v>
+        <v>213.83</v>
       </c>
     </row>
     <row r="116">
@@ -3531,22 +3531,22 @@
         </is>
       </c>
       <c r="B116" s="8" t="n">
-        <v>393.35</v>
+        <v>411.8</v>
       </c>
       <c r="C116" s="10" t="n">
-        <v>384.5</v>
+        <v>405.2</v>
       </c>
       <c r="D116" s="13" t="n">
-        <v>389.6</v>
+        <v>0</v>
       </c>
       <c r="E116" s="20" t="n">
-        <v>389.45</v>
+        <v>0</v>
       </c>
       <c r="F116" s="16" t="n">
-        <v>64</v>
+        <v>115</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>392.2</v>
+        <v>411</v>
       </c>
     </row>
     <row r="117">
@@ -3556,22 +3556,22 @@
         </is>
       </c>
       <c r="B117" s="8" t="n">
-        <v>849.8</v>
+        <v>917.7</v>
       </c>
       <c r="C117" s="10" t="n">
-        <v>823.65</v>
+        <v>906.2</v>
       </c>
       <c r="D117" s="13" t="n">
-        <v>847</v>
+        <v>0</v>
       </c>
       <c r="E117" s="20" t="n">
-        <v>846.55</v>
+        <v>0</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>846.6</v>
+        <v>912.35</v>
       </c>
     </row>
     <row r="118">
@@ -3581,22 +3581,22 @@
         </is>
       </c>
       <c r="B118" s="8" t="n">
-        <v>1499.9</v>
+        <v>1779.5</v>
       </c>
       <c r="C118" s="10" t="n">
-        <v>1475</v>
+        <v>1764.4</v>
       </c>
       <c r="D118" s="13" t="n">
-        <v>1482.7</v>
+        <v>0</v>
       </c>
       <c r="E118" s="20" t="n">
-        <v>1481.65</v>
+        <v>0</v>
       </c>
       <c r="F118" s="16" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>1499.15</v>
+        <v>1779.5</v>
       </c>
     </row>
     <row r="119">
@@ -3606,22 +3606,22 @@
         </is>
       </c>
       <c r="B119" s="8" t="n">
-        <v>2749.15</v>
+        <v>3150.8</v>
       </c>
       <c r="C119" s="10" t="n">
-        <v>2667.8</v>
+        <v>3025.8</v>
       </c>
       <c r="D119" s="13" t="n">
-        <v>2711</v>
+        <v>0</v>
       </c>
       <c r="E119" s="20" t="n">
-        <v>2715.85</v>
+        <v>0</v>
       </c>
       <c r="F119" s="16" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>2738.35</v>
+        <v>3061.1</v>
       </c>
     </row>
     <row r="120">
@@ -3631,22 +3631,22 @@
         </is>
       </c>
       <c r="B120" s="8" t="n">
-        <v>2774</v>
+        <v>3032</v>
       </c>
       <c r="C120" s="10" t="n">
-        <v>2705</v>
+        <v>2948.6</v>
       </c>
       <c r="D120" s="13" t="n">
-        <v>2730.95</v>
+        <v>0</v>
       </c>
       <c r="E120" s="20" t="n">
-        <v>2744.4</v>
+        <v>0</v>
       </c>
       <c r="F120" s="16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>2754.2</v>
+        <v>2953.2</v>
       </c>
     </row>
     <row r="121">
@@ -3656,22 +3656,22 @@
         </is>
       </c>
       <c r="B121" s="8" t="n">
-        <v>219.5</v>
+        <v>228.8</v>
       </c>
       <c r="C121" s="10" t="n">
-        <v>215.01</v>
+        <v>223.22</v>
       </c>
       <c r="D121" s="13" t="n">
-        <v>583</v>
+        <v>0</v>
       </c>
       <c r="E121" s="20" t="n">
-        <v>584.4</v>
+        <v>0</v>
       </c>
       <c r="F121" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G121" s="4" t="n">
-        <v>0</v>
+        <v>223.7</v>
       </c>
     </row>
     <row r="122">
@@ -3681,22 +3681,22 @@
         </is>
       </c>
       <c r="B122" s="8" t="n">
-        <v>1679.75</v>
+        <v>1765</v>
       </c>
       <c r="C122" s="10" t="n">
-        <v>1647</v>
+        <v>1726.6</v>
       </c>
       <c r="D122" s="13" t="n">
-        <v>1651.75</v>
+        <v>0</v>
       </c>
       <c r="E122" s="20" t="n">
-        <v>1652.2</v>
+        <v>0</v>
       </c>
       <c r="F122" s="16" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="G122" s="4" t="n">
-        <v>1674.35</v>
+        <v>1740.1</v>
       </c>
     </row>
     <row r="123">
@@ -3706,22 +3706,22 @@
         </is>
       </c>
       <c r="B123" s="8" t="n">
-        <v>693.2</v>
+        <v>649</v>
       </c>
       <c r="C123" s="10" t="n">
-        <v>682.25</v>
+        <v>641</v>
       </c>
       <c r="D123" s="13" t="n">
-        <v>692.1</v>
+        <v>0</v>
       </c>
       <c r="E123" s="20" t="n">
-        <v>691.7</v>
+        <v>0</v>
       </c>
       <c r="F123" s="16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G123" s="4" t="n">
-        <v>687.65</v>
+        <v>648</v>
       </c>
     </row>
     <row r="124">
@@ -3731,22 +3731,22 @@
         </is>
       </c>
       <c r="B124" s="8" t="n">
-        <v>1556.15</v>
+        <v>1662</v>
       </c>
       <c r="C124" s="10" t="n">
-        <v>1528.2</v>
+        <v>1614.2</v>
       </c>
       <c r="D124" s="13" t="n">
-        <v>1542.05</v>
+        <v>0</v>
       </c>
       <c r="E124" s="20" t="n">
-        <v>1547.35</v>
+        <v>0</v>
       </c>
       <c r="F124" s="16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G124" s="4" t="n">
-        <v>1549.95</v>
+        <v>1626.4</v>
       </c>
     </row>
     <row r="125">
@@ -3756,22 +3756,22 @@
         </is>
       </c>
       <c r="B125" s="8" t="n">
-        <v>594.9</v>
+        <v>738</v>
       </c>
       <c r="C125" s="10" t="n">
-        <v>581.05</v>
+        <v>728</v>
       </c>
       <c r="D125" s="13" t="n">
-        <v>584.5</v>
+        <v>0</v>
       </c>
       <c r="E125" s="20" t="n">
-        <v>582.9</v>
+        <v>0</v>
       </c>
       <c r="F125" s="16" t="n">
-        <v>174</v>
+        <v>104</v>
       </c>
       <c r="G125" s="4" t="n">
-        <v>589.3</v>
+        <v>734.95</v>
       </c>
     </row>
     <row r="126">
@@ -3781,22 +3781,22 @@
         </is>
       </c>
       <c r="B126" s="8" t="n">
-        <v>3270</v>
+        <v>3543</v>
       </c>
       <c r="C126" s="10" t="n">
-        <v>3227</v>
+        <v>3512.8</v>
       </c>
       <c r="D126" s="13" t="n">
-        <v>3239</v>
+        <v>0</v>
       </c>
       <c r="E126" s="20" t="n">
-        <v>3246.6</v>
+        <v>0</v>
       </c>
       <c r="F126" s="16" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G126" s="4" t="n">
-        <v>3246</v>
+        <v>3533.2</v>
       </c>
     </row>
     <row r="127">
@@ -3806,22 +3806,22 @@
         </is>
       </c>
       <c r="B127" s="8" t="n">
-        <v>1286.4</v>
+        <v>1613.2</v>
       </c>
       <c r="C127" s="10" t="n">
-        <v>1264.35</v>
+        <v>1593.1</v>
       </c>
       <c r="D127" s="13" t="n">
-        <v>1270.95</v>
+        <v>0</v>
       </c>
       <c r="E127" s="20" t="n">
-        <v>1272.75</v>
+        <v>0</v>
       </c>
       <c r="F127" s="16" t="n">
-        <v>37</v>
+        <v>6</v>
       </c>
       <c r="G127" s="4" t="n">
-        <v>1278.75</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="128">
@@ -3831,22 +3831,22 @@
         </is>
       </c>
       <c r="B128" s="8" t="n">
-        <v>3188.25</v>
+        <v>3649.5</v>
       </c>
       <c r="C128" s="10" t="n">
-        <v>3092.9</v>
+        <v>3611.4</v>
       </c>
       <c r="D128" s="13" t="n">
-        <v>3178.95</v>
+        <v>0</v>
       </c>
       <c r="E128" s="20" t="n">
-        <v>3174.15</v>
+        <v>0</v>
       </c>
       <c r="F128" s="16" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G128" s="4" t="n">
-        <v>3105</v>
+        <v>3641.3</v>
       </c>
     </row>
     <row r="129">
@@ -3856,22 +3856,22 @@
         </is>
       </c>
       <c r="B129" s="8" t="n">
-        <v>3232.1</v>
+        <v>3314</v>
       </c>
       <c r="C129" s="10" t="n">
-        <v>3107.4</v>
+        <v>3265.7</v>
       </c>
       <c r="D129" s="13" t="n">
-        <v>3108.85</v>
+        <v>0</v>
       </c>
       <c r="E129" s="20" t="n">
-        <v>3126.8</v>
+        <v>0</v>
       </c>
       <c r="F129" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G129" s="4" t="n">
-        <v>3224.1</v>
+        <v>3277.3</v>
       </c>
     </row>
     <row r="130">
@@ -3881,22 +3881,22 @@
         </is>
       </c>
       <c r="B130" s="8" t="n">
-        <v>1535.35</v>
+        <v>1469.8</v>
       </c>
       <c r="C130" s="10" t="n">
-        <v>1484.45</v>
+        <v>1421.3</v>
       </c>
       <c r="D130" s="13" t="n">
-        <v>1526.15</v>
+        <v>0</v>
       </c>
       <c r="E130" s="20" t="n">
-        <v>1530.9</v>
+        <v>0</v>
       </c>
       <c r="F130" s="16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G130" s="4" t="n">
-        <v>1504.35</v>
+        <v>1457.3</v>
       </c>
     </row>
     <row r="131">
@@ -3906,22 +3906,22 @@
         </is>
       </c>
       <c r="B131" s="8" t="n">
-        <v>4729</v>
+        <v>5628</v>
       </c>
       <c r="C131" s="10" t="n">
-        <v>4605</v>
+        <v>5530</v>
       </c>
       <c r="D131" s="13" t="n">
-        <v>4625.7</v>
+        <v>0</v>
       </c>
       <c r="E131" s="20" t="n">
-        <v>4620.2</v>
+        <v>0</v>
       </c>
       <c r="F131" s="16" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>4722</v>
+        <v>5610.5</v>
       </c>
     </row>
     <row r="132">
@@ -3931,22 +3931,22 @@
         </is>
       </c>
       <c r="B132" s="8" t="n">
-        <v>2488.7</v>
+        <v>2878.9</v>
       </c>
       <c r="C132" s="10" t="n">
-        <v>2426.15</v>
+        <v>2815.2</v>
       </c>
       <c r="D132" s="13" t="n">
-        <v>2473.6</v>
+        <v>0</v>
       </c>
       <c r="E132" s="20" t="n">
-        <v>2475.25</v>
+        <v>0</v>
       </c>
       <c r="F132" s="16" t="n">
         <v>8</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>2451.9</v>
+        <v>2870</v>
       </c>
     </row>
     <row r="133">
@@ -3956,22 +3956,22 @@
         </is>
       </c>
       <c r="B133" s="8" t="n">
-        <v>2035</v>
+        <v>2090</v>
       </c>
       <c r="C133" s="10" t="n">
-        <v>1996.75</v>
+        <v>2029</v>
       </c>
       <c r="D133" s="13" t="n">
-        <v>2009</v>
+        <v>0</v>
       </c>
       <c r="E133" s="20" t="n">
-        <v>2001.75</v>
+        <v>0</v>
       </c>
       <c r="F133" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G133" s="4" t="n">
-        <v>0</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="134">
@@ -3981,22 +3981,22 @@
         </is>
       </c>
       <c r="B134" s="8" t="n">
-        <v>11423</v>
+        <v>11991</v>
       </c>
       <c r="C134" s="10" t="n">
-        <v>11180</v>
+        <v>11898</v>
       </c>
       <c r="D134" s="13" t="n">
-        <v>11367</v>
+        <v>0</v>
       </c>
       <c r="E134" s="20" t="n">
-        <v>11397.05</v>
+        <v>0</v>
       </c>
       <c r="F134" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G134" s="4" t="n">
-        <v>11258.7</v>
+        <v>11926</v>
       </c>
     </row>
     <row r="135">
@@ -4006,22 +4006,22 @@
         </is>
       </c>
       <c r="B135" s="8" t="n">
-        <v>615.8</v>
+        <v>654.8</v>
       </c>
       <c r="C135" s="10" t="n">
-        <v>601.2</v>
+        <v>644.45</v>
       </c>
       <c r="D135" s="13" t="n">
-        <v>613.45</v>
+        <v>0</v>
       </c>
       <c r="E135" s="20" t="n">
-        <v>614.25</v>
+        <v>0</v>
       </c>
       <c r="F135" s="16" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G135" s="4" t="n">
-        <v>612.2</v>
+        <v>647.65</v>
       </c>
     </row>
     <row r="136">
@@ -4031,22 +4031,22 @@
         </is>
       </c>
       <c r="B136" s="8" t="n">
-        <v>377.45</v>
+        <v>446.9</v>
       </c>
       <c r="C136" s="10" t="n">
-        <v>368.6</v>
+        <v>440.65</v>
       </c>
       <c r="D136" s="13" t="n">
-        <v>370.45</v>
+        <v>0</v>
       </c>
       <c r="E136" s="20" t="n">
-        <v>370.55</v>
+        <v>0</v>
       </c>
       <c r="F136" s="16" t="n">
-        <v>139</v>
+        <v>47</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>370.8</v>
+        <v>443.5</v>
       </c>
     </row>
     <row r="137">
@@ -4056,22 +4056,22 @@
         </is>
       </c>
       <c r="B137" s="8" t="n">
-        <v>1299.7</v>
+        <v>1281.9</v>
       </c>
       <c r="C137" s="10" t="n">
-        <v>1274</v>
+        <v>1261</v>
       </c>
       <c r="D137" s="13" t="n">
-        <v>1276</v>
+        <v>0</v>
       </c>
       <c r="E137" s="20" t="n">
-        <v>1277.75</v>
+        <v>0</v>
       </c>
       <c r="F137" s="16" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>1298.9</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="138">
@@ -4081,22 +4081,22 @@
         </is>
       </c>
       <c r="B138" s="8" t="n">
-        <v>105.5</v>
+        <v>130.43</v>
       </c>
       <c r="C138" s="10" t="n">
-        <v>103.05</v>
+        <v>127.21</v>
       </c>
       <c r="D138" s="13" t="n">
-        <v>103.83</v>
+        <v>0</v>
       </c>
       <c r="E138" s="20" t="n">
-        <v>104.01</v>
+        <v>0</v>
       </c>
       <c r="F138" s="16" t="n">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>104.99</v>
+        <v>130.25</v>
       </c>
     </row>
     <row r="139" ht="15.75" customHeight="1" thickBot="1">
@@ -4106,22 +4106,22 @@
         </is>
       </c>
       <c r="B139" s="18" t="n">
-        <v>849.85</v>
+        <v>919.8</v>
       </c>
       <c r="C139" s="11" t="n">
-        <v>835.25</v>
+        <v>902.65</v>
       </c>
       <c r="D139" s="14" t="n">
-        <v>846</v>
+        <v>0</v>
       </c>
       <c r="E139" s="21" t="n">
-        <v>844.4</v>
+        <v>0</v>
       </c>
       <c r="F139" s="17" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>839</v>
+        <v>910</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed webdriver issue in cash and algo.py
</commit_message>
<xml_diff>
--- a/algo high low.xlsx
+++ b/algo high low.xlsx
@@ -634,7 +634,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G139"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="10.28515625" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -681,22 +681,22 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>492.25</v>
+        <v>472.5</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>482.4</v>
+        <v>466.15</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>0</v>
+        <v>469.5</v>
       </c>
       <c r="E2" s="19" t="n">
-        <v>0</v>
+        <v>469.3</v>
       </c>
       <c r="F2" s="15" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>484.15</v>
+        <v>471.8</v>
       </c>
     </row>
     <row r="3">
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>5895</v>
+        <v>6048</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>5824</v>
+        <v>5975</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0</v>
+        <v>5960</v>
       </c>
       <c r="E3" s="20" t="n">
-        <v>0</v>
+        <v>5961</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>5885</v>
+        <v>6014.5</v>
       </c>
     </row>
     <row r="4">
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>218.6</v>
+        <v>223.57</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>213.98</v>
+        <v>219.01</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0</v>
+        <v>222</v>
       </c>
       <c r="E4" s="20" t="n">
-        <v>0</v>
+        <v>222.29</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>217.96</v>
+        <v>221.09</v>
       </c>
     </row>
     <row r="5">
@@ -756,22 +756,22 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>295.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>278.65</v>
+        <v>86.2</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>0</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="E5" s="20" t="n">
-        <v>0</v>
+        <v>88.55</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>280.85</v>
+        <v>89.05</v>
       </c>
     </row>
     <row r="6">
@@ -781,22 +781,22 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>2578.8</v>
+        <v>2567</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>2536</v>
+        <v>2541.3</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>0</v>
+        <v>2537</v>
       </c>
       <c r="E6" s="20" t="n">
-        <v>0</v>
+        <v>2540</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2566.8</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="7">
@@ -806,22 +806,22 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1409.1</v>
+        <v>1410.6</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>1392</v>
+        <v>1394.8</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>0</v>
+        <v>1394</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>0</v>
+        <v>1395.4</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1406.2</v>
+        <v>1403.3</v>
       </c>
     </row>
     <row r="8">
@@ -831,22 +831,22 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>5400</v>
+        <v>5356.5</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>5200.5</v>
+        <v>5218.5</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>0</v>
+        <v>5302</v>
       </c>
       <c r="E8" s="20" t="n">
-        <v>0</v>
+        <v>5288</v>
       </c>
       <c r="F8" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>5213</v>
+        <v>5350</v>
       </c>
     </row>
     <row r="9">
@@ -856,22 +856,22 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>569.55</v>
+        <v>573.85</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>559.35</v>
+        <v>564.4</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>0</v>
+        <v>571.35</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>0</v>
+        <v>570.9</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>562.75</v>
+        <v>573.1</v>
       </c>
     </row>
     <row r="10">
@@ -881,22 +881,22 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>7061</v>
+        <v>7120</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>6965.5</v>
+        <v>7080</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>0</v>
+        <v>7062</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>0</v>
+        <v>7064.5</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>7029</v>
+        <v>7090.5</v>
       </c>
     </row>
     <row r="11">
@@ -906,22 +906,22 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>498.3</v>
+        <v>500.55</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>487.65</v>
+        <v>489.5</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0</v>
+        <v>494.7</v>
       </c>
       <c r="E11" s="20" t="n">
-        <v>0</v>
+        <v>494.7</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>495.8</v>
+        <v>489.65</v>
       </c>
     </row>
     <row r="12">
@@ -931,22 +931,22 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>243.25</v>
+        <v>241.9</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>237.01</v>
+        <v>237.05</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>0</v>
+        <v>238.26</v>
       </c>
       <c r="E12" s="20" t="n">
-        <v>0</v>
+        <v>239.61</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>73</v>
+        <v>155</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>237.65</v>
+        <v>238.72</v>
       </c>
     </row>
     <row r="13">
@@ -956,22 +956,22 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>1428.9</v>
+        <v>1514.4</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>1362.6</v>
+        <v>1461</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>0</v>
+        <v>1455.5</v>
       </c>
       <c r="E13" s="20" t="n">
-        <v>0</v>
+        <v>1456.7</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>1372.6</v>
+        <v>1462.5</v>
       </c>
     </row>
     <row r="14">
@@ -981,22 +981,22 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>6912</v>
+        <v>7222.5</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>6750.5</v>
+        <v>7090.5</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>0</v>
+        <v>7203.5</v>
       </c>
       <c r="E14" s="20" t="n">
-        <v>0</v>
+        <v>7203</v>
       </c>
       <c r="F14" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>6771</v>
+        <v>7222</v>
       </c>
     </row>
     <row r="15">
@@ -1006,22 +1006,22 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>690.5</v>
+        <v>708.55</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>683.65</v>
+        <v>692.45</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>0</v>
+        <v>696.7</v>
       </c>
       <c r="E15" s="20" t="n">
-        <v>0</v>
+        <v>696.2</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>689.95</v>
+        <v>704.4</v>
       </c>
     </row>
     <row r="16">
@@ -1031,22 +1031,22 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>1225.9</v>
+        <v>1204.9</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>1201.4</v>
+        <v>1175.5</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>0</v>
+        <v>1191.7</v>
       </c>
       <c r="E16" s="20" t="n">
-        <v>0</v>
+        <v>1197.1</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>1205.9</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="17">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>8861.5</v>
+        <v>8978.5</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>8615</v>
+        <v>8807.5</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>0</v>
+        <v>8740</v>
       </c>
       <c r="E17" s="20" t="n">
-        <v>0</v>
+        <v>8741</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8630</v>
+        <v>8848</v>
       </c>
     </row>
     <row r="18">
@@ -1081,22 +1081,22 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>2053</v>
+        <v>2070</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>2035.5</v>
+        <v>2046</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>0</v>
+        <v>2040</v>
       </c>
       <c r="E18" s="20" t="n">
-        <v>0</v>
+        <v>2036.5</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>2046.9</v>
+        <v>2055.1</v>
       </c>
     </row>
     <row r="19">
@@ -1106,22 +1106,22 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>9275</v>
+        <v>9336.5</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>9211</v>
+        <v>9250</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>0</v>
+        <v>9248</v>
       </c>
       <c r="E19" s="20" t="n">
-        <v>0</v>
+        <v>9243.5</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>9244.5</v>
+        <v>9298</v>
       </c>
     </row>
     <row r="20">
@@ -1131,22 +1131,22 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>2764</v>
+        <v>2508.9</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>2681</v>
+        <v>2383</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>0</v>
+        <v>2671</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>0</v>
+        <v>2660.2</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>2727.5</v>
+        <v>2409.9</v>
       </c>
     </row>
     <row r="21">
@@ -1156,22 +1156,22 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>573.25</v>
+        <v>567.95</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>550.1</v>
+        <v>558.6</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0</v>
+        <v>554</v>
       </c>
       <c r="E21" s="20" t="n">
-        <v>0</v>
+        <v>553.1</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>558.1</v>
+        <v>563.65</v>
       </c>
     </row>
     <row r="22">
@@ -1181,22 +1181,22 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>173.2</v>
+        <v>166.68</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>169.94</v>
+        <v>164.4</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>0</v>
+        <v>165.25</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>0</v>
+        <v>165.46</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>171.28</v>
+        <v>166.15</v>
       </c>
     </row>
     <row r="23">
@@ -1206,22 +1206,22 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>242.8</v>
+        <v>244.85</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>236.2</v>
+        <v>240.8</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>0</v>
+        <v>242.7</v>
       </c>
       <c r="E23" s="20" t="n">
-        <v>0</v>
+        <v>243.04</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>236.75</v>
+        <v>244.43</v>
       </c>
     </row>
     <row r="24">
@@ -1231,22 +1231,22 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>1258.5</v>
+        <v>1300.7</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>1240.3</v>
+        <v>1276.7</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>0</v>
+        <v>1277.9</v>
       </c>
       <c r="E24" s="20" t="n">
-        <v>0</v>
+        <v>1275.7</v>
       </c>
       <c r="F24" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>1254.4</v>
+        <v>1283.2</v>
       </c>
     </row>
     <row r="25">
@@ -1256,22 +1256,22 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>373.5</v>
+        <v>385.65</v>
       </c>
       <c r="C25" s="10" t="n">
-        <v>362.55</v>
+        <v>378.5</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>0</v>
+        <v>383.35</v>
       </c>
       <c r="E25" s="20" t="n">
-        <v>0</v>
+        <v>383.8</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>520</v>
+        <v>267</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>371.5</v>
+        <v>383.05</v>
       </c>
     </row>
     <row r="26">
@@ -1281,22 +1281,22 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>1279</v>
+        <v>1259.6</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>1251.6</v>
+        <v>1242.9</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>0</v>
+        <v>1242</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>0</v>
+        <v>1245.1</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>1275.9</v>
+        <v>1251.3</v>
       </c>
     </row>
     <row r="27">
@@ -1306,22 +1306,22 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>252.25</v>
+        <v>262.35</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>243.2</v>
+        <v>256</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>0</v>
+        <v>255.05</v>
       </c>
       <c r="E27" s="20" t="n">
-        <v>0</v>
+        <v>254.8</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>157</v>
+        <v>182</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>252.07</v>
+        <v>257.63</v>
       </c>
     </row>
     <row r="28">
@@ -1331,22 +1331,22 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>345.15</v>
+        <v>335.3</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>338.5</v>
+        <v>331.15</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>0</v>
+        <v>331</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>0</v>
+        <v>330.75</v>
       </c>
       <c r="F28" s="16" t="n">
         <v>13</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>341.8</v>
+        <v>333</v>
       </c>
     </row>
     <row r="29">
@@ -1359,19 +1359,19 @@
         <v>5547.5</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>5470.5</v>
+        <v>5489</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>0</v>
+        <v>5490</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>0</v>
+        <v>5486.5</v>
       </c>
       <c r="F29" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>5505.5</v>
+        <v>5522.5</v>
       </c>
     </row>
     <row r="30">
@@ -1381,22 +1381,22 @@
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>434</v>
+        <v>426.6</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>423.8</v>
+        <v>415.45</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>0</v>
+        <v>424.45</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>0</v>
+        <v>424.8</v>
       </c>
       <c r="F30" s="16" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>431.3</v>
+        <v>426.2</v>
       </c>
     </row>
     <row r="31">
@@ -1406,22 +1406,22 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>109.5</v>
+        <v>108.15</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>107.76</v>
+        <v>106.61</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>0</v>
+        <v>107.2</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>0</v>
+        <v>107.21</v>
       </c>
       <c r="F31" s="16" t="n">
-        <v>261</v>
+        <v>173</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>108.2</v>
+        <v>107.82</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>754.3</v>
+        <v>759</v>
       </c>
       <c r="C32" s="10" t="n">
-        <v>736</v>
+        <v>744.7</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>0</v>
+        <v>739.5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>0</v>
+        <v>738.7</v>
       </c>
       <c r="F32" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>747.4</v>
+        <v>750.4</v>
       </c>
     </row>
     <row r="33">
@@ -1456,22 +1456,22 @@
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>631.9</v>
+        <v>593.95</v>
       </c>
       <c r="C33" s="10" t="n">
-        <v>619.45</v>
+        <v>585</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>0</v>
+        <v>595.6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>0</v>
+        <v>594.3</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>630.4</v>
+        <v>592.2</v>
       </c>
     </row>
     <row r="34">
@@ -1481,22 +1481,22 @@
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>1639.5</v>
+        <v>1648.5</v>
       </c>
       <c r="C34" s="10" t="n">
-        <v>1619.6</v>
+        <v>1629</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>0</v>
+        <v>1626.7</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>0</v>
+        <v>1628</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>1629.5</v>
+        <v>1637.1</v>
       </c>
     </row>
     <row r="35">
@@ -1506,22 +1506,22 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>1511.7</v>
+        <v>1490.8</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>1489</v>
+        <v>1478.5</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>0</v>
+        <v>1483</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>0</v>
+        <v>1484.2</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>1496.5</v>
+        <v>1484.5</v>
       </c>
     </row>
     <row r="36">
@@ -1531,22 +1531,22 @@
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>8400</v>
+        <v>8485</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>8252.5</v>
+        <v>8283</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>0</v>
+        <v>8325</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>0</v>
+        <v>8321.5</v>
       </c>
       <c r="F36" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>8367.5</v>
+        <v>8336</v>
       </c>
     </row>
     <row r="37">
@@ -1556,22 +1556,22 @@
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>756.35</v>
+        <v>745.6</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>726.5</v>
+        <v>722.95</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>0</v>
+        <v>720.9</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>732.65</v>
+        <v>723</v>
       </c>
     </row>
     <row r="38">
@@ -1581,22 +1581,22 @@
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>2509</v>
+        <v>2438</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>2420</v>
+        <v>2389.4</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>0</v>
+        <v>2383.5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>0</v>
+        <v>2389.5</v>
       </c>
       <c r="F38" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>2456.5</v>
+        <v>2425.1</v>
       </c>
     </row>
     <row r="39">
@@ -1606,22 +1606,22 @@
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>362.75</v>
+        <v>359.3</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>349.1</v>
+        <v>352</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>0</v>
+        <v>351.1</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>0</v>
+        <v>351.55</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>362.25</v>
+        <v>352.5</v>
       </c>
     </row>
     <row r="40">
@@ -1631,22 +1631,22 @@
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>3062.2</v>
+        <v>2973.2</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>2981.3</v>
+        <v>2915.6</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>0</v>
+        <v>2946</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>0</v>
+        <v>2940.4</v>
       </c>
       <c r="F40" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>3052.7</v>
+        <v>2947.8</v>
       </c>
     </row>
     <row r="41">
@@ -1656,22 +1656,22 @@
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>484.5</v>
+        <v>484.7</v>
       </c>
       <c r="C41" s="10" t="n">
-        <v>478.65</v>
+        <v>479.75</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>0</v>
+        <v>482</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>0</v>
+        <v>481.95</v>
       </c>
       <c r="F41" s="16" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>479.4</v>
+        <v>484.05</v>
       </c>
     </row>
     <row r="42">
@@ -1681,22 +1681,22 @@
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>2096</v>
+        <v>2137.3</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>2061.3</v>
+        <v>2050</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>0</v>
+        <v>2137.2</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>0</v>
+        <v>2143</v>
       </c>
       <c r="F42" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>2084.1</v>
+        <v>2133.4</v>
       </c>
     </row>
     <row r="43">
@@ -1706,22 +1706,22 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>1390</v>
+        <v>1374.9</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>1340.8</v>
+        <v>1336.3</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>0</v>
+        <v>1323</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>0</v>
+        <v>1327.4</v>
       </c>
       <c r="F43" s="16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>1366.2</v>
+        <v>1346.1</v>
       </c>
     </row>
     <row r="44">
@@ -1731,22 +1731,22 @@
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>2174</v>
+        <v>2096.8</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>2113.4</v>
+        <v>2035</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>0</v>
+        <v>2066</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>0</v>
+        <v>2069.2</v>
       </c>
       <c r="F44" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>2149.9</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="45">
@@ -1756,22 +1756,22 @@
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>95.75</v>
+        <v>93.05</v>
       </c>
       <c r="C45" s="10" t="n">
-        <v>93.33</v>
+        <v>91.25</v>
       </c>
       <c r="D45" s="13" t="n">
-        <v>0</v>
+        <v>91.62</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>0</v>
+        <v>91.52</v>
       </c>
       <c r="F45" s="16" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>94.78</v>
+        <v>93.05</v>
       </c>
     </row>
     <row r="46">
@@ -1781,22 +1781,22 @@
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>6705</v>
+        <v>6764</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>6415</v>
+        <v>6668</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>0</v>
+        <v>6482.5</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>0</v>
+        <v>6483</v>
       </c>
       <c r="F46" s="16" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>6462</v>
+        <v>6716</v>
       </c>
     </row>
     <row r="47">
@@ -1806,22 +1806,22 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>16727</v>
+        <v>15189</v>
       </c>
       <c r="C47" s="10" t="n">
-        <v>16420</v>
+        <v>15050</v>
       </c>
       <c r="D47" s="13" t="n">
-        <v>0</v>
+        <v>15025</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>0</v>
+        <v>15019</v>
       </c>
       <c r="F47" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>16674</v>
+        <v>15168</v>
       </c>
     </row>
     <row r="48">
@@ -1831,22 +1831,22 @@
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>739</v>
+        <v>790.5</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>722.35</v>
+        <v>775</v>
       </c>
       <c r="D48" s="13" t="n">
-        <v>0</v>
+        <v>773.9</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>0</v>
+        <v>776.5</v>
       </c>
       <c r="F48" s="16" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>724.45</v>
+        <v>775</v>
       </c>
     </row>
     <row r="49">
@@ -1856,22 +1856,22 @@
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>1241.8</v>
+        <v>1247.9</v>
       </c>
       <c r="C49" s="10" t="n">
-        <v>1214.2</v>
+        <v>1234.8</v>
       </c>
       <c r="D49" s="13" t="n">
-        <v>0</v>
+        <v>1229</v>
       </c>
       <c r="E49" s="20" t="n">
-        <v>0</v>
+        <v>1230.1</v>
       </c>
       <c r="F49" s="16" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>1227.5</v>
+        <v>1235.6</v>
       </c>
     </row>
     <row r="50">
@@ -1881,22 +1881,22 @@
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>3556.4</v>
+        <v>3535</v>
       </c>
       <c r="C50" s="10" t="n">
-        <v>3508.1</v>
+        <v>3454.6</v>
       </c>
       <c r="D50" s="13" t="n">
-        <v>0</v>
+        <v>3497</v>
       </c>
       <c r="E50" s="20" t="n">
-        <v>0</v>
+        <v>3510.6</v>
       </c>
       <c r="F50" s="16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>3545.9</v>
+        <v>3519.9</v>
       </c>
     </row>
     <row r="51">
@@ -1906,22 +1906,22 @@
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>396.65</v>
+        <v>387.65</v>
       </c>
       <c r="C51" s="10" t="n">
-        <v>390.65</v>
+        <v>383.5</v>
       </c>
       <c r="D51" s="13" t="n">
-        <v>0</v>
+        <v>381.95</v>
       </c>
       <c r="E51" s="20" t="n">
-        <v>0</v>
+        <v>382.15</v>
       </c>
       <c r="F51" s="16" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>396.25</v>
+        <v>384.4</v>
       </c>
     </row>
     <row r="52">
@@ -1931,22 +1931,22 @@
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>1471.1</v>
+        <v>1430</v>
       </c>
       <c r="C52" s="10" t="n">
-        <v>1425</v>
+        <v>1371</v>
       </c>
       <c r="D52" s="13" t="n">
-        <v>0</v>
+        <v>1421.9</v>
       </c>
       <c r="E52" s="20" t="n">
-        <v>0</v>
+        <v>1420.2</v>
       </c>
       <c r="F52" s="16" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>1444.8</v>
+        <v>1414.7</v>
       </c>
     </row>
     <row r="53">
@@ -1956,22 +1956,22 @@
         </is>
       </c>
       <c r="B53" s="8" t="n">
-        <v>1155.2</v>
+        <v>1145</v>
       </c>
       <c r="C53" s="10" t="n">
-        <v>1115</v>
+        <v>1099.1</v>
       </c>
       <c r="D53" s="13" t="n">
+        <v>1114.9</v>
+      </c>
+      <c r="E53" s="20" t="n">
+        <v>1117</v>
+      </c>
+      <c r="F53" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="16" t="n">
-        <v>1</v>
-      </c>
       <c r="G53" s="4" t="n">
-        <v>1129</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="54">
@@ -1981,22 +1981,22 @@
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>519.3</v>
+        <v>553.65</v>
       </c>
       <c r="C54" s="10" t="n">
-        <v>507.05</v>
+        <v>529</v>
       </c>
       <c r="D54" s="13" t="n">
-        <v>0</v>
+        <v>512.1</v>
       </c>
       <c r="E54" s="20" t="n">
-        <v>0</v>
+        <v>513.4</v>
       </c>
       <c r="F54" s="16" t="n">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>517.75</v>
+        <v>546.15</v>
       </c>
     </row>
     <row r="55">
@@ -2006,22 +2006,22 @@
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>1308.2</v>
+        <v>1291.2</v>
       </c>
       <c r="C55" s="10" t="n">
-        <v>1290</v>
+        <v>1277.5</v>
       </c>
       <c r="D55" s="13" t="n">
-        <v>0</v>
+        <v>1278.8</v>
       </c>
       <c r="E55" s="20" t="n">
-        <v>0</v>
+        <v>1277.4</v>
       </c>
       <c r="F55" s="16" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>1305.7</v>
+        <v>1286.5</v>
       </c>
     </row>
     <row r="56">
@@ -2031,22 +2031,22 @@
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>2269.1</v>
+        <v>2254.3</v>
       </c>
       <c r="C56" s="10" t="n">
-        <v>2176.1</v>
+        <v>2188.4</v>
       </c>
       <c r="D56" s="13" t="n">
-        <v>0</v>
+        <v>2180</v>
       </c>
       <c r="E56" s="20" t="n">
-        <v>0</v>
+        <v>2182.4</v>
       </c>
       <c r="F56" s="16" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>2181.5</v>
+        <v>2194.1</v>
       </c>
     </row>
     <row r="57">
@@ -2056,22 +2056,22 @@
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>521.1</v>
+        <v>526.75</v>
       </c>
       <c r="C57" s="10" t="n">
-        <v>507.55</v>
+        <v>518.5</v>
       </c>
       <c r="D57" s="13" t="n">
-        <v>0</v>
+        <v>518.25</v>
       </c>
       <c r="E57" s="20" t="n">
-        <v>0</v>
+        <v>517.95</v>
       </c>
       <c r="F57" s="16" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>513.2</v>
+        <v>523.6</v>
       </c>
     </row>
     <row r="58">
@@ -2081,22 +2081,22 @@
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>2791.9</v>
+        <v>2687.6</v>
       </c>
       <c r="C58" s="10" t="n">
-        <v>2721</v>
+        <v>2640.1</v>
       </c>
       <c r="D58" s="13" t="n">
-        <v>0</v>
+        <v>2656</v>
       </c>
       <c r="E58" s="20" t="n">
-        <v>0</v>
+        <v>2659.4</v>
       </c>
       <c r="F58" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>2788.2</v>
+        <v>2687.6</v>
       </c>
     </row>
     <row r="59">
@@ -2106,22 +2106,22 @@
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>474.75</v>
+        <v>467.7</v>
       </c>
       <c r="C59" s="10" t="n">
-        <v>465.25</v>
+        <v>459.2</v>
       </c>
       <c r="D59" s="13" t="n">
-        <v>0</v>
+        <v>462.75</v>
       </c>
       <c r="E59" s="20" t="n">
-        <v>0</v>
+        <v>462.05</v>
       </c>
       <c r="F59" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>474.75</v>
+        <v>466.8</v>
       </c>
     </row>
     <row r="60">
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="B60" s="8" t="n">
-        <v>5140.9</v>
+        <v>5034.1</v>
       </c>
       <c r="C60" s="10" t="n">
-        <v>4972</v>
+        <v>4950</v>
       </c>
       <c r="D60" s="13" t="n">
-        <v>0</v>
+        <v>4966</v>
       </c>
       <c r="E60" s="20" t="n">
-        <v>0</v>
+        <v>4961.6</v>
       </c>
       <c r="F60" s="16" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>5135.1</v>
+        <v>4971.2</v>
       </c>
     </row>
     <row r="61">
@@ -2156,22 +2156,22 @@
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>1600.8</v>
+        <v>1584.5</v>
       </c>
       <c r="C61" s="10" t="n">
-        <v>1579.2</v>
+        <v>1565.1</v>
       </c>
       <c r="D61" s="13" t="n">
-        <v>0</v>
+        <v>1574</v>
       </c>
       <c r="E61" s="20" t="n">
-        <v>0</v>
+        <v>1573.6</v>
       </c>
       <c r="F61" s="16" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>1593.9</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="62">
@@ -2181,22 +2181,22 @@
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>1658</v>
+        <v>1675.8</v>
       </c>
       <c r="C62" s="10" t="n">
-        <v>1642.6</v>
+        <v>1660.6</v>
       </c>
       <c r="D62" s="13" t="n">
-        <v>0</v>
+        <v>1649.5</v>
       </c>
       <c r="E62" s="20" t="n">
-        <v>0</v>
+        <v>1648.2</v>
       </c>
       <c r="F62" s="16" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>1651.4</v>
+        <v>1663.1</v>
       </c>
     </row>
     <row r="63">
@@ -2206,22 +2206,22 @@
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>4845</v>
+        <v>4887.4</v>
       </c>
       <c r="C63" s="10" t="n">
         <v>4800</v>
       </c>
       <c r="D63" s="13" t="n">
-        <v>0</v>
+        <v>4810</v>
       </c>
       <c r="E63" s="20" t="n">
-        <v>0</v>
+        <v>4814.1</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4812</v>
+        <v>4884</v>
       </c>
     </row>
     <row r="64">
@@ -2231,22 +2231,22 @@
         </is>
       </c>
       <c r="B64" s="8" t="n">
-        <v>755.5</v>
+        <v>785.6</v>
       </c>
       <c r="C64" s="10" t="n">
-        <v>749</v>
+        <v>777.7</v>
       </c>
       <c r="D64" s="13" t="n">
-        <v>0</v>
+        <v>780.65</v>
       </c>
       <c r="E64" s="20" t="n">
-        <v>0</v>
+        <v>780.4</v>
       </c>
       <c r="F64" s="16" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>754.5</v>
+        <v>780.35</v>
       </c>
     </row>
     <row r="65">
@@ -2256,22 +2256,22 @@
         </is>
       </c>
       <c r="B65" s="8" t="n">
-        <v>661.75</v>
+        <v>669.7</v>
       </c>
       <c r="C65" s="10" t="n">
-        <v>652</v>
+        <v>654.65</v>
       </c>
       <c r="D65" s="13" t="n">
-        <v>0</v>
+        <v>650.05</v>
       </c>
       <c r="E65" s="20" t="n">
-        <v>0</v>
+        <v>650.1</v>
       </c>
       <c r="F65" s="16" t="n">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>655.05</v>
+        <v>659.25</v>
       </c>
     </row>
     <row r="66">
@@ -2281,22 +2281,22 @@
         </is>
       </c>
       <c r="B66" s="8" t="n">
-        <v>231.5</v>
+        <v>245.65</v>
       </c>
       <c r="C66" s="10" t="n">
-        <v>225.93</v>
+        <v>240.25</v>
       </c>
       <c r="D66" s="13" t="n">
-        <v>0</v>
+        <v>237.5</v>
       </c>
       <c r="E66" s="20" t="n">
-        <v>0</v>
+        <v>238.13</v>
       </c>
       <c r="F66" s="16" t="n">
-        <v>56</v>
+        <v>113</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>229.39</v>
+        <v>242.68</v>
       </c>
     </row>
     <row r="67">
@@ -2306,22 +2306,22 @@
         </is>
       </c>
       <c r="B67" s="8" t="n">
-        <v>1901</v>
+        <v>1889.9</v>
       </c>
       <c r="C67" s="10" t="n">
-        <v>1844.4</v>
+        <v>1833</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>0</v>
+        <v>1892</v>
       </c>
       <c r="E67" s="20" t="n">
-        <v>0</v>
+        <v>1895.1</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>1854.3</v>
+        <v>1887.6</v>
       </c>
     </row>
     <row r="68">
@@ -2331,22 +2331,22 @@
         </is>
       </c>
       <c r="B68" s="8" t="n">
-        <v>627.85</v>
+        <v>655.65</v>
       </c>
       <c r="C68" s="10" t="n">
-        <v>613.2</v>
+        <v>643.15</v>
       </c>
       <c r="D68" s="13" t="n">
-        <v>0</v>
+        <v>643.5</v>
       </c>
       <c r="E68" s="20" t="n">
-        <v>0</v>
+        <v>642.2</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>616.2</v>
+        <v>650.3</v>
       </c>
     </row>
     <row r="69">
@@ -2356,22 +2356,22 @@
         </is>
       </c>
       <c r="B69" s="8" t="n">
-        <v>202.39</v>
+        <v>197.09</v>
       </c>
       <c r="C69" s="10" t="n">
+        <v>193.59</v>
+      </c>
+      <c r="D69" s="13" t="n">
+        <v>194.71</v>
+      </c>
+      <c r="E69" s="20" t="n">
+        <v>195.03</v>
+      </c>
+      <c r="F69" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="G69" s="4" t="n">
         <v>197</v>
-      </c>
-      <c r="D69" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="16" t="n">
-        <v>52</v>
-      </c>
-      <c r="G69" s="4" t="n">
-        <v>201.44</v>
       </c>
     </row>
     <row r="70">
@@ -2381,22 +2381,22 @@
         </is>
       </c>
       <c r="B70" s="8" t="n">
-        <v>214.18</v>
+        <v>207.49</v>
       </c>
       <c r="C70" s="10" t="n">
-        <v>208.35</v>
+        <v>205</v>
       </c>
       <c r="D70" s="13" t="n">
-        <v>0</v>
+        <v>206.09</v>
       </c>
       <c r="E70" s="20" t="n">
-        <v>0</v>
+        <v>205.83</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>208.75</v>
+        <v>207.32</v>
       </c>
     </row>
     <row r="71">
@@ -2406,22 +2406,22 @@
         </is>
       </c>
       <c r="B71" s="8" t="n">
-        <v>781.75</v>
+        <v>781.4</v>
       </c>
       <c r="C71" s="10" t="n">
-        <v>769.2</v>
+        <v>770.75</v>
       </c>
       <c r="D71" s="13" t="n">
-        <v>0</v>
+        <v>769.5</v>
       </c>
       <c r="E71" s="20" t="n">
-        <v>0</v>
+        <v>770.45</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>775.3</v>
+        <v>771.25</v>
       </c>
     </row>
     <row r="72">
@@ -2431,22 +2431,22 @@
         </is>
       </c>
       <c r="B72" s="8" t="n">
-        <v>323.8</v>
+        <v>333.2</v>
       </c>
       <c r="C72" s="10" t="n">
-        <v>315.05</v>
+        <v>324.7</v>
       </c>
       <c r="D72" s="13" t="n">
-        <v>0</v>
+        <v>332</v>
       </c>
       <c r="E72" s="20" t="n">
-        <v>0</v>
+        <v>332.55</v>
       </c>
       <c r="F72" s="16" t="n">
         <v>3</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>318</v>
+        <v>332.45</v>
       </c>
     </row>
     <row r="73">
@@ -2456,22 +2456,22 @@
         </is>
       </c>
       <c r="B73" s="8" t="n">
-        <v>2389.8</v>
+        <v>2351.6</v>
       </c>
       <c r="C73" s="10" t="n">
-        <v>2340</v>
+        <v>2323.1</v>
       </c>
       <c r="D73" s="13" t="n">
-        <v>0</v>
+        <v>2370</v>
       </c>
       <c r="E73" s="20" t="n">
-        <v>0</v>
+        <v>2368.1</v>
       </c>
       <c r="F73" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>2343</v>
+        <v>2348.1</v>
       </c>
     </row>
     <row r="74">
@@ -2481,22 +2481,22 @@
         </is>
       </c>
       <c r="B74" s="8" t="n">
-        <v>5665.5</v>
+        <v>5537</v>
       </c>
       <c r="C74" s="10" t="n">
-        <v>5557.5</v>
+        <v>5410.5</v>
       </c>
       <c r="D74" s="13" t="n">
-        <v>0</v>
+        <v>5510</v>
       </c>
       <c r="E74" s="20" t="n">
-        <v>0</v>
+        <v>5521</v>
       </c>
       <c r="F74" s="16" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>5619</v>
+        <v>5532</v>
       </c>
     </row>
     <row r="75">
@@ -2506,22 +2506,22 @@
         </is>
       </c>
       <c r="B75" s="8" t="n">
-        <v>791.95</v>
+        <v>802</v>
       </c>
       <c r="C75" s="10" t="n">
-        <v>771.45</v>
+        <v>790.75</v>
       </c>
       <c r="D75" s="13" t="n">
-        <v>0</v>
+        <v>792.6</v>
       </c>
       <c r="E75" s="20" t="n">
-        <v>0</v>
+        <v>793.4</v>
       </c>
       <c r="F75" s="16" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>776.5</v>
+        <v>797.75</v>
       </c>
     </row>
     <row r="76">
@@ -2531,22 +2531,22 @@
         </is>
       </c>
       <c r="B76" s="8" t="n">
-        <v>402.15</v>
+        <v>383.35</v>
       </c>
       <c r="C76" s="10" t="n">
-        <v>382</v>
+        <v>375.6</v>
       </c>
       <c r="D76" s="13" t="n">
-        <v>0</v>
+        <v>383</v>
       </c>
       <c r="E76" s="20" t="n">
-        <v>0</v>
+        <v>383.6</v>
       </c>
       <c r="F76" s="16" t="n">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>401.3</v>
+        <v>382.75</v>
       </c>
     </row>
     <row r="77">
@@ -2556,22 +2556,22 @@
         </is>
       </c>
       <c r="B77" s="8" t="n">
-        <v>1110</v>
+        <v>1100</v>
       </c>
       <c r="C77" s="10" t="n">
-        <v>1045.55</v>
+        <v>1080</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>0</v>
+        <v>1071.7</v>
       </c>
       <c r="E77" s="20" t="n">
-        <v>0</v>
+        <v>1082.1</v>
       </c>
       <c r="F77" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>1102</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="78">
@@ -2581,22 +2581,22 @@
         </is>
       </c>
       <c r="B78" s="8" t="n">
-        <v>1464.1</v>
+        <v>1483.7</v>
       </c>
       <c r="C78" s="10" t="n">
-        <v>1404.6</v>
+        <v>1443.1</v>
       </c>
       <c r="D78" s="13" t="n">
-        <v>0</v>
+        <v>1461.2</v>
       </c>
       <c r="E78" s="20" t="n">
-        <v>0</v>
+        <v>1460</v>
       </c>
       <c r="F78" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>1409.1</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="79">
@@ -2606,22 +2606,22 @@
         </is>
       </c>
       <c r="B79" s="8" t="n">
-        <v>979.65</v>
+        <v>969.8</v>
       </c>
       <c r="C79" s="10" t="n">
-        <v>955.25</v>
+        <v>953.15</v>
       </c>
       <c r="D79" s="13" t="n">
-        <v>0</v>
+        <v>954.8</v>
       </c>
       <c r="E79" s="20" t="n">
-        <v>0</v>
+        <v>953.4</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>972.2</v>
+        <v>962.3</v>
       </c>
     </row>
     <row r="80">
@@ -2631,22 +2631,22 @@
         </is>
       </c>
       <c r="B80" s="8" t="n">
-        <v>5287.5</v>
+        <v>5550</v>
       </c>
       <c r="C80" s="10" t="n">
-        <v>5207</v>
+        <v>5165</v>
       </c>
       <c r="D80" s="13" t="n">
-        <v>0</v>
+        <v>5107</v>
       </c>
       <c r="E80" s="20" t="n">
-        <v>0</v>
+        <v>5108.5</v>
       </c>
       <c r="F80" s="16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>5222.5</v>
+        <v>5382</v>
       </c>
     </row>
     <row r="81">
@@ -2656,22 +2656,22 @@
         </is>
       </c>
       <c r="B81" s="8" t="n">
-        <v>1030.8</v>
+        <v>1036</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>1016.7</v>
+        <v>979.5</v>
       </c>
       <c r="D81" s="13" t="n">
-        <v>0</v>
+        <v>1009.2</v>
       </c>
       <c r="E81" s="20" t="n">
-        <v>0</v>
+        <v>1008.5</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>1023.5</v>
+        <v>1014.6</v>
       </c>
     </row>
     <row r="82">
@@ -2681,22 +2681,22 @@
         </is>
       </c>
       <c r="B82" s="8" t="n">
-        <v>703</v>
+        <v>665.7</v>
       </c>
       <c r="C82" s="10" t="n">
-        <v>665.1</v>
+        <v>658.8</v>
       </c>
       <c r="D82" s="13" t="n">
-        <v>0</v>
+        <v>664</v>
       </c>
       <c r="E82" s="20" t="n">
-        <v>0</v>
+        <v>664.45</v>
       </c>
       <c r="F82" s="16" t="n">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>672.9</v>
+        <v>663.5</v>
       </c>
     </row>
     <row r="83">
@@ -2706,22 +2706,22 @@
         </is>
       </c>
       <c r="B83" s="8" t="n">
-        <v>2124</v>
+        <v>2112</v>
       </c>
       <c r="C83" s="10" t="n">
-        <v>2105.3</v>
+        <v>2085.1</v>
       </c>
       <c r="D83" s="13" t="n">
-        <v>0</v>
+        <v>2101</v>
       </c>
       <c r="E83" s="20" t="n">
-        <v>0</v>
+        <v>2100.8</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>2116.9</v>
+        <v>2107.8</v>
       </c>
     </row>
     <row r="84">
@@ -2731,22 +2731,22 @@
         </is>
       </c>
       <c r="B84" s="8" t="n">
-        <v>2809.4</v>
+        <v>2906.2</v>
       </c>
       <c r="C84" s="10" t="n">
-        <v>2773.2</v>
+        <v>2830</v>
       </c>
       <c r="D84" s="13" t="n">
+        <v>2838.6</v>
+      </c>
+      <c r="E84" s="20" t="n">
+        <v>2849.8</v>
+      </c>
+      <c r="F84" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E84" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F84" s="16" t="n">
-        <v>1</v>
-      </c>
       <c r="G84" s="4" t="n">
-        <v>2802</v>
+        <v>2878.7</v>
       </c>
     </row>
     <row r="85">
@@ -2756,22 +2756,22 @@
         </is>
       </c>
       <c r="B85" s="8" t="n">
-        <v>620.35</v>
+        <v>602.6</v>
       </c>
       <c r="C85" s="10" t="n">
-        <v>604</v>
+        <v>592.6</v>
       </c>
       <c r="D85" s="13" t="n">
-        <v>0</v>
+        <v>592</v>
       </c>
       <c r="E85" s="20" t="n">
-        <v>0</v>
+        <v>593.3</v>
       </c>
       <c r="F85" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="G85" s="4" t="n">
-        <v>607.45</v>
+        <v>595.25</v>
       </c>
     </row>
     <row r="86">
@@ -2781,22 +2781,22 @@
         </is>
       </c>
       <c r="B86" s="8" t="n">
-        <v>608.9</v>
+        <v>605.5</v>
       </c>
       <c r="C86" s="10" t="n">
-        <v>599</v>
+        <v>597.05</v>
       </c>
       <c r="D86" s="13" t="n">
-        <v>0</v>
+        <v>593.4</v>
       </c>
       <c r="E86" s="20" t="n">
-        <v>0</v>
+        <v>596.95</v>
       </c>
       <c r="F86" s="16" t="n">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>605.8</v>
+        <v>600.6</v>
       </c>
     </row>
     <row r="87">
@@ -2806,22 +2806,22 @@
         </is>
       </c>
       <c r="B87" s="8" t="n">
-        <v>5079.4</v>
+        <v>5135.9</v>
       </c>
       <c r="C87" s="10" t="n">
-        <v>4981.8</v>
+        <v>5054.8</v>
       </c>
       <c r="D87" s="13" t="n">
-        <v>0</v>
+        <v>5031.3</v>
       </c>
       <c r="E87" s="20" t="n">
-        <v>0</v>
+        <v>5045.8</v>
       </c>
       <c r="F87" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G87" s="4" t="n">
-        <v>5052.2</v>
+        <v>5068</v>
       </c>
     </row>
     <row r="88">
@@ -2831,22 +2831,22 @@
         </is>
       </c>
       <c r="B88" s="8" t="n">
-        <v>4555</v>
+        <v>4525</v>
       </c>
       <c r="C88" s="10" t="n">
-        <v>4475.1</v>
+        <v>4471.6</v>
       </c>
       <c r="D88" s="13" t="n">
-        <v>0</v>
+        <v>4466</v>
       </c>
       <c r="E88" s="20" t="n">
-        <v>0</v>
+        <v>4482.5</v>
       </c>
       <c r="F88" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>4512.6</v>
+        <v>4501</v>
       </c>
     </row>
     <row r="89">
@@ -2856,22 +2856,22 @@
         </is>
       </c>
       <c r="B89" s="8" t="n">
-        <v>2075.8</v>
+        <v>2004.9</v>
       </c>
       <c r="C89" s="10" t="n">
-        <v>2025.6</v>
+        <v>1971.5</v>
       </c>
       <c r="D89" s="13" t="n">
-        <v>0</v>
+        <v>1978.2</v>
       </c>
       <c r="E89" s="20" t="n">
-        <v>0</v>
+        <v>1978.9</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>2060.2</v>
+        <v>1994.4</v>
       </c>
     </row>
     <row r="90">
@@ -2881,22 +2881,22 @@
         </is>
       </c>
       <c r="B90" s="8" t="n">
-        <v>268.9</v>
+        <v>259.4</v>
       </c>
       <c r="C90" s="10" t="n">
-        <v>264.15</v>
+        <v>255.65</v>
       </c>
       <c r="D90" s="13" t="n">
-        <v>0</v>
+        <v>256.95</v>
       </c>
       <c r="E90" s="20" t="n">
-        <v>0</v>
+        <v>256.1</v>
       </c>
       <c r="F90" s="16" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>267.2</v>
+        <v>258.25</v>
       </c>
     </row>
     <row r="91">
@@ -2906,22 +2906,22 @@
         </is>
       </c>
       <c r="B91" s="8" t="n">
-        <v>229.8</v>
+        <v>231.48</v>
       </c>
       <c r="C91" s="10" t="n">
-        <v>228.33</v>
+        <v>230.06</v>
       </c>
       <c r="D91" s="13" t="n">
-        <v>0</v>
+        <v>230.3</v>
       </c>
       <c r="E91" s="20" t="n">
-        <v>0</v>
+        <v>230.73</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>229.5</v>
+        <v>231.2</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1" thickBot="1">
@@ -2931,22 +2931,22 @@
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>726.8</v>
+        <v>712.5</v>
       </c>
       <c r="C92" s="10" t="n">
-        <v>713.55</v>
+        <v>704.1</v>
       </c>
       <c r="D92" s="13" t="n">
-        <v>0</v>
+        <v>701.65</v>
       </c>
       <c r="E92" s="22" t="n">
-        <v>0</v>
+        <v>700.85</v>
       </c>
       <c r="F92" s="16" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G92" s="4" t="n">
-        <v>724.35</v>
+        <v>705</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1" thickBot="1">
@@ -2956,22 +2956,22 @@
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>1567.7</v>
+        <v>1582.7</v>
       </c>
       <c r="C93" s="10" t="n">
-        <v>1539</v>
+        <v>1553</v>
       </c>
       <c r="D93" s="13" t="n">
-        <v>0</v>
+        <v>1571.7</v>
       </c>
       <c r="E93" s="23" t="n">
-        <v>0</v>
+        <v>1578.9</v>
       </c>
       <c r="F93" s="16" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G93" s="4" t="n">
-        <v>1550.4</v>
+        <v>1574.5</v>
       </c>
     </row>
     <row r="94">
@@ -2981,22 +2981,22 @@
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>6558</v>
+        <v>6544</v>
       </c>
       <c r="C94" s="10" t="n">
-        <v>6345.5</v>
+        <v>6418.5</v>
       </c>
       <c r="D94" s="13" t="n">
-        <v>0</v>
+        <v>6480</v>
       </c>
       <c r="E94" s="19" t="n">
-        <v>0</v>
+        <v>6492.5</v>
       </c>
       <c r="F94" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G94" s="4" t="n">
-        <v>6490</v>
+        <v>6544</v>
       </c>
     </row>
     <row r="95">
@@ -3006,22 +3006,22 @@
         </is>
       </c>
       <c r="B95" s="8" t="n">
-        <v>1665</v>
+        <v>1670</v>
       </c>
       <c r="C95" s="10" t="n">
-        <v>1617</v>
+        <v>1640.7</v>
       </c>
       <c r="D95" s="13" t="n">
-        <v>0</v>
+        <v>1633</v>
       </c>
       <c r="E95" s="20" t="n">
-        <v>0</v>
+        <v>1626.3</v>
       </c>
       <c r="F95" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G95" s="4" t="n">
-        <v>1637.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -3031,22 +3031,22 @@
         </is>
       </c>
       <c r="B96" s="8" t="n">
-        <v>1398.5</v>
+        <v>1494.3</v>
       </c>
       <c r="C96" s="10" t="n">
-        <v>1357.8</v>
+        <v>1467.2</v>
       </c>
       <c r="D96" s="13" t="n">
-        <v>0</v>
+        <v>1473.7</v>
       </c>
       <c r="E96" s="20" t="n">
-        <v>0</v>
+        <v>1470</v>
       </c>
       <c r="F96" s="16" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>1360.1</v>
+        <v>1482.6</v>
       </c>
     </row>
     <row r="97">
@@ -3056,22 +3056,22 @@
         </is>
       </c>
       <c r="B97" s="8" t="n">
-        <v>1434.2</v>
+        <v>1361.8</v>
       </c>
       <c r="C97" s="10" t="n">
-        <v>1397.4</v>
+        <v>1336.4</v>
       </c>
       <c r="D97" s="13" t="n">
-        <v>0</v>
+        <v>1349.2</v>
       </c>
       <c r="E97" s="20" t="n">
-        <v>0</v>
+        <v>1348.8</v>
       </c>
       <c r="F97" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G97" s="4" t="n">
-        <v>1425</v>
+        <v>1361.4</v>
       </c>
     </row>
     <row r="98">
@@ -3081,22 +3081,22 @@
         </is>
       </c>
       <c r="B98" s="8" t="n">
-        <v>2594.3</v>
+        <v>2556.2</v>
       </c>
       <c r="C98" s="10" t="n">
-        <v>2531</v>
+        <v>2524.8</v>
       </c>
       <c r="D98" s="13" t="n">
-        <v>0</v>
+        <v>2538</v>
       </c>
       <c r="E98" s="20" t="n">
-        <v>0</v>
+        <v>2541.4</v>
       </c>
       <c r="F98" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G98" s="4" t="n">
-        <v>2581.3</v>
+        <v>2553.1</v>
       </c>
     </row>
     <row r="99">
@@ -3106,22 +3106,22 @@
         </is>
       </c>
       <c r="B99" s="8" t="n">
-        <v>2103</v>
+        <v>2114</v>
       </c>
       <c r="C99" s="10" t="n">
-        <v>2083.5</v>
+        <v>2092.1</v>
       </c>
       <c r="D99" s="13" t="n">
-        <v>0</v>
+        <v>2088.9</v>
       </c>
       <c r="E99" s="20" t="n">
-        <v>0</v>
+        <v>2090</v>
       </c>
       <c r="F99" s="16" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>2096</v>
+        <v>2109.1</v>
       </c>
     </row>
     <row r="100">
@@ -3131,22 +3131,22 @@
         </is>
       </c>
       <c r="B100" s="8" t="n">
-        <v>749.8</v>
+        <v>737</v>
       </c>
       <c r="C100" s="10" t="n">
-        <v>723.95</v>
+        <v>722.1</v>
       </c>
       <c r="D100" s="13" t="n">
-        <v>0</v>
+        <v>724</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>0</v>
+        <v>725.25</v>
       </c>
       <c r="F100" s="16" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>730</v>
+        <v>734.95</v>
       </c>
     </row>
     <row r="101">
@@ -3156,22 +3156,22 @@
         </is>
       </c>
       <c r="B101" s="8" t="n">
-        <v>1487</v>
+        <v>1494.5</v>
       </c>
       <c r="C101" s="10" t="n">
-        <v>1453</v>
+        <v>1468</v>
       </c>
       <c r="D101" s="13" t="n">
-        <v>0</v>
+        <v>1482.5</v>
       </c>
       <c r="E101" s="20" t="n">
-        <v>0</v>
+        <v>1489</v>
       </c>
       <c r="F101" s="16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>1479.5</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="102">
@@ -3181,22 +3181,22 @@
         </is>
       </c>
       <c r="B102" s="8" t="n">
-        <v>4323.4</v>
+        <v>4290</v>
       </c>
       <c r="C102" s="10" t="n">
-        <v>4189.4</v>
+        <v>4245</v>
       </c>
       <c r="D102" s="13" t="n">
+        <v>4269</v>
+      </c>
+      <c r="E102" s="20" t="n">
+        <v>4287.7</v>
+      </c>
+      <c r="F102" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E102" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F102" s="16" t="n">
-        <v>1</v>
-      </c>
       <c r="G102" s="4" t="n">
-        <v>4216.1</v>
+        <v>4278</v>
       </c>
     </row>
     <row r="103">
@@ -3206,22 +3206,22 @@
         </is>
       </c>
       <c r="B103" s="8" t="n">
-        <v>71.31999999999999</v>
+        <v>73.53</v>
       </c>
       <c r="C103" s="10" t="n">
-        <v>69.55</v>
+        <v>72.70999999999999</v>
       </c>
       <c r="D103" s="13" t="n">
-        <v>0</v>
+        <v>72.47</v>
       </c>
       <c r="E103" s="20" t="n">
-        <v>0</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="F103" s="16" t="n">
-        <v>193</v>
+        <v>161</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>70.34999999999999</v>
+        <v>72.97</v>
       </c>
     </row>
     <row r="104">
@@ -3231,22 +3231,22 @@
         </is>
       </c>
       <c r="B104" s="8" t="n">
-        <v>347.7</v>
+        <v>349.2</v>
       </c>
       <c r="C104" s="10" t="n">
-        <v>344</v>
+        <v>342.55</v>
       </c>
       <c r="D104" s="13" t="n">
-        <v>0</v>
+        <v>344.6</v>
       </c>
       <c r="E104" s="20" t="n">
-        <v>0</v>
+        <v>344.6</v>
       </c>
       <c r="F104" s="16" t="n">
-        <v>62</v>
+        <v>166</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>346.55</v>
+        <v>348.9</v>
       </c>
     </row>
     <row r="105">
@@ -3256,22 +3256,22 @@
         </is>
       </c>
       <c r="B105" s="8" t="n">
-        <v>1746</v>
+        <v>1760.3</v>
       </c>
       <c r="C105" s="10" t="n">
-        <v>1678.4</v>
+        <v>1733.4</v>
       </c>
       <c r="D105" s="13" t="n">
-        <v>0</v>
+        <v>1739</v>
       </c>
       <c r="E105" s="20" t="n">
-        <v>0</v>
+        <v>1738.3</v>
       </c>
       <c r="F105" s="16" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>1687.5</v>
+        <v>1741.3</v>
       </c>
     </row>
     <row r="106">
@@ -3281,22 +3281,22 @@
         </is>
       </c>
       <c r="B106" s="8" t="n">
-        <v>249.34</v>
+        <v>247.13</v>
       </c>
       <c r="C106" s="10" t="n">
-        <v>244.91</v>
+        <v>244.81</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>0</v>
+        <v>244.22</v>
       </c>
       <c r="E106" s="20" t="n">
-        <v>0</v>
+        <v>244.24</v>
       </c>
       <c r="F106" s="16" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>249.17</v>
+        <v>246.26</v>
       </c>
     </row>
     <row r="107">
@@ -3306,22 +3306,22 @@
         </is>
       </c>
       <c r="B107" s="8" t="n">
-        <v>1146.2</v>
+        <v>1105.6</v>
       </c>
       <c r="C107" s="10" t="n">
-        <v>1106.1</v>
+        <v>1079.65</v>
       </c>
       <c r="D107" s="13" t="n">
-        <v>0</v>
+        <v>1100.2</v>
       </c>
       <c r="E107" s="20" t="n">
-        <v>0</v>
+        <v>1100.75</v>
       </c>
       <c r="F107" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>1114.7</v>
+        <v>1101.95</v>
       </c>
     </row>
     <row r="108">
@@ -3331,22 +3331,22 @@
         </is>
       </c>
       <c r="B108" s="8" t="n">
-        <v>5732</v>
+        <v>5701</v>
       </c>
       <c r="C108" s="10" t="n">
-        <v>5626</v>
+        <v>5632.5</v>
       </c>
       <c r="D108" s="13" t="n">
-        <v>0</v>
+        <v>5668</v>
       </c>
       <c r="E108" s="20" t="n">
-        <v>0</v>
+        <v>5662</v>
       </c>
       <c r="F108" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>5667</v>
+        <v>5672.5</v>
       </c>
     </row>
     <row r="109">
@@ -3356,22 +3356,22 @@
         </is>
       </c>
       <c r="B109" s="8" t="n">
-        <v>324.1</v>
+        <v>325</v>
       </c>
       <c r="C109" s="10" t="n">
-        <v>319</v>
+        <v>317.8</v>
       </c>
       <c r="D109" s="13" t="n">
-        <v>0</v>
+        <v>319.5</v>
       </c>
       <c r="E109" s="20" t="n">
-        <v>0</v>
+        <v>319.9</v>
       </c>
       <c r="F109" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G109" s="4" t="n">
-        <v>322.65</v>
+        <v>322.15</v>
       </c>
     </row>
     <row r="110">
@@ -3381,22 +3381,22 @@
         </is>
       </c>
       <c r="B110" s="8" t="n">
-        <v>3105</v>
+        <v>3070.9</v>
       </c>
       <c r="C110" s="10" t="n">
-        <v>3062</v>
+        <v>3033.7</v>
       </c>
       <c r="D110" s="13" t="n">
-        <v>0</v>
+        <v>3038.5</v>
       </c>
       <c r="E110" s="20" t="n">
-        <v>0</v>
+        <v>3031.7</v>
       </c>
       <c r="F110" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>3104.3</v>
+        <v>3058</v>
       </c>
     </row>
     <row r="111">
@@ -3406,22 +3406,22 @@
         </is>
       </c>
       <c r="B111" s="8" t="n">
-        <v>6167</v>
+        <v>5968</v>
       </c>
       <c r="C111" s="10" t="n">
-        <v>6061.5</v>
+        <v>5908.5</v>
       </c>
       <c r="D111" s="13" t="n">
-        <v>0</v>
+        <v>5885</v>
       </c>
       <c r="E111" s="20" t="n">
-        <v>0</v>
+        <v>5883.5</v>
       </c>
       <c r="F111" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>6093.5</v>
+        <v>5955</v>
       </c>
     </row>
     <row r="112">
@@ -3431,22 +3431,22 @@
         </is>
       </c>
       <c r="B112" s="8" t="n">
-        <v>304.5</v>
+        <v>302.95</v>
       </c>
       <c r="C112" s="10" t="n">
-        <v>300.8</v>
+        <v>295.75</v>
       </c>
       <c r="D112" s="13" t="n">
-        <v>0</v>
+        <v>298.05</v>
       </c>
       <c r="E112" s="20" t="n">
-        <v>0</v>
+        <v>298.1</v>
       </c>
       <c r="F112" s="16" t="n">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>301.4</v>
+        <v>301.55</v>
       </c>
     </row>
     <row r="113">
@@ -3456,22 +3456,22 @@
         </is>
       </c>
       <c r="B113" s="8" t="n">
-        <v>152.43</v>
+        <v>146</v>
       </c>
       <c r="C113" s="10" t="n">
-        <v>148.88</v>
+        <v>144</v>
       </c>
       <c r="D113" s="13" t="n">
-        <v>0</v>
+        <v>144.86</v>
       </c>
       <c r="E113" s="20" t="n">
-        <v>0</v>
+        <v>144.99</v>
       </c>
       <c r="F113" s="16" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G113" s="4" t="n">
-        <v>149.47</v>
+        <v>145.9</v>
       </c>
     </row>
     <row r="114">
@@ -3481,22 +3481,22 @@
         </is>
       </c>
       <c r="B114" s="8" t="n">
-        <v>1011.75</v>
+        <v>998.55</v>
       </c>
       <c r="C114" s="10" t="n">
-        <v>997.15</v>
+        <v>978.85</v>
       </c>
       <c r="D114" s="13" t="n">
-        <v>0</v>
+        <v>1002.65</v>
       </c>
       <c r="E114" s="20" t="n">
-        <v>0</v>
+        <v>1006.1</v>
       </c>
       <c r="F114" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G114" s="4" t="n">
-        <v>1004.6</v>
+        <v>997.55</v>
       </c>
     </row>
     <row r="115">
@@ -3506,22 +3506,22 @@
         </is>
       </c>
       <c r="B115" s="8" t="n">
-        <v>216.46</v>
+        <v>211.25</v>
       </c>
       <c r="C115" s="10" t="n">
-        <v>211.25</v>
+        <v>203.9</v>
       </c>
       <c r="D115" s="13" t="n">
-        <v>0</v>
+        <v>208.97</v>
       </c>
       <c r="E115" s="20" t="n">
-        <v>0</v>
+        <v>209.95</v>
       </c>
       <c r="F115" s="16" t="n">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="G115" s="4" t="n">
-        <v>213.83</v>
+        <v>210.84</v>
       </c>
     </row>
     <row r="116">
@@ -3531,22 +3531,22 @@
         </is>
       </c>
       <c r="B116" s="8" t="n">
-        <v>411.8</v>
+        <v>408.75</v>
       </c>
       <c r="C116" s="10" t="n">
-        <v>405.2</v>
+        <v>405.65</v>
       </c>
       <c r="D116" s="13" t="n">
-        <v>0</v>
+        <v>403</v>
       </c>
       <c r="E116" s="20" t="n">
-        <v>0</v>
+        <v>402.5</v>
       </c>
       <c r="F116" s="16" t="n">
-        <v>115</v>
+        <v>51</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>411</v>
+        <v>406.15</v>
       </c>
     </row>
     <row r="117">
@@ -3556,22 +3556,22 @@
         </is>
       </c>
       <c r="B117" s="8" t="n">
-        <v>917.7</v>
+        <v>914.8</v>
       </c>
       <c r="C117" s="10" t="n">
-        <v>906.2</v>
+        <v>902.05</v>
       </c>
       <c r="D117" s="13" t="n">
-        <v>0</v>
+        <v>896</v>
       </c>
       <c r="E117" s="20" t="n">
-        <v>0</v>
+        <v>897.7</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>912.35</v>
+        <v>902.95</v>
       </c>
     </row>
     <row r="118">
@@ -3581,22 +3581,22 @@
         </is>
       </c>
       <c r="B118" s="8" t="n">
-        <v>1779.5</v>
+        <v>1808.4</v>
       </c>
       <c r="C118" s="10" t="n">
-        <v>1764.4</v>
+        <v>1790.1</v>
       </c>
       <c r="D118" s="13" t="n">
-        <v>0</v>
+        <v>1796.9</v>
       </c>
       <c r="E118" s="20" t="n">
-        <v>0</v>
+        <v>1798.7</v>
       </c>
       <c r="F118" s="16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>1779.5</v>
+        <v>1803.5</v>
       </c>
     </row>
     <row r="119">
@@ -3606,22 +3606,22 @@
         </is>
       </c>
       <c r="B119" s="8" t="n">
-        <v>3150.8</v>
+        <v>3308.9</v>
       </c>
       <c r="C119" s="10" t="n">
-        <v>3025.8</v>
+        <v>3240</v>
       </c>
       <c r="D119" s="13" t="n">
-        <v>0</v>
+        <v>3269.3</v>
       </c>
       <c r="E119" s="20" t="n">
-        <v>0</v>
+        <v>3277.3</v>
       </c>
       <c r="F119" s="16" t="n">
         <v>5</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>3061.1</v>
+        <v>3284.8</v>
       </c>
     </row>
     <row r="120">
@@ -3631,22 +3631,22 @@
         </is>
       </c>
       <c r="B120" s="8" t="n">
-        <v>3032</v>
+        <v>2923.9</v>
       </c>
       <c r="C120" s="10" t="n">
-        <v>2948.6</v>
+        <v>2880</v>
       </c>
       <c r="D120" s="13" t="n">
-        <v>0</v>
+        <v>2898</v>
       </c>
       <c r="E120" s="20" t="n">
-        <v>0</v>
+        <v>2900.2</v>
       </c>
       <c r="F120" s="16" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>2953.2</v>
+        <v>2919.7</v>
       </c>
     </row>
     <row r="121">
@@ -3656,22 +3656,22 @@
         </is>
       </c>
       <c r="B121" s="8" t="n">
-        <v>228.8</v>
+        <v>223.65</v>
       </c>
       <c r="C121" s="10" t="n">
-        <v>223.22</v>
+        <v>219.46</v>
       </c>
       <c r="D121" s="13" t="n">
-        <v>0</v>
+        <v>730.05</v>
       </c>
       <c r="E121" s="20" t="n">
-        <v>0</v>
+        <v>731.65</v>
       </c>
       <c r="F121" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G121" s="4" t="n">
-        <v>223.7</v>
+        <v>221.8</v>
       </c>
     </row>
     <row r="122">
@@ -3681,22 +3681,22 @@
         </is>
       </c>
       <c r="B122" s="8" t="n">
-        <v>1765</v>
+        <v>1692.9</v>
       </c>
       <c r="C122" s="10" t="n">
-        <v>1726.6</v>
+        <v>1667</v>
       </c>
       <c r="D122" s="13" t="n">
-        <v>0</v>
+        <v>1689.1</v>
       </c>
       <c r="E122" s="20" t="n">
-        <v>0</v>
+        <v>1683.6</v>
       </c>
       <c r="F122" s="16" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G122" s="4" t="n">
-        <v>1740.1</v>
+        <v>1688.5</v>
       </c>
     </row>
     <row r="123">
@@ -3706,22 +3706,22 @@
         </is>
       </c>
       <c r="B123" s="8" t="n">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="C123" s="10" t="n">
-        <v>641</v>
+        <v>638.5</v>
       </c>
       <c r="D123" s="13" t="n">
-        <v>0</v>
+        <v>635</v>
       </c>
       <c r="E123" s="20" t="n">
-        <v>0</v>
+        <v>637.25</v>
       </c>
       <c r="F123" s="16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G123" s="4" t="n">
-        <v>648</v>
+        <v>640.45</v>
       </c>
     </row>
     <row r="124">
@@ -3731,22 +3731,22 @@
         </is>
       </c>
       <c r="B124" s="8" t="n">
-        <v>1662</v>
+        <v>1693.6</v>
       </c>
       <c r="C124" s="10" t="n">
-        <v>1614.2</v>
+        <v>1661.8</v>
       </c>
       <c r="D124" s="13" t="n">
-        <v>0</v>
+        <v>1668.7</v>
       </c>
       <c r="E124" s="20" t="n">
-        <v>0</v>
+        <v>1674.6</v>
       </c>
       <c r="F124" s="16" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G124" s="4" t="n">
-        <v>1626.4</v>
+        <v>1683.6</v>
       </c>
     </row>
     <row r="125">
@@ -3759,19 +3759,19 @@
         <v>738</v>
       </c>
       <c r="C125" s="10" t="n">
-        <v>728</v>
+        <v>726.5</v>
       </c>
       <c r="D125" s="13" t="n">
-        <v>0</v>
+        <v>718</v>
       </c>
       <c r="E125" s="20" t="n">
-        <v>0</v>
+        <v>718.25</v>
       </c>
       <c r="F125" s="16" t="n">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="G125" s="4" t="n">
-        <v>734.95</v>
+        <v>727.95</v>
       </c>
     </row>
     <row r="126">
@@ -3781,22 +3781,22 @@
         </is>
       </c>
       <c r="B126" s="8" t="n">
-        <v>3543</v>
+        <v>3545</v>
       </c>
       <c r="C126" s="10" t="n">
-        <v>3512.8</v>
+        <v>3524.6</v>
       </c>
       <c r="D126" s="13" t="n">
-        <v>0</v>
+        <v>3508</v>
       </c>
       <c r="E126" s="20" t="n">
-        <v>0</v>
+        <v>3514.6</v>
       </c>
       <c r="F126" s="16" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="G126" s="4" t="n">
-        <v>3533.2</v>
+        <v>3533.4</v>
       </c>
     </row>
     <row r="127">
@@ -3806,22 +3806,22 @@
         </is>
       </c>
       <c r="B127" s="8" t="n">
-        <v>1613.2</v>
+        <v>1604.4</v>
       </c>
       <c r="C127" s="10" t="n">
-        <v>1593.1</v>
+        <v>1587.9</v>
       </c>
       <c r="D127" s="13" t="n">
-        <v>0</v>
+        <v>1581.2</v>
       </c>
       <c r="E127" s="20" t="n">
-        <v>0</v>
+        <v>1580.3</v>
       </c>
       <c r="F127" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G127" s="4" t="n">
-        <v>1611</v>
+        <v>1603.5</v>
       </c>
     </row>
     <row r="128">
@@ -3831,22 +3831,22 @@
         </is>
       </c>
       <c r="B128" s="8" t="n">
-        <v>3649.5</v>
+        <v>3640</v>
       </c>
       <c r="C128" s="10" t="n">
-        <v>3611.4</v>
+        <v>3582.5</v>
       </c>
       <c r="D128" s="13" t="n">
-        <v>0</v>
+        <v>3579</v>
       </c>
       <c r="E128" s="20" t="n">
-        <v>0</v>
+        <v>3579.7</v>
       </c>
       <c r="F128" s="16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G128" s="4" t="n">
-        <v>3641.3</v>
+        <v>3629.9</v>
       </c>
     </row>
     <row r="129">
@@ -3856,22 +3856,22 @@
         </is>
       </c>
       <c r="B129" s="8" t="n">
-        <v>3314</v>
+        <v>3192.6</v>
       </c>
       <c r="C129" s="10" t="n">
-        <v>3265.7</v>
+        <v>3142.8</v>
       </c>
       <c r="D129" s="13" t="n">
-        <v>0</v>
+        <v>3170</v>
       </c>
       <c r="E129" s="20" t="n">
-        <v>0</v>
+        <v>3174.7</v>
       </c>
       <c r="F129" s="16" t="n">
         <v>2</v>
       </c>
       <c r="G129" s="4" t="n">
-        <v>3277.3</v>
+        <v>3182.4</v>
       </c>
     </row>
     <row r="130">
@@ -3881,22 +3881,22 @@
         </is>
       </c>
       <c r="B130" s="8" t="n">
-        <v>1469.8</v>
+        <v>1439</v>
       </c>
       <c r="C130" s="10" t="n">
-        <v>1421.3</v>
+        <v>1412.1</v>
       </c>
       <c r="D130" s="13" t="n">
-        <v>0</v>
+        <v>1414.9</v>
       </c>
       <c r="E130" s="20" t="n">
-        <v>0</v>
+        <v>1401.9</v>
       </c>
       <c r="F130" s="16" t="n">
         <v>5</v>
       </c>
       <c r="G130" s="4" t="n">
-        <v>1457.3</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="131">
@@ -3906,22 +3906,22 @@
         </is>
       </c>
       <c r="B131" s="8" t="n">
-        <v>5628</v>
+        <v>5536.5</v>
       </c>
       <c r="C131" s="10" t="n">
-        <v>5530</v>
+        <v>5416.5</v>
       </c>
       <c r="D131" s="13" t="n">
-        <v>0</v>
+        <v>5428</v>
       </c>
       <c r="E131" s="20" t="n">
-        <v>0</v>
+        <v>5435.5</v>
       </c>
       <c r="F131" s="16" t="n">
         <v>6</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>5610.5</v>
+        <v>5454</v>
       </c>
     </row>
     <row r="132">
@@ -3931,22 +3931,22 @@
         </is>
       </c>
       <c r="B132" s="8" t="n">
-        <v>2878.9</v>
+        <v>2815</v>
       </c>
       <c r="C132" s="10" t="n">
-        <v>2815.2</v>
+        <v>2769.7</v>
       </c>
       <c r="D132" s="13" t="n">
-        <v>0</v>
+        <v>2778</v>
       </c>
       <c r="E132" s="20" t="n">
-        <v>0</v>
+        <v>2780.6</v>
       </c>
       <c r="F132" s="16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>2870</v>
+        <v>2804.9</v>
       </c>
     </row>
     <row r="133">
@@ -3956,22 +3956,22 @@
         </is>
       </c>
       <c r="B133" s="8" t="n">
-        <v>2090</v>
+        <v>2069.2</v>
       </c>
       <c r="C133" s="10" t="n">
+        <v>2018.1</v>
+      </c>
+      <c r="D133" s="13" t="n">
+        <v>2018.1</v>
+      </c>
+      <c r="E133" s="20" t="n">
+        <v>2024.6</v>
+      </c>
+      <c r="F133" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" s="4" t="n">
         <v>2029</v>
-      </c>
-      <c r="D133" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E133" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F133" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G133" s="4" t="n">
-        <v>2052</v>
       </c>
     </row>
     <row r="134">
@@ -3981,22 +3981,22 @@
         </is>
       </c>
       <c r="B134" s="8" t="n">
-        <v>11991</v>
+        <v>11812</v>
       </c>
       <c r="C134" s="10" t="n">
-        <v>11898</v>
+        <v>11645</v>
       </c>
       <c r="D134" s="13" t="n">
-        <v>0</v>
+        <v>11738</v>
       </c>
       <c r="E134" s="20" t="n">
-        <v>0</v>
+        <v>11746</v>
       </c>
       <c r="F134" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G134" s="4" t="n">
-        <v>11926</v>
+        <v>11805</v>
       </c>
     </row>
     <row r="135">
@@ -4006,22 +4006,22 @@
         </is>
       </c>
       <c r="B135" s="8" t="n">
-        <v>654.8</v>
+        <v>634.65</v>
       </c>
       <c r="C135" s="10" t="n">
-        <v>644.45</v>
+        <v>629.9</v>
       </c>
       <c r="D135" s="13" t="n">
-        <v>0</v>
+        <v>630.9</v>
       </c>
       <c r="E135" s="20" t="n">
-        <v>0</v>
+        <v>630.5</v>
       </c>
       <c r="F135" s="16" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="G135" s="4" t="n">
-        <v>647.65</v>
+        <v>632.4</v>
       </c>
     </row>
     <row r="136">
@@ -4031,22 +4031,22 @@
         </is>
       </c>
       <c r="B136" s="8" t="n">
-        <v>446.9</v>
+        <v>447.4</v>
       </c>
       <c r="C136" s="10" t="n">
-        <v>440.65</v>
+        <v>442.6</v>
       </c>
       <c r="D136" s="13" t="n">
-        <v>0</v>
+        <v>439.5</v>
       </c>
       <c r="E136" s="20" t="n">
-        <v>0</v>
+        <v>440.05</v>
       </c>
       <c r="F136" s="16" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>443.5</v>
+        <v>443.75</v>
       </c>
     </row>
     <row r="137">
@@ -4056,22 +4056,22 @@
         </is>
       </c>
       <c r="B137" s="8" t="n">
-        <v>1281.9</v>
+        <v>1264</v>
       </c>
       <c r="C137" s="10" t="n">
-        <v>1261</v>
+        <v>1248.4</v>
       </c>
       <c r="D137" s="13" t="n">
-        <v>0</v>
+        <v>1262</v>
       </c>
       <c r="E137" s="20" t="n">
-        <v>0</v>
+        <v>1260.3</v>
       </c>
       <c r="F137" s="16" t="n">
         <v>11</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>1269</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="138">
@@ -4081,22 +4081,22 @@
         </is>
       </c>
       <c r="B138" s="8" t="n">
-        <v>130.43</v>
+        <v>128.69</v>
       </c>
       <c r="C138" s="10" t="n">
+        <v>126.42</v>
+      </c>
+      <c r="D138" s="13" t="n">
         <v>127.21</v>
       </c>
-      <c r="D138" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="E138" s="20" t="n">
-        <v>0</v>
+        <v>128.1</v>
       </c>
       <c r="F138" s="16" t="n">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>130.25</v>
+        <v>127.7</v>
       </c>
     </row>
     <row r="139" ht="15.75" customHeight="1" thickBot="1">
@@ -4106,22 +4106,22 @@
         </is>
       </c>
       <c r="B139" s="18" t="n">
-        <v>919.8</v>
+        <v>921</v>
       </c>
       <c r="C139" s="11" t="n">
-        <v>902.65</v>
+        <v>908.1</v>
       </c>
       <c r="D139" s="14" t="n">
-        <v>0</v>
+        <v>907</v>
       </c>
       <c r="E139" s="21" t="n">
-        <v>0</v>
+        <v>908.6</v>
       </c>
       <c r="F139" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>910</v>
+        <v>913.15</v>
       </c>
     </row>
   </sheetData>
@@ -4137,7 +4137,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G139"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" bestFit="1" customWidth="1" min="1" max="1"/>
   </cols>

</xml_diff>